<commit_message>
feat: enrich TechXXL component library
</commit_message>
<xml_diff>
--- a/config/product-master-data.xlsx
+++ b/config/product-master-data.xlsx
@@ -2,23 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start &amp; beheer" sheetId="1" r:id="Rdf6432cf3c17481d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataclassificatie" sheetId="2" r:id="R5ead287792bc4ecb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Productcategorieen" sheetId="3" r:id="Reaf3251f259647f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Producten" sheetId="4" r:id="Rd068d4601d744b75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materialen" sheetId="5" r:id="Rf852cb5a928a4dd0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Componenten" sheetId="6" r:id="R38053d9f4d6e4fe9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verbindingsrecepten" sheetId="7" r:id="Rd3e453a482c0404d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categorie-regels" sheetId="8" r:id="R042108ade96f4832"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product-regels" sheetId="9" r:id="R7478a7195eb44bcf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controles" sheetId="10" r:id="R0412999478904e5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open punten" sheetId="11" r:id="R58119502ed9c414e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wijzigingslog" sheetId="12" r:id="R54a4a3c1c43b4b85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keuzelijsten" sheetId="13" r:id="Rf401395462564ffa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prijs &amp; inkoop" sheetId="14" r:id="R10409fdf9877495f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gereedschappen" sheetId="15" r:id="R71be81314f6249d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAM-parameters" sheetId="16" r:id="Rc72e11f70e3a4b0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leveranciers" sheetId="17" r:id="Ra69044b1b29648bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start &amp; beheer" sheetId="1" r:id="R3f53383f595a426a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataclassificatie" sheetId="2" r:id="Re03c085da6194f1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Productcategorieen" sheetId="3" r:id="R2965705b732e4089"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Producten" sheetId="4" r:id="Rf5aff206fbea478f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materialen" sheetId="5" r:id="R845fa8cbc85643eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Componenten" sheetId="6" r:id="R5cbea1c42bb747d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verbindingsrecepten" sheetId="7" r:id="R2af48bb399bb4a82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categorie-regels" sheetId="8" r:id="R86b6f6fd41624efd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product-regels" sheetId="9" r:id="R42945ec559364a55"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controles" sheetId="10" r:id="R2fe50815c88e40a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open punten" sheetId="11" r:id="Rcf6b4eacf7ec4e92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wijzigingslog" sheetId="12" r:id="R8ea7756d35cd42e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keuzelijsten" sheetId="13" r:id="R3a325089842843a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prijs &amp; inkoop" sheetId="14" r:id="Ra8e4ece3299a4210"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gereedschappen" sheetId="15" r:id="Rfa17131f1182421c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAM-parameters" sheetId="16" r:id="R086c9134db654e1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leveranciers" sheetId="17" r:id="R296b4c2b7c6c4ef8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2001,7 +2001,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R30144ec48a8c4a6e"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R65a1fa61195043b0"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2028,7 +2028,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R18a4cb8686194e7e"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R7985e69eeff74958"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2055,7 +2055,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R9437b7d5bd154eef"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R42eceb6f22b446cc"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2082,7 +2082,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc1a5c020b5634297"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R47f46ea2e8cc4add"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2109,7 +2109,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rce3699baaeed454b"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rf8e873c465e24683"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2136,7 +2136,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R4f344d7fcf564549"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R670c914049c14b3e"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2163,7 +2163,169 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R3570955caa46441e"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R25385919b43241e5"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1066800" cy="742950"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="/xl/media/image8.jpg"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rade81ebaf7854c02"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1066800" cy="742950"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="/xl/media/image9.jpg"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re414e36ddf8c4bcd"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1066800" cy="742950"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="/xl/media/image10.jpg"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra08bf67c7dba45f5"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1066800" cy="742950"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="/xl/media/image11.jpg"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R6347a02472424af3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1066800" cy="742950"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="12" name="/xl/media/image12.jpg"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R919ae79b4c544b1b"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1066800" cy="742950"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13" name="/xl/media/image13.jpg"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R80ec3857901c4714"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2797,7 +2959,7 @@
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="19" t="str">
-        <x:v>Productregels, materialen, gereedschappen, prijzen en verbindingen — beheerfundering v1.8</x:v>
+        <x:v>Productregels, materialen, gereedschappen, prijzen en verbindingen — beheerfundering v1.9</x:v>
       </x:c>
       <x:c r="B1" s="19"/>
       <x:c r="C1" s="19"/>
@@ -2896,8 +3058,7 @@
         <x:v>Componenten</x:v>
       </x:c>
       <x:c r="B10" s="30" t="n">
-        <x:f>COUNTA('Componenten'!A6:A500)</x:f>
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="D10" s="28" t="str">
         <x:v>Productreferentiefouten</x:v>
@@ -2961,8 +3122,7 @@
         <x:v>Prijs- en inkoopregels</x:v>
       </x:c>
       <x:c r="B14" s="63" t="n">
-        <x:f>COUNTA('Prijs &amp; inkoop'!A6:A500)</x:f>
-        <x:v>29</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="D14" s="38" t="str">
         <x:v>2</x:v>
@@ -3176,7 +3336,7 @@
       </x:c>
       <x:c r="B32" s="6" t="n">
         <x:f>COUNTIF('Prijs &amp; inkoop'!U6:U500,"&lt;&gt;")</x:f>
-        <x:v>7</x:v>
+        <x:v>13</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3637,7 +3797,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6bc7f3aca924cd7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffbd8e77ad4d41cb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4139,7 +4299,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd45edb5032e9483b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R714f0f34affe47a4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4704,9 +4864,9 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" t="str">
-        <x:v>CHG-0019</x:v>
-      </x:c>
-      <x:c r="B25" t="n">
+        <x:v>CHG-0020</x:v>
+      </x:c>
+      <x:c r="B25" s="64" t="n">
         <x:v>46256</x:v>
       </x:c>
       <x:c r="C25" t="str">
@@ -4726,6 +4886,32 @@
       </x:c>
       <x:c r="H25" t="str">
         <x:v>App-reader migreert gelijktijdig naar Leverancier-ID, subcategorie en productscope; machinebasis toegevoegd als geldig basisproduct.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="64.5" customHeight="1">
+      <x:c r="A26" t="str">
+        <x:v>CHG-0021</x:v>
+      </x:c>
+      <x:c r="B26" s="64" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="C26" t="str">
+        <x:v>Dylan / Codex</x:v>
+      </x:c>
+      <x:c r="D26" t="str">
+        <x:v>1.9</x:v>
+      </x:c>
+      <x:c r="E26" s="6" t="str">
+        <x:v>TechXXL-bibliotheek verrijkt met geverifieerde artikelen en previews</x:v>
+      </x:c>
+      <x:c r="F26" s="6" t="str">
+        <x:v>Generieke 30x30-, 40x40- en 45x45-profielaanbiedingen vervangen door actuele TechXXL-artikelen; groef-8 eindkappen 80x80 en 80x40 vrijgegeven als leveranciersdata; losse T-moer 8 M8 toegevoegd; zes bronafbeeldingen extern geregistreerd en als Excel-preview ingebed.</x:v>
+      </x:c>
+      <x:c r="G26" s="6" t="str">
+        <x:v>alu_profile_30x30;alu_profile_40x40;alu_profile_45x45;end_cap_8_80x80_black_candidate;end_cap_8_80x40_black_candidate;techxxl_t_nut_8_m8;image-catalog.json</x:v>
+      </x:c>
+      <x:c r="H26" s="6" t="str">
+        <x:v>De bestaande kandidaat-ID's van de eindkappen blijven stabiel. De complete M8x22 + Nut 8-set blijft apart te controleren; de gevonden T-moer is bewust niet als complete set aangemerkt.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4735,7 +4921,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac4c802922b8491b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf99656508a0495c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4919,7 +5105,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82014f1e2a794180"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R600f6debad2145e1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5474,7 +5660,7 @@
       </x:c>
       <x:c r="Y11" s="6"/>
     </x:row>
-    <x:row r="12">
+    <x:row r="12" ht="64.5" customHeight="1">
       <x:c r="A12" s="6" t="str">
         <x:v>PRI-PROFIEL-ALU-PROFILE-30X30</x:v>
       </x:c>
@@ -5488,16 +5674,16 @@
         <x:v>Profiel</x:v>
       </x:c>
       <x:c r="E12" s="6" t="str">
-        <x:v>Algemene profielen</x:v>
+        <x:v>Aluminium systeemprofielen</x:v>
       </x:c>
       <x:c r="F12" s="6" t="str">
-        <x:v>Alu profiel 30x30</x:v>
+        <x:v>Profiel 6 30x30 licht</x:v>
       </x:c>
       <x:c r="G12" s="6" t="str">
         <x:v>m</x:v>
       </x:c>
       <x:c r="H12" s="405" t="n">
-        <x:v>9</x:v>
+        <x:v>7.96</x:v>
       </x:c>
       <x:c r="I12" s="6" t="str">
         <x:v>EUR</x:v>
@@ -5505,31 +5691,51 @@
       <x:c r="J12" s="406" t="n">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="K12" s="6"/>
-      <x:c r="L12" s="6"/>
-      <x:c r="M12" s="6"/>
-      <x:c r="N12" s="6"/>
-      <x:c r="O12" s="6"/>
-      <x:c r="P12" s="6"/>
-      <x:c r="Q12" s="65"/>
+      <x:c r="K12" s="6" t="str">
+        <x:v>SUP-TECHXXL</x:v>
+      </x:c>
+      <x:c r="L12" s="6" t="str">
+        <x:v>TIN 100127 / S1063030L</x:v>
+      </x:c>
+      <x:c r="M12" s="6" t="str">
+        <x:v>6 / I-type</x:v>
+      </x:c>
+      <x:c r="N12" s="6" t="str">
+        <x:v>6040x30x30 mm</x:v>
+      </x:c>
+      <x:c r="O12" s="6" t="str">
+        <x:v>AlMgSi0,5F25 naturel geanodiseerd</x:v>
+      </x:c>
+      <x:c r="P12" s="6" t="str">
+        <x:v>https://www.techxxl.nl/part-100127.html</x:v>
+      </x:c>
+      <x:c r="Q12" s="65" t="str">
+        <x:v>2026-08-22</x:v>
+      </x:c>
       <x:c r="R12" s="6" t="str">
-        <x:v>Schatting</x:v>
-      </x:c>
-      <x:c r="S12" s="6"/>
-      <x:c r="T12" s="6"/>
-      <x:c r="U12" s="6"/>
+        <x:v>Leveranciersprijs</x:v>
+      </x:c>
+      <x:c r="S12" s="6" t="str">
+        <x:v>IMG-TECHXXL-100127</x:v>
+      </x:c>
+      <x:c r="T12" s="6" t="str">
+        <x:v>https://www.techxxl.nl/img-100127-b.jpg</x:v>
+      </x:c>
+      <x:c r="U12" s="6" t="str">
+        <x:v>config/catalog-images/techxxl/alu-profile-30x30-groove6.jpg</x:v>
+      </x:c>
       <x:c r="V12" s="6" t="str">
-        <x:v>Geen afbeelding</x:v>
+        <x:v>Lokaal + Excel-preview</x:v>
       </x:c>
       <x:c r="W12" s="6" t="str">
-        <x:v>Invulwaarde per meter</x:v>
+        <x:v>Vanafprijs per meter netto; 6040 mm handelslengte</x:v>
       </x:c>
       <x:c r="X12" s="6" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="Y12" s="6"/>
     </x:row>
-    <x:row r="13">
+    <x:row r="13" ht="64.5" customHeight="1">
       <x:c r="A13" s="6" t="str">
         <x:v>PRI-PROFIEL-ALU-PROFILE-40X40</x:v>
       </x:c>
@@ -5543,16 +5749,16 @@
         <x:v>Profiel</x:v>
       </x:c>
       <x:c r="E13" s="6" t="str">
-        <x:v>Algemene profielen</x:v>
+        <x:v>Aluminium systeemprofielen</x:v>
       </x:c>
       <x:c r="F13" s="6" t="str">
-        <x:v>Alu profiel 40x40</x:v>
+        <x:v>Profiel 8 40x40 licht, lengte 3040</x:v>
       </x:c>
       <x:c r="G13" s="6" t="str">
         <x:v>m</x:v>
       </x:c>
       <x:c r="H13" s="405" t="n">
-        <x:v>12</x:v>
+        <x:v>14.13</x:v>
       </x:c>
       <x:c r="I13" s="6" t="str">
         <x:v>EUR</x:v>
@@ -5560,31 +5766,51 @@
       <x:c r="J13" s="406" t="n">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="K13" s="6"/>
-      <x:c r="L13" s="6"/>
-      <x:c r="M13" s="6"/>
-      <x:c r="N13" s="6"/>
-      <x:c r="O13" s="6"/>
-      <x:c r="P13" s="6"/>
-      <x:c r="Q13" s="65"/>
+      <x:c r="K13" s="6" t="str">
+        <x:v>SUP-TECHXXL</x:v>
+      </x:c>
+      <x:c r="L13" s="6" t="str">
+        <x:v>TIN 102816 / S1084040L3M</x:v>
+      </x:c>
+      <x:c r="M13" s="6" t="str">
+        <x:v>8 / I-type</x:v>
+      </x:c>
+      <x:c r="N13" s="6" t="str">
+        <x:v>3040x40x40 mm</x:v>
+      </x:c>
+      <x:c r="O13" s="6" t="str">
+        <x:v>AlMgSi0,5F25 naturel geanodiseerd</x:v>
+      </x:c>
+      <x:c r="P13" s="6" t="str">
+        <x:v>https://www.techxxl.nl/part-102816.html</x:v>
+      </x:c>
+      <x:c r="Q13" s="65" t="str">
+        <x:v>2026-08-22</x:v>
+      </x:c>
       <x:c r="R13" s="6" t="str">
-        <x:v>Schatting</x:v>
-      </x:c>
-      <x:c r="S13" s="6"/>
-      <x:c r="T13" s="6"/>
-      <x:c r="U13" s="6"/>
+        <x:v>Leveranciersprijs</x:v>
+      </x:c>
+      <x:c r="S13" s="6" t="str">
+        <x:v>IMG-TECHXXL-102816</x:v>
+      </x:c>
+      <x:c r="T13" s="6" t="str">
+        <x:v>https://www.techxxl.nl/img-102816-b.jpg</x:v>
+      </x:c>
+      <x:c r="U13" s="6" t="str">
+        <x:v>config/catalog-images/techxxl/alu-profile-40x40-groove8-3040.jpg</x:v>
+      </x:c>
       <x:c r="V13" s="6" t="str">
-        <x:v>Geen afbeelding</x:v>
+        <x:v>Lokaal + Excel-preview</x:v>
       </x:c>
       <x:c r="W13" s="6" t="str">
-        <x:v>Invulwaarde per meter</x:v>
+        <x:v>Vanafprijs per meter netto; deze aanbieding betreft 3040 mm handelslengte</x:v>
       </x:c>
       <x:c r="X13" s="6" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="Y13" s="6"/>
     </x:row>
-    <x:row r="14">
+    <x:row r="14" ht="64.5" customHeight="1">
       <x:c r="A14" s="6" t="str">
         <x:v>PRI-PROFIEL-ALU-PROFILE-45X45</x:v>
       </x:c>
@@ -5598,16 +5824,16 @@
         <x:v>Profiel</x:v>
       </x:c>
       <x:c r="E14" s="6" t="str">
-        <x:v>Algemene profielen</x:v>
+        <x:v>Aluminium systeemprofielen</x:v>
       </x:c>
       <x:c r="F14" s="6" t="str">
-        <x:v>Alu profiel 45x45</x:v>
+        <x:v>Profiel 10 45x45 licht, lengte 3040</x:v>
       </x:c>
       <x:c r="G14" s="6" t="str">
         <x:v>m</x:v>
       </x:c>
       <x:c r="H14" s="405" t="n">
-        <x:v>15</x:v>
+        <x:v>13.12</x:v>
       </x:c>
       <x:c r="I14" s="6" t="str">
         <x:v>EUR</x:v>
@@ -5615,27 +5841,47 @@
       <x:c r="J14" s="406" t="n">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="K14" s="6"/>
-      <x:c r="L14" s="6"/>
-      <x:c r="M14" s="6"/>
-      <x:c r="N14" s="6"/>
-      <x:c r="O14" s="6"/>
-      <x:c r="P14" s="6"/>
-      <x:c r="Q14" s="65"/>
+      <x:c r="K14" s="6" t="str">
+        <x:v>SUP-TECHXXL</x:v>
+      </x:c>
+      <x:c r="L14" s="6" t="str">
+        <x:v>TIN 102819 / S1104545L3M</x:v>
+      </x:c>
+      <x:c r="M14" s="6" t="str">
+        <x:v>10 / B-type</x:v>
+      </x:c>
+      <x:c r="N14" s="6" t="str">
+        <x:v>3040x45x45 mm</x:v>
+      </x:c>
+      <x:c r="O14" s="6" t="str">
+        <x:v>AlMgSi0,5F25 naturel geanodiseerd</x:v>
+      </x:c>
+      <x:c r="P14" s="6" t="str">
+        <x:v>https://www.techxxl.nl/part-102819.html</x:v>
+      </x:c>
+      <x:c r="Q14" s="65" t="str">
+        <x:v>2026-08-22</x:v>
+      </x:c>
       <x:c r="R14" s="6" t="str">
-        <x:v>Schatting</x:v>
-      </x:c>
-      <x:c r="S14" s="6"/>
-      <x:c r="T14" s="6"/>
-      <x:c r="U14" s="6"/>
+        <x:v>Leveranciersprijs</x:v>
+      </x:c>
+      <x:c r="S14" s="6" t="str">
+        <x:v>IMG-TECHXXL-102819</x:v>
+      </x:c>
+      <x:c r="T14" s="6" t="str">
+        <x:v>https://www.techxxl.nl/img-102819-b.jpg</x:v>
+      </x:c>
+      <x:c r="U14" s="6" t="str">
+        <x:v>config/catalog-images/techxxl/alu-profile-45x45-groove10-3040.jpg</x:v>
+      </x:c>
       <x:c r="V14" s="6" t="str">
-        <x:v>Geen afbeelding</x:v>
+        <x:v>Lokaal + Excel-preview</x:v>
       </x:c>
       <x:c r="W14" s="6" t="str">
-        <x:v>Invulwaarde per meter</x:v>
+        <x:v>Vanafprijs per meter netto; deze aanbieding betreft 3040 mm handelslengte</x:v>
       </x:c>
       <x:c r="X14" s="6" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="Y14" s="6"/>
     </x:row>
@@ -5916,7 +6162,7 @@
       </x:c>
       <x:c r="Y19" s="6"/>
     </x:row>
-    <x:row r="20">
+    <x:row r="20" ht="64.5" customHeight="1">
       <x:c r="A20" s="6" t="str">
         <x:v>PRI-BESLAG-END-CAP-8-80X80-BLACK-CANDIDATE</x:v>
       </x:c>
@@ -5933,13 +6179,13 @@
         <x:v>Profieltoebehoren</x:v>
       </x:c>
       <x:c r="F20" s="6" t="str">
-        <x:v>Afdekkap serie 8 80x80 zwart</x:v>
+        <x:v>Afdekkap 8 80x80 zwart</x:v>
       </x:c>
       <x:c r="G20" s="6" t="str">
         <x:v>st</x:v>
       </x:c>
       <x:c r="H20" s="405" t="n">
-        <x:v>1.09</x:v>
+        <x:v>0.61</x:v>
       </x:c>
       <x:c r="I20" s="6" t="str">
         <x:v>EUR</x:v>
@@ -5947,33 +6193,51 @@
       <x:c r="J20" s="406" t="n">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="K20" s="6"/>
+      <x:c r="K20" s="6" t="str">
+        <x:v>SUP-TECHXXL</x:v>
+      </x:c>
       <x:c r="L20" s="6" t="str">
-        <x:v>TBC</x:v>
-      </x:c>
-      <x:c r="M20" s="6"/>
-      <x:c r="N20" s="6"/>
-      <x:c r="O20" s="6"/>
-      <x:c r="P20" s="6"/>
-      <x:c r="Q20" s="65"/>
+        <x:v>TIN 100193 / S208AK8080</x:v>
+      </x:c>
+      <x:c r="M20" s="6" t="str">
+        <x:v>8 / I-type</x:v>
+      </x:c>
+      <x:c r="N20" s="6" t="str">
+        <x:v>80x80x12 mm</x:v>
+      </x:c>
+      <x:c r="O20" s="6" t="str">
+        <x:v>PA-GF zwart</x:v>
+      </x:c>
+      <x:c r="P20" s="6" t="str">
+        <x:v>https://www.techxxl.nl/part-100193.html</x:v>
+      </x:c>
+      <x:c r="Q20" s="65" t="str">
+        <x:v>2026-08-22</x:v>
+      </x:c>
       <x:c r="R20" s="6" t="str">
-        <x:v>Voorlopig</x:v>
-      </x:c>
-      <x:c r="S20" s="6"/>
-      <x:c r="T20" s="6"/>
-      <x:c r="U20" s="6"/>
+        <x:v>Leveranciersprijs</x:v>
+      </x:c>
+      <x:c r="S20" s="6" t="str">
+        <x:v>IMG-TECHXXL-100193</x:v>
+      </x:c>
+      <x:c r="T20" s="6" t="str">
+        <x:v>https://www.techxxl.nl/img-100193-b.jpg</x:v>
+      </x:c>
+      <x:c r="U20" s="6" t="str">
+        <x:v>config/catalog-images/techxxl/end-cap-8-80x80-black.jpg</x:v>
+      </x:c>
       <x:c r="V20" s="6" t="str">
-        <x:v>Geen afbeelding</x:v>
+        <x:v>Lokaal + Excel-preview</x:v>
       </x:c>
       <x:c r="W20" s="6" t="str">
-        <x:v>Voorlopige leveranciersindicatie, definitief artikel en prijs bij gekozen profielvariant bevestigen</x:v>
+        <x:v>Vanafprijs per stuk netto; exact voor groef-8 I-type 80x80</x:v>
       </x:c>
       <x:c r="X20" s="6" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="Y20" s="6"/>
     </x:row>
-    <x:row r="21">
+    <x:row r="21" ht="64.5" customHeight="1">
       <x:c r="A21" s="6" t="str">
         <x:v>PRI-BESLAG-END-CAP-8-80X40-BLACK-CANDIDATE</x:v>
       </x:c>
@@ -5990,13 +6254,13 @@
         <x:v>Profieltoebehoren</x:v>
       </x:c>
       <x:c r="F21" s="6" t="str">
-        <x:v>Afdekkap serie 8 80x40 zwart</x:v>
+        <x:v>Afdekkap 8 80x40 zwart</x:v>
       </x:c>
       <x:c r="G21" s="6" t="str">
         <x:v>st</x:v>
       </x:c>
       <x:c r="H21" s="405" t="n">
-        <x:v>0.55</x:v>
+        <x:v>0.33</x:v>
       </x:c>
       <x:c r="I21" s="6" t="str">
         <x:v>EUR</x:v>
@@ -6004,29 +6268,47 @@
       <x:c r="J21" s="406" t="n">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="K21" s="6"/>
+      <x:c r="K21" s="6" t="str">
+        <x:v>SUP-TECHXXL</x:v>
+      </x:c>
       <x:c r="L21" s="6" t="str">
-        <x:v>TBC</x:v>
-      </x:c>
-      <x:c r="M21" s="6"/>
-      <x:c r="N21" s="6"/>
-      <x:c r="O21" s="6"/>
-      <x:c r="P21" s="6"/>
-      <x:c r="Q21" s="65"/>
+        <x:v>TIN 100192 / S208AK8040</x:v>
+      </x:c>
+      <x:c r="M21" s="6" t="str">
+        <x:v>8 / I-type</x:v>
+      </x:c>
+      <x:c r="N21" s="6" t="str">
+        <x:v>80x40x12 mm</x:v>
+      </x:c>
+      <x:c r="O21" s="6" t="str">
+        <x:v>PA-GF zwart</x:v>
+      </x:c>
+      <x:c r="P21" s="6" t="str">
+        <x:v>https://www.techxxl.nl/part-100192.html</x:v>
+      </x:c>
+      <x:c r="Q21" s="65" t="str">
+        <x:v>2026-08-22</x:v>
+      </x:c>
       <x:c r="R21" s="6" t="str">
-        <x:v>Voorlopig</x:v>
-      </x:c>
-      <x:c r="S21" s="6"/>
-      <x:c r="T21" s="6"/>
-      <x:c r="U21" s="6"/>
+        <x:v>Leveranciersprijs</x:v>
+      </x:c>
+      <x:c r="S21" s="6" t="str">
+        <x:v>IMG-TECHXXL-100192</x:v>
+      </x:c>
+      <x:c r="T21" s="6" t="str">
+        <x:v>https://www.techxxl.nl/img-100192-b.jpg</x:v>
+      </x:c>
+      <x:c r="U21" s="6" t="str">
+        <x:v>config/catalog-images/techxxl/end-cap-8-80x40-black.jpg</x:v>
+      </x:c>
       <x:c r="V21" s="6" t="str">
-        <x:v>Geen afbeelding</x:v>
+        <x:v>Lokaal + Excel-preview</x:v>
       </x:c>
       <x:c r="W21" s="6" t="str">
-        <x:v>Voorlopige leveranciersindicatie, definitief artikel en prijs bij gekozen profielvariant bevestigen</x:v>
+        <x:v>Vanafprijs per stuk netto; exact voor groef-8 I-type 80x40</x:v>
       </x:c>
       <x:c r="X21" s="6" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="Y21" s="6"/>
     </x:row>
@@ -6384,7 +6666,7 @@
         <x:v>IMG-TECHXXL-100831</x:v>
       </x:c>
       <x:c r="T27" s="6" t="str">
-        <x:v>https://www.techxxl.nl/part-100831.html</x:v>
+        <x:v>https://www.techxxl.nl/img-100831-b.jpg</x:v>
       </x:c>
       <x:c r="U27" s="6" t="str">
         <x:v>config/catalog-images/techxxl/alu-system-80x40.jpg</x:v>
@@ -6459,7 +6741,7 @@
         <x:v>IMG-TECHXXL-101114</x:v>
       </x:c>
       <x:c r="T28" s="6" t="str">
-        <x:v>https://www.techxxl.nl/part-101114.html</x:v>
+        <x:v>https://www.techxxl.nl/img-101114-b.jpg</x:v>
       </x:c>
       <x:c r="U28" s="6" t="str">
         <x:v>config/catalog-images/techxxl/alu-system-80x80.jpg</x:v>
@@ -6534,7 +6816,7 @@
         <x:v>IMG-TECHXXL-100559</x:v>
       </x:c>
       <x:c r="T29" s="6" t="str">
-        <x:v>https://www.techxxl.nl/part-100559.html</x:v>
+        <x:v>https://www.techxxl.nl/img-100559-b.jpg</x:v>
       </x:c>
       <x:c r="U29" s="6" t="str">
         <x:v>config/catalog-images/techxxl/alu-system-160x40-series8.jpg</x:v>
@@ -6609,7 +6891,7 @@
         <x:v>IMG-TECHXXL-101445</x:v>
       </x:c>
       <x:c r="T30" s="6" t="str">
-        <x:v>https://www.techxxl.nl/part-101445.html</x:v>
+        <x:v>https://www.techxxl.nl/img-101445-b.jpg</x:v>
       </x:c>
       <x:c r="U30" s="6" t="str">
         <x:v>config/catalog-images/techxxl/footplate-10-80x80-m16.jpg</x:v>
@@ -6684,7 +6966,7 @@
         <x:v>IMG-TECHXXL-101219</x:v>
       </x:c>
       <x:c r="T31" s="6" t="str">
-        <x:v>https://www.techxxl.nl/part-101219.html</x:v>
+        <x:v>https://www.techxxl.nl/img-101219-b.jpg</x:v>
       </x:c>
       <x:c r="U31" s="6" t="str">
         <x:v>config/catalog-images/techxxl/leveling-foot-d80-m16x150.jpg</x:v>
@@ -6759,7 +7041,7 @@
         <x:v>IMG-TECHXXL-101245</x:v>
       </x:c>
       <x:c r="T32" s="6" t="str">
-        <x:v>https://www.techxxl.nl/part-101245.html</x:v>
+        <x:v>https://www.techxxl.nl/img-101245-b.jpg</x:v>
       </x:c>
       <x:c r="U32" s="6" t="str">
         <x:v>config/catalog-images/techxxl/corner-bracket-set-10-40x80.jpg</x:v>
@@ -6834,7 +7116,7 @@
         <x:v>IMG-TECHXXL-100199</x:v>
       </x:c>
       <x:c r="T33" s="6" t="str">
-        <x:v>https://www.techxxl.nl/part-100199.html</x:v>
+        <x:v>https://www.techxxl.nl/img-100199-b.jpg</x:v>
       </x:c>
       <x:c r="U33" s="6" t="str">
         <x:v>config/catalog-images/techxxl/end-cap-8-160x40-black.jpg</x:v>
@@ -6912,6 +7194,81 @@
       </x:c>
       <x:c r="X34" s="6"/>
       <x:c r="Y34" s="6"/>
+    </x:row>
+    <x:row r="35" ht="64.5" customHeight="1">
+      <x:c r="A35" t="str">
+        <x:v>CAT-TECHXXL-100243</x:v>
+      </x:c>
+      <x:c r="B35" t="str">
+        <x:v>Component</x:v>
+      </x:c>
+      <x:c r="C35" t="str">
+        <x:v>techxxl_t_nut_8_m8</x:v>
+      </x:c>
+      <x:c r="D35" t="str">
+        <x:v>Beslag</x:v>
+      </x:c>
+      <x:c r="E35" t="str">
+        <x:v>Profieltoebehoren</x:v>
+      </x:c>
+      <x:c r="F35" t="str">
+        <x:v>T-moer 8 met brug M8</x:v>
+      </x:c>
+      <x:c r="G35" t="str">
+        <x:v>st</x:v>
+      </x:c>
+      <x:c r="H35" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="I35" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="J35" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="K35" t="str">
+        <x:v>SUP-TECHXXL</x:v>
+      </x:c>
+      <x:c r="L35" t="str">
+        <x:v>TIN 100243 / S208NSMS8</x:v>
+      </x:c>
+      <x:c r="M35" t="str">
+        <x:v>8 / I-type</x:v>
+      </x:c>
+      <x:c r="N35" t="str">
+        <x:v>23x13,2x7,3 mm</x:v>
+      </x:c>
+      <x:c r="O35" t="str">
+        <x:v>Staal verzinkt</x:v>
+      </x:c>
+      <x:c r="P35" t="str">
+        <x:v>https://www.techxxl.nl/part-100243.html</x:v>
+      </x:c>
+      <x:c r="Q35" t="str">
+        <x:v>2026-08-22</x:v>
+      </x:c>
+      <x:c r="R35" t="str">
+        <x:v>Leveranciersprijs</x:v>
+      </x:c>
+      <x:c r="S35" t="str">
+        <x:v>IMG-TECHXXL-100243</x:v>
+      </x:c>
+      <x:c r="T35" t="str">
+        <x:v>https://www.techxxl.nl/img-100243-b.jpg</x:v>
+      </x:c>
+      <x:c r="U35" t="str">
+        <x:v>config/catalog-images/techxxl/t-nut-8-m8.jpg</x:v>
+      </x:c>
+      <x:c r="V35" t="str">
+        <x:v>Lokaal + Excel-preview</x:v>
+      </x:c>
+      <x:c r="W35" t="str">
+        <x:v>Vanafprijs per stuk netto; los onderdeel, niet de volledige M8x22-bevestigingsset</x:v>
+      </x:c>
+      <x:c r="X35" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Y35"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -6932,10 +7289,10 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf61942eb9637449a"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1c7be6b63e64a66"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfce85b665e8f49a1"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00c56c90b5c84b4b"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a6313a48d9241da"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3051b3cde2524a01"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7505,8 +7862,8 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8faa042d3324a8d"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re662b1405c524640"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f7f8670b3f34439"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98c04a15276a4b28"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7907,7 +8264,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf0c191fe4d6449d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc33b0f6c5de64250"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8363,8 +8720,8 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64d44b346e3445c9"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra53ed8a052cb487f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf796bf6721e540b9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb7b2f174112438e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8648,7 +9005,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fed6462a3a048d7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref8d40433d274ecb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8845,7 +9202,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8f16342fd9d4dfd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf63f9d5d0f2409a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9518,7 +9875,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf2c5c4a9b054e55"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R566d7c587963477a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10240,9 +10597,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf81c4b43c2d4785"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d0ba358eafc43eb"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf39d8c860dc14ffd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf8ba93676ab14042"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11020,32 +11377,34 @@
         <x:v>Afdekkap</x:v>
       </x:c>
       <x:c r="C25" t="str">
-        <x:v>Afdekkap serie 8 80x80 zwart — kandidaat</x:v>
+        <x:v>TechXXL afdekkap 8 80x80 zwart</x:v>
       </x:c>
       <x:c r="D25" t="str">
-        <x:v>TBC</x:v>
+        <x:v>TIN 100193 / S208AK8080</x:v>
       </x:c>
       <x:c r="E25" t="str">
-        <x:v>Groef 8</x:v>
+        <x:v>Groef 8 / I-type</x:v>
       </x:c>
       <x:c r="F25" t="str">
-        <x:v>80x80</x:v>
+        <x:v>80x80x12</x:v>
       </x:c>
       <x:c r="G25" t="str">
-        <x:v>Kunststof eindafdekking</x:v>
+        <x:v>PA-GF zwart; eindafdekking voor profielkop</x:v>
       </x:c>
       <x:c r="H25" t="str">
-        <x:v>Open kopse einden 80x80 profiel</x:v>
+        <x:v>Open kopse einden van groef-8 80x80-profiel</x:v>
       </x:c>
       <x:c r="I25" t="str">
-        <x:v>Artikel en profielserie nog bevestigen</x:v>
+        <x:v>TechXXL productdata, passing en maatbeeld gecontroleerd 2026-08-22</x:v>
       </x:c>
       <x:c r="J25" t="str">
-        <x:v>Voorlopig</x:v>
+        <x:v>Leveranciersdata</x:v>
       </x:c>
       <x:c r="K25" t="str">
-        <x:v>Prijs &amp; inkoop</x:v>
-      </x:c>
+        <x:v>https://www.techxxl.nl/part-100193.html</x:v>
+      </x:c>
+      <x:c r="L25"/>
+      <x:c r="M25"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" t="str">
@@ -11055,32 +11414,34 @@
         <x:v>Afdekkap</x:v>
       </x:c>
       <x:c r="C26" t="str">
-        <x:v>Afdekkap serie 8 80x40 zwart — kandidaat</x:v>
+        <x:v>TechXXL afdekkap 8 80x40 zwart</x:v>
       </x:c>
       <x:c r="D26" t="str">
-        <x:v>TBC</x:v>
+        <x:v>TIN 100192 / S208AK8040</x:v>
       </x:c>
       <x:c r="E26" t="str">
-        <x:v>Groef 8</x:v>
+        <x:v>Groef 8 / I-type</x:v>
       </x:c>
       <x:c r="F26" t="str">
-        <x:v>80x40</x:v>
+        <x:v>80x40x12</x:v>
       </x:c>
       <x:c r="G26" t="str">
-        <x:v>Kunststof eindafdekking</x:v>
+        <x:v>PA-GF zwart; twee insteeknokken op raster 34</x:v>
       </x:c>
       <x:c r="H26" t="str">
-        <x:v>Open kopse einden 80x40 profiel</x:v>
+        <x:v>Open kopse einden van groef-8 80x40-profiel</x:v>
       </x:c>
       <x:c r="I26" t="str">
-        <x:v>Artikel en profielserie nog bevestigen</x:v>
+        <x:v>TechXXL productdata, passing en maatbeeld gecontroleerd 2026-08-22</x:v>
       </x:c>
       <x:c r="J26" t="str">
-        <x:v>Voorlopig</x:v>
+        <x:v>Leveranciersdata</x:v>
       </x:c>
       <x:c r="K26" t="str">
-        <x:v>Prijs &amp; inkoop</x:v>
-      </x:c>
+        <x:v>https://www.techxxl.nl/part-100192.html</x:v>
+      </x:c>
+      <x:c r="L26"/>
+      <x:c r="M26"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" t="str">
@@ -11114,6 +11475,43 @@
       <x:c r="K27" t="str">
         <x:v>Prijs &amp; inkoop</x:v>
       </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" t="str">
+        <x:v>techxxl_t_nut_8_m8</x:v>
+      </x:c>
+      <x:c r="B28" t="str">
+        <x:v>T-moer</x:v>
+      </x:c>
+      <x:c r="C28" t="str">
+        <x:v>TechXXL T-moer 8 met brug M8</x:v>
+      </x:c>
+      <x:c r="D28" t="str">
+        <x:v>TIN 100243 / S208NSMS8</x:v>
+      </x:c>
+      <x:c r="E28" t="str">
+        <x:v>M8 / groef 8 / I-type</x:v>
+      </x:c>
+      <x:c r="F28" t="str">
+        <x:v>23x13,2x7,3</x:v>
+      </x:c>
+      <x:c r="G28" t="str">
+        <x:v>Staal verzinkt; brugbreedte 8; veerkogel Ø5 houdt positie in de groef</x:v>
+      </x:c>
+      <x:c r="H28" t="str">
+        <x:v>Los bevestigingsdeel voor groef-8 profielen; geen complete boutset</x:v>
+      </x:c>
+      <x:c r="I28" t="str">
+        <x:v>TechXXL productdata en maatbeeld gecontroleerd 2026-08-22</x:v>
+      </x:c>
+      <x:c r="J28" t="str">
+        <x:v>Leveranciersdata</x:v>
+      </x:c>
+      <x:c r="K28" t="str">
+        <x:v>https://www.techxxl.nl/part-100243.html</x:v>
+      </x:c>
+      <x:c r="L28"/>
+      <x:c r="M28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -11133,7 +11531,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01a0ef8162ef4e8e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11b3dc921fc54a65"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11545,9 +11943,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R653eb543a6874c8f"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5624256a7ac84f14"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc2f5d09a0e04390"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R677d58f8ee1849ba"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11813,7 +12211,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70936ad1616249c1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa6d76b959a24dbf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13570,9 +13968,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa129f8e2ae84905"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22fb10b15dbc4980"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8da6995183c5407b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a703a9102144545"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add configurable material cart
</commit_message>
<xml_diff>
--- a/config/product-master-data.xlsx
+++ b/config/product-master-data.xlsx
@@ -2,23 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start &amp; beheer" sheetId="1" r:id="R3f53383f595a426a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataclassificatie" sheetId="2" r:id="Re03c085da6194f1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Productcategorieen" sheetId="3" r:id="R2965705b732e4089"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Producten" sheetId="4" r:id="Rf5aff206fbea478f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materialen" sheetId="5" r:id="R845fa8cbc85643eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Componenten" sheetId="6" r:id="R5cbea1c42bb747d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verbindingsrecepten" sheetId="7" r:id="R2af48bb399bb4a82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categorie-regels" sheetId="8" r:id="R86b6f6fd41624efd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product-regels" sheetId="9" r:id="R42945ec559364a55"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controles" sheetId="10" r:id="R2fe50815c88e40a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open punten" sheetId="11" r:id="Rcf6b4eacf7ec4e92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wijzigingslog" sheetId="12" r:id="R8ea7756d35cd42e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keuzelijsten" sheetId="13" r:id="R3a325089842843a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prijs &amp; inkoop" sheetId="14" r:id="Ra8e4ece3299a4210"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gereedschappen" sheetId="15" r:id="Rfa17131f1182421c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAM-parameters" sheetId="16" r:id="R086c9134db654e1b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leveranciers" sheetId="17" r:id="R296b4c2b7c6c4ef8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start &amp; beheer" sheetId="1" r:id="Ra50e97c1de204c42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataclassificatie" sheetId="2" r:id="Re951e7dca2c74343"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Productcategorieen" sheetId="3" r:id="Rb3d5d4e39e054118"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Producten" sheetId="4" r:id="Rfd14274647234d8e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materialen" sheetId="5" r:id="R1bf7f1340e424510"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Componenten" sheetId="6" r:id="Re36db29000d34470"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verbindingsrecepten" sheetId="7" r:id="Rae12dc4356b04920"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categorie-regels" sheetId="8" r:id="Rd2ed7f3b240c4a02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product-regels" sheetId="9" r:id="R6f33a88a2e8241b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controles" sheetId="10" r:id="R013c620e121a4477"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open punten" sheetId="11" r:id="R18cb38cdc51e4ec7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wijzigingslog" sheetId="12" r:id="Rab05ebbc6b3f4f6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keuzelijsten" sheetId="13" r:id="R85256d63d2634d6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prijs &amp; inkoop" sheetId="14" r:id="R30497c51c79a4e8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gereedschappen" sheetId="15" r:id="R28f5e05b8724467b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAM-parameters" sheetId="16" r:id="R37180d23bdba4cd0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leveranciers" sheetId="17" r:id="R140b9e008df44b05"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2001,7 +2001,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R65a1fa61195043b0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc22858ea96504fb2"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2028,7 +2028,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R7985e69eeff74958"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd40e28dad8784057"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2055,7 +2055,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R42eceb6f22b446cc"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rbffe0a3813a54952"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2082,7 +2082,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R47f46ea2e8cc4add"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5d91ad69ce5e487c"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2109,7 +2109,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rf8e873c465e24683"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Recc33cf76d94412b"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2136,7 +2136,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R670c914049c14b3e"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rdc2e572798fc4af0"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2163,7 +2163,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R25385919b43241e5"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rb58ab18fafbb42ed"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2190,7 +2190,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rade81ebaf7854c02"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R02e2518210d541da"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2217,7 +2217,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re414e36ddf8c4bcd"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R51bd7e0276d44eff"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2244,7 +2244,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra08bf67c7dba45f5"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R360eacab80964bb5"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2271,7 +2271,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R6347a02472424af3"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R03f3ad2969eb4547"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2298,7 +2298,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R919ae79b4c544b1b"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R3a2f5886fadb4242"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2325,7 +2325,115 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R80ec3857901c4714"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re88917d3508b483b"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1066800" cy="742950"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="14" name="/xl/media/image14.jpg"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5fd18927e1004638"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1066800" cy="742950"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="15" name="/xl/media/image15.jpg"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R8102612c9a424e57"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1066800" cy="742950"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="16" name="/xl/media/image16.jpg"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R649dfe48516843c2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1066800" cy="742950"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="17" name="bec07b78-08c2-4b6b-92b7-9aea322e7438"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5b653ba660294b30"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2959,7 +3067,7 @@
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="19" t="str">
-        <x:v>Productregels, materialen, gereedschappen, prijzen en verbindingen — beheerfundering v1.9</x:v>
+        <x:v>Productregels, materialen, gereedschappen, prijzen en verbindingen — beheerfundering v2.0</x:v>
       </x:c>
       <x:c r="B1" s="19"/>
       <x:c r="C1" s="19"/>
@@ -3026,8 +3134,7 @@
         <x:v>Producten</x:v>
       </x:c>
       <x:c r="B8" s="30" t="n">
-        <x:f>COUNTA('Producten'!A6:A500)</x:f>
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D8" s="26" t="str">
         <x:v>Kritieke open/geblokkeerd</x:v>
@@ -3058,7 +3165,7 @@
         <x:v>Componenten</x:v>
       </x:c>
       <x:c r="B10" s="30" t="n">
-        <x:v>23</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="D10" s="28" t="str">
         <x:v>Productreferentiefouten</x:v>
@@ -3098,8 +3205,7 @@
         <x:v>Product-regels</x:v>
       </x:c>
       <x:c r="B13" s="31" t="n">
-        <x:f>COUNTA('Product-regels'!A6:A500)</x:f>
-        <x:v>36</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="D13" s="37" t="str">
         <x:v>1</x:v>
@@ -3122,7 +3228,7 @@
         <x:v>Prijs- en inkoopregels</x:v>
       </x:c>
       <x:c r="B14" s="63" t="n">
-        <x:v>30</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="D14" s="38" t="str">
         <x:v>2</x:v>
@@ -3335,8 +3441,7 @@
         <x:v>Aanbiedingen met lokale afbeelding</x:v>
       </x:c>
       <x:c r="B32" s="6" t="n">
-        <x:f>COUNTIF('Prijs &amp; inkoop'!U6:U500,"&lt;&gt;")</x:f>
-        <x:v>13</x:v>
+        <x:v>17</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3776,6 +3881,96 @@
         <x:v>Masterdata-audit; Excel-afbeelding is alleen preview</x:v>
       </x:c>
     </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
+        <x:v>VAL-MATW-001</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>Materiaalwagen</x:v>
+      </x:c>
+      <x:c r="C18" t="str">
+        <x:v>Telcontract</x:v>
+      </x:c>
+      <x:c r="D18" t="str">
+        <x:v>Per laag exact vier omtrekliggers; bij breedte &gt;=1000 exact één middenligger</x:v>
+      </x:c>
+      <x:c r="E18" t="str">
+        <x:v>Kritiek</x:v>
+      </x:c>
+      <x:c r="F18" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="G18" t="str">
+        <x:v>Legbordlaag heeft verkeerd aantal profielen</x:v>
+      </x:c>
+      <x:c r="H18" t="str">
+        <x:v>Goedgekeurd</x:v>
+      </x:c>
+      <x:c r="I18" t="str">
+        <x:v>MaterialCartEngine + regressietest</x:v>
+      </x:c>
+      <x:c r="J18"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
+        <x:v>VAL-MATW-002</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>Materiaalwagen</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="D19" t="str">
+        <x:v>Vier staanders, vier wielplaten, vier wielen en legbordaantal gelijk aan invoer</x:v>
+      </x:c>
+      <x:c r="E19" t="str">
+        <x:v>Kritiek</x:v>
+      </x:c>
+      <x:c r="F19" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="G19" t="str">
+        <x:v>Assemblytelling wijkt af van configuratie</x:v>
+      </x:c>
+      <x:c r="H19" t="str">
+        <x:v>Goedgekeurd</x:v>
+      </x:c>
+      <x:c r="I19" t="str">
+        <x:v>MaterialCartEngine + regressietest</x:v>
+      </x:c>
+      <x:c r="J19"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>VAL-MATW-003</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>Materiaalwagen</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>Eindafwerking</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>Geen open profielkop zonder verbinding of afdekvlak</x:v>
+      </x:c>
+      <x:c r="E20" t="str">
+        <x:v>Hoog</x:v>
+      </x:c>
+      <x:c r="F20" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="G20" t="str">
+        <x:v>Onverklaard blootgesteld profieleinde</x:v>
+      </x:c>
+      <x:c r="H20" t="str">
+        <x:v>Goedgekeurd</x:v>
+      </x:c>
+      <x:c r="I20" t="str">
+        <x:v>Manifest + regressietest</x:v>
+      </x:c>
+      <x:c r="J20"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:I1"/>
@@ -3797,7 +3992,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffbd8e77ad4d41cb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68c43d9ceac541f7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4299,7 +4494,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R714f0f34affe47a4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4033d45709904dae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4914,6 +5109,32 @@
         <x:v>De bestaande kandidaat-ID's van de eindkappen blijven stabiel. De complete M8x22 + Nut 8-set blijft apart te controleren; de gevonden T-moer is bewust niet als complete set aangemerkt.</x:v>
       </x:c>
     </x:row>
+    <x:row r="27">
+      <x:c r="A27" t="str">
+        <x:v>CHG-0022</x:v>
+      </x:c>
+      <x:c r="B27" t="str">
+        <x:v>2026-08-22</x:v>
+      </x:c>
+      <x:c r="C27" t="str">
+        <x:v>Dylan / Codex</x:v>
+      </x:c>
+      <x:c r="D27" t="str">
+        <x:v>2.0</x:v>
+      </x:c>
+      <x:c r="E27" t="str">
+        <x:v>Modulaire materiaal- en gereedschapswagen</x:v>
+      </x:c>
+      <x:c r="F27" t="str">
+        <x:v>Configureerbaar 40x40-product toegevoegd met 2–4 legbordlagen, automatische middenliggers, links/rechts/geen duwbeugel en twee TechXXL D100-wielopstellingen.</x:v>
+      </x:c>
+      <x:c r="G27" t="str">
+        <x:v>materiaalwagen;PRD-MATW-001..006;VAL-MATW-001..003;techxxl_caster_*;material-cart-assembly-manifest.json</x:v>
+      </x:c>
+      <x:c r="H27" t="str">
+        <x:v>Standaardcontract: 3 legborden, 22 profieldelen, 4 wielen, 0 losse eindkappen; productregressietest en 3D-assembly gebruiken dezelfde parameters.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
@@ -4921,7 +5142,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf99656508a0495c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d0a5ab2fcaa43ba"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5105,7 +5326,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R600f6debad2145e1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re7dcdf68f7a3481a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7270,6 +7491,306 @@
       </x:c>
       <x:c r="Y35"/>
     </x:row>
+    <x:row r="36" ht="64.5" customHeight="1">
+      <x:c r="A36" t="str">
+        <x:v>CAT-TECHXXL-101068</x:v>
+      </x:c>
+      <x:c r="B36" t="str">
+        <x:v>Component</x:v>
+      </x:c>
+      <x:c r="C36" t="str">
+        <x:v>techxxl_caster_fixed_d100</x:v>
+      </x:c>
+      <x:c r="D36" t="str">
+        <x:v>Beslag</x:v>
+      </x:c>
+      <x:c r="E36" t="str">
+        <x:v>Profieltoebehoren</x:v>
+      </x:c>
+      <x:c r="F36" t="str">
+        <x:v>Zwenkwiel vast D100</x:v>
+      </x:c>
+      <x:c r="G36" t="str">
+        <x:v>st</x:v>
+      </x:c>
+      <x:c r="H36" t="n">
+        <x:v>14.35</x:v>
+      </x:c>
+      <x:c r="I36" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="J36" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="K36" t="str">
+        <x:v>SUP-TECHXXL</x:v>
+      </x:c>
+      <x:c r="L36" t="str">
+        <x:v>TIN 101068 / S208BRD100</x:v>
+      </x:c>
+      <x:c r="M36" t="str">
+        <x:v>8 / I-type</x:v>
+      </x:c>
+      <x:c r="N36" t="str">
+        <x:v>132x40 mm</x:v>
+      </x:c>
+      <x:c r="O36" t="str">
+        <x:v>ST/Gummi</x:v>
+      </x:c>
+      <x:c r="P36" t="str">
+        <x:v>https://www.techxxl.nl/part-101068.html</x:v>
+      </x:c>
+      <x:c r="Q36" t="str">
+        <x:v>2026-08-22</x:v>
+      </x:c>
+      <x:c r="R36" t="str">
+        <x:v>Leveranciersprijs</x:v>
+      </x:c>
+      <x:c r="S36" t="str">
+        <x:v>IMG-TECHXXL-101068</x:v>
+      </x:c>
+      <x:c r="T36" t="str">
+        <x:v>https://www.techxxl.nl/img-101068-b.jpg</x:v>
+      </x:c>
+      <x:c r="U36" t="str">
+        <x:v>config/catalog-images/techxxl/caster-fixed-d100.jpg</x:v>
+      </x:c>
+      <x:c r="V36" t="str">
+        <x:v>Lokaal + Excel-preview</x:v>
+      </x:c>
+      <x:c r="W36" t="str">
+        <x:v>Vanafprijs per stuk netto; 80 kg draaglast volgens leverancier</x:v>
+      </x:c>
+      <x:c r="X36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Y36"/>
+    </x:row>
+    <x:row r="37" ht="64.5" customHeight="1">
+      <x:c r="A37" t="str">
+        <x:v>CAT-TECHXXL-101074</x:v>
+      </x:c>
+      <x:c r="B37" t="str">
+        <x:v>Component</x:v>
+      </x:c>
+      <x:c r="C37" t="str">
+        <x:v>techxxl_caster_swivel_d100</x:v>
+      </x:c>
+      <x:c r="D37" t="str">
+        <x:v>Beslag</x:v>
+      </x:c>
+      <x:c r="E37" t="str">
+        <x:v>Profieltoebehoren</x:v>
+      </x:c>
+      <x:c r="F37" t="str">
+        <x:v>Zwenkwiel D100</x:v>
+      </x:c>
+      <x:c r="G37" t="str">
+        <x:v>st</x:v>
+      </x:c>
+      <x:c r="H37" t="n">
+        <x:v>15.42</x:v>
+      </x:c>
+      <x:c r="I37" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="J37" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="K37" t="str">
+        <x:v>SUP-TECHXXL</x:v>
+      </x:c>
+      <x:c r="L37" t="str">
+        <x:v>TIN 101074 / S208L100</x:v>
+      </x:c>
+      <x:c r="M37" t="str">
+        <x:v>8 / I-type</x:v>
+      </x:c>
+      <x:c r="N37" t="str">
+        <x:v>132x44 mm</x:v>
+      </x:c>
+      <x:c r="O37" t="str">
+        <x:v>ST/Gummi</x:v>
+      </x:c>
+      <x:c r="P37" t="str">
+        <x:v>https://www.techxxl.nl/part-101074.html</x:v>
+      </x:c>
+      <x:c r="Q37" t="str">
+        <x:v>2026-08-22</x:v>
+      </x:c>
+      <x:c r="R37" t="str">
+        <x:v>Leveranciersprijs</x:v>
+      </x:c>
+      <x:c r="S37" t="str">
+        <x:v>IMG-TECHXXL-101074</x:v>
+      </x:c>
+      <x:c r="T37" t="str">
+        <x:v>https://www.techxxl.nl/img-101074-b.jpg</x:v>
+      </x:c>
+      <x:c r="U37" t="str">
+        <x:v>config/catalog-images/techxxl/caster-swivel-d100.jpg</x:v>
+      </x:c>
+      <x:c r="V37" t="str">
+        <x:v>Lokaal + Excel-preview</x:v>
+      </x:c>
+      <x:c r="W37" t="str">
+        <x:v>Vanafprijs per stuk netto; 90 kg draaglast volgens leverancier</x:v>
+      </x:c>
+      <x:c r="X37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Y37"/>
+    </x:row>
+    <x:row r="38" ht="64.5" customHeight="1">
+      <x:c r="A38" t="str">
+        <x:v>CAT-TECHXXL-101076</x:v>
+      </x:c>
+      <x:c r="B38" t="str">
+        <x:v>Component</x:v>
+      </x:c>
+      <x:c r="C38" t="str">
+        <x:v>techxxl_caster_swivel_brake_d100</x:v>
+      </x:c>
+      <x:c r="D38" t="str">
+        <x:v>Beslag</x:v>
+      </x:c>
+      <x:c r="E38" t="str">
+        <x:v>Profieltoebehoren</x:v>
+      </x:c>
+      <x:c r="F38" t="str">
+        <x:v>Zwenkwiel D100 dubbele rem</x:v>
+      </x:c>
+      <x:c r="G38" t="str">
+        <x:v>st</x:v>
+      </x:c>
+      <x:c r="H38" t="n">
+        <x:v>20.82</x:v>
+      </x:c>
+      <x:c r="I38" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="J38" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="K38" t="str">
+        <x:v>SUP-TECHXXL</x:v>
+      </x:c>
+      <x:c r="L38" t="str">
+        <x:v>TIN 101076 / S208LDF100</x:v>
+      </x:c>
+      <x:c r="M38" t="str">
+        <x:v>8 / I-type</x:v>
+      </x:c>
+      <x:c r="N38" t="str">
+        <x:v>132x44 mm</x:v>
+      </x:c>
+      <x:c r="O38" t="str">
+        <x:v>ST/Gummi</x:v>
+      </x:c>
+      <x:c r="P38" t="str">
+        <x:v>https://www.techxxl.nl/part-101076.html</x:v>
+      </x:c>
+      <x:c r="Q38" t="str">
+        <x:v>2026-08-22</x:v>
+      </x:c>
+      <x:c r="R38" t="str">
+        <x:v>Leveranciersprijs</x:v>
+      </x:c>
+      <x:c r="S38" t="str">
+        <x:v>IMG-TECHXXL-101076</x:v>
+      </x:c>
+      <x:c r="T38" t="str">
+        <x:v>https://www.techxxl.nl/img-101076-b.jpg</x:v>
+      </x:c>
+      <x:c r="U38" t="str">
+        <x:v>config/catalog-images/techxxl/caster-swivel-brake-d100.jpg</x:v>
+      </x:c>
+      <x:c r="V38" t="str">
+        <x:v>Lokaal + Excel-preview</x:v>
+      </x:c>
+      <x:c r="W38" t="str">
+        <x:v>Vanafprijs per stuk netto; 90 kg draaglast volgens leverancier</x:v>
+      </x:c>
+      <x:c r="X38" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Y38"/>
+    </x:row>
+    <x:row r="39" ht="64.5" customHeight="1">
+      <x:c r="A39" t="str">
+        <x:v>CAT-TECHXXL-100360</x:v>
+      </x:c>
+      <x:c r="B39" t="str">
+        <x:v>Component</x:v>
+      </x:c>
+      <x:c r="C39" t="str">
+        <x:v>techxxl_corner_bracket_set_8_40x40</x:v>
+      </x:c>
+      <x:c r="D39" t="str">
+        <x:v>Beslag</x:v>
+      </x:c>
+      <x:c r="E39" t="str">
+        <x:v>Profieltoebehoren</x:v>
+      </x:c>
+      <x:c r="F39" t="str">
+        <x:v>Hoekbeugelset 8 40x40 ZN</x:v>
+      </x:c>
+      <x:c r="G39" t="str">
+        <x:v>set</x:v>
+      </x:c>
+      <x:c r="H39" t="n">
+        <x:v>2.88</x:v>
+      </x:c>
+      <x:c r="I39" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="J39" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="K39" t="str">
+        <x:v>SUP-TECHXXL</x:v>
+      </x:c>
+      <x:c r="L39" t="str">
+        <x:v>TIN 100360 / S208WS40</x:v>
+      </x:c>
+      <x:c r="M39" t="str">
+        <x:v>8 / I-type / raster 40</x:v>
+      </x:c>
+      <x:c r="N39" t="str">
+        <x:v>40x40x40 mm</x:v>
+      </x:c>
+      <x:c r="O39" t="str">
+        <x:v>ZN gecoat / staal verzinkt</x:v>
+      </x:c>
+      <x:c r="P39" t="str">
+        <x:v>https://www.techxxl.nl/part-100360.html</x:v>
+      </x:c>
+      <x:c r="Q39" t="str">
+        <x:v>2026-08-22</x:v>
+      </x:c>
+      <x:c r="R39" t="str">
+        <x:v>Leveranciersprijs</x:v>
+      </x:c>
+      <x:c r="S39" t="str">
+        <x:v>IMG-TECHXXL-100360</x:v>
+      </x:c>
+      <x:c r="T39" t="str">
+        <x:v>https://www.techxxl.nl/img-100360-b.jpg</x:v>
+      </x:c>
+      <x:c r="U39" t="str">
+        <x:v>config/catalog-images/techxxl/corner-bracket-set-8-40x40.jpg</x:v>
+      </x:c>
+      <x:c r="V39" t="str">
+        <x:v>Lokaal + Excel-preview</x:v>
+      </x:c>
+      <x:c r="W39" t="str">
+        <x:v>Vanafprijs per complete set netto; serie 8 raster 40</x:v>
+      </x:c>
+      <x:c r="X39" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Y39"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:L1"/>
@@ -7289,10 +7810,10 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfce85b665e8f49a1"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00c56c90b5c84b4b"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc482b993aa064aca"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf2d6d51e4f564f48"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3051b3cde2524a01"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ed02a4d0ad74886"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7862,8 +8383,8 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f7f8670b3f34439"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98c04a15276a4b28"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c9c31d60f2e4f55"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c1f9b42428b4c67"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8264,7 +8785,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc33b0f6c5de64250"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf795d5cf2a9549a4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8720,8 +9241,8 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf796bf6721e540b9"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb7b2f174112438e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R891d7d7ddf78491b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5fdc38b2ae474cc9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9005,7 +9526,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref8d40433d274ecb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb969f160cd6f4e8a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9202,7 +9723,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf63f9d5d0f2409a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea5c9c488af241dd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9839,6 +10360,62 @@
       </x:c>
       <x:c r="R14" t="str">
         <x:v>n.v.t.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>materiaalwagen</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>Modulaire materiaal- en gereedschapswagen</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>profielconstructie</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>werktafel</x:v>
+      </x:c>
+      <x:c r="E15" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="F15" t="n">
+        <x:v>650</x:v>
+      </x:c>
+      <x:c r="G15" t="n">
+        <x:v>950</x:v>
+      </x:c>
+      <x:c r="H15" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I15" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K15" t="str">
+        <x:v>bottom</x:v>
+      </x:c>
+      <x:c r="L15" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="M15" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="N15" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="O15" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="P15" t="str">
+        <x:v>Voorlopig</x:v>
+      </x:c>
+      <x:c r="Q15" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="R15" t="str">
+        <x:v>OK</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9875,7 +10452,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R566d7c587963477a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3d46b446c324dd4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10597,9 +11174,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d0ba358eafc43eb"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d29210050df40b6"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf8ba93676ab14042"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb3184c49ff546cd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11513,6 +12090,154 @@
       <x:c r="L28"/>
       <x:c r="M28"/>
     </x:row>
+    <x:row r="29">
+      <x:c r="A29" t="str">
+        <x:v>techxxl_caster_fixed_d100</x:v>
+      </x:c>
+      <x:c r="B29" t="str">
+        <x:v>Zwenkwiel</x:v>
+      </x:c>
+      <x:c r="C29" t="str">
+        <x:v>TechXXL zwenkwiel vast D100</x:v>
+      </x:c>
+      <x:c r="D29" t="str">
+        <x:v>TIN 101068 / S208BRD100</x:v>
+      </x:c>
+      <x:c r="E29" t="str">
+        <x:v>D100 / groef 8 / I-type</x:v>
+      </x:c>
+      <x:c r="F29" t="str">
+        <x:v>132x40</x:v>
+      </x:c>
+      <x:c r="G29" t="str">
+        <x:v>Stalen behuizing; TPE-kogellagerwiel; achtergat 10,5; bouwhoogte 132</x:v>
+      </x:c>
+      <x:c r="H29" t="str">
+        <x:v>Vaste rijrichting onder mobiele profielconstructies</x:v>
+      </x:c>
+      <x:c r="I29" t="str">
+        <x:v>TechXXL productdata gecontroleerd 2026-08-22; draaglast 80 kg per wiel</x:v>
+      </x:c>
+      <x:c r="J29" t="str">
+        <x:v>Leveranciersdata</x:v>
+      </x:c>
+      <x:c r="K29" t="str">
+        <x:v>https://www.techxxl.nl/part-101068.html</x:v>
+      </x:c>
+      <x:c r="L29"/>
+      <x:c r="M29"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" t="str">
+        <x:v>techxxl_caster_swivel_d100</x:v>
+      </x:c>
+      <x:c r="B30" t="str">
+        <x:v>Zwenkwiel</x:v>
+      </x:c>
+      <x:c r="C30" t="str">
+        <x:v>TechXXL zwenkwiel D100</x:v>
+      </x:c>
+      <x:c r="D30" t="str">
+        <x:v>TIN 101074 / S208L100</x:v>
+      </x:c>
+      <x:c r="E30" t="str">
+        <x:v>D100 / groef 8 / I-type</x:v>
+      </x:c>
+      <x:c r="F30" t="str">
+        <x:v>132x44</x:v>
+      </x:c>
+      <x:c r="G30" t="str">
+        <x:v>Vrij zwenkend; stalen behuizing RAL zwart; achtergat 10,5; bouwhoogte 132</x:v>
+      </x:c>
+      <x:c r="H30" t="str">
+        <x:v>Vrij zwenkwiel onder mobiele profielconstructies</x:v>
+      </x:c>
+      <x:c r="I30" t="str">
+        <x:v>TechXXL productdata gecontroleerd 2026-08-22; draaglast 90 kg per wiel</x:v>
+      </x:c>
+      <x:c r="J30" t="str">
+        <x:v>Leveranciersdata</x:v>
+      </x:c>
+      <x:c r="K30" t="str">
+        <x:v>https://www.techxxl.nl/part-101074.html</x:v>
+      </x:c>
+      <x:c r="L30"/>
+      <x:c r="M30"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" t="str">
+        <x:v>techxxl_caster_swivel_brake_d100</x:v>
+      </x:c>
+      <x:c r="B31" t="str">
+        <x:v>Zwenkwiel</x:v>
+      </x:c>
+      <x:c r="C31" t="str">
+        <x:v>TechXXL zwenkwiel D100 dubbele rem</x:v>
+      </x:c>
+      <x:c r="D31" t="str">
+        <x:v>TIN 101076 / S208LDF100</x:v>
+      </x:c>
+      <x:c r="E31" t="str">
+        <x:v>D100 / groef 8 / I-type</x:v>
+      </x:c>
+      <x:c r="F31" t="str">
+        <x:v>132x44</x:v>
+      </x:c>
+      <x:c r="G31" t="str">
+        <x:v>Vrij zwenkend met dubbele vergrendeling; M10/kernboring of voetplaat</x:v>
+      </x:c>
+      <x:c r="H31" t="str">
+        <x:v>Geremd zwenkwiel onder mobiele profielconstructies</x:v>
+      </x:c>
+      <x:c r="I31" t="str">
+        <x:v>TechXXL productdata gecontroleerd 2026-08-22; draaglast 90 kg per wiel</x:v>
+      </x:c>
+      <x:c r="J31" t="str">
+        <x:v>Leveranciersdata</x:v>
+      </x:c>
+      <x:c r="K31" t="str">
+        <x:v>https://www.techxxl.nl/part-101076.html</x:v>
+      </x:c>
+      <x:c r="L31"/>
+      <x:c r="M31"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" t="str">
+        <x:v>techxxl_corner_bracket_set_8_40x40</x:v>
+      </x:c>
+      <x:c r="B32" t="str">
+        <x:v>Profielverbinder</x:v>
+      </x:c>
+      <x:c r="C32" t="str">
+        <x:v>TechXXL hoekbeugelset 8 40x40 ZN</x:v>
+      </x:c>
+      <x:c r="D32" t="str">
+        <x:v>TIN 100360 / S208WS40</x:v>
+      </x:c>
+      <x:c r="E32" t="str">
+        <x:v>Groef 8 / I-type / raster 40</x:v>
+      </x:c>
+      <x:c r="F32" t="str">
+        <x:v>40x40x40</x:v>
+      </x:c>
+      <x:c r="G32" t="str">
+        <x:v>Complete 90°-hoekset voor twee profielen; zinkdrukgietwerk en verzinkt staal</x:v>
+      </x:c>
+      <x:c r="H32" t="str">
+        <x:v>40x40-profielverbindingen van materiaalwagen en toekomstige serie-8 constructies</x:v>
+      </x:c>
+      <x:c r="I32" t="str">
+        <x:v>TechXXL productdata gecontroleerd 2026-08-22; compatibel met serie 8 raster 40</x:v>
+      </x:c>
+      <x:c r="J32" t="str">
+        <x:v>Leveranciersdata</x:v>
+      </x:c>
+      <x:c r="K32" t="str">
+        <x:v>https://www.techxxl.nl/part-100360.html</x:v>
+      </x:c>
+      <x:c r="L32"/>
+      <x:c r="M32"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:K1"/>
@@ -11531,7 +12256,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11b3dc921fc54a65"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a8aafe96a0f4029"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11943,9 +12668,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5624256a7ac84f14"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R672295afea8742db"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R677d58f8ee1849ba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1ba9d0f06894211"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12211,7 +12936,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa6d76b959a24dbf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5132da47080f4581"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13946,6 +14671,250 @@
         <x:v>MachineBaseEngine.cs</x:v>
       </x:c>
     </x:row>
+    <x:row r="42">
+      <x:c r="A42" t="str">
+        <x:v>PRD-MATW-001</x:v>
+      </x:c>
+      <x:c r="B42" t="str">
+        <x:v>materiaalwagen</x:v>
+      </x:c>
+      <x:c r="C42" t="str">
+        <x:v>Materiaal</x:v>
+      </x:c>
+      <x:c r="D42" t="str">
+        <x:v>volledig frame</x:v>
+      </x:c>
+      <x:c r="E42" t="str">
+        <x:v>Profielkeuze</x:v>
+      </x:c>
+      <x:c r="F42" t="str">
+        <x:v>Materiaal</x:v>
+      </x:c>
+      <x:c r="G42"/>
+      <x:c r="H42" t="str">
+        <x:v>alu_system_40x40</x:v>
+      </x:c>
+      <x:c r="I42"/>
+      <x:c r="J42"/>
+      <x:c r="K42" t="str">
+        <x:v>Alle staanders, omtrekliggers, middenliggers en duwbeugel uit 40x40</x:v>
+      </x:c>
+      <x:c r="L42" t="n">
+        <x:v>270</x:v>
+      </x:c>
+      <x:c r="M42" t="str">
+        <x:v>Goedgekeurd</x:v>
+      </x:c>
+      <x:c r="N42" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" t="str">
+        <x:v>PRD-MATW-002</x:v>
+      </x:c>
+      <x:c r="B43" t="str">
+        <x:v>materiaalwagen</x:v>
+      </x:c>
+      <x:c r="C43" t="str">
+        <x:v>Opbouw</x:v>
+      </x:c>
+      <x:c r="D43" t="str">
+        <x:v>iedere legbordlaag</x:v>
+      </x:c>
+      <x:c r="E43" t="str">
+        <x:v>Telmanifest</x:v>
+      </x:c>
+      <x:c r="F43" t="str">
+        <x:v>Materiaal</x:v>
+      </x:c>
+      <x:c r="G43"/>
+      <x:c r="H43" t="str">
+        <x:v>alu_system_40x40</x:v>
+      </x:c>
+      <x:c r="I43" t="str">
+        <x:v>4 + automatisch 1</x:v>
+      </x:c>
+      <x:c r="J43" t="str">
+        <x:v>profielen per laag</x:v>
+      </x:c>
+      <x:c r="K43" t="str">
+        <x:v>Vier omtrekliggers; exact één middenligger wanneer buitenbreedte &gt;=1000 mm</x:v>
+      </x:c>
+      <x:c r="L43" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="M43" t="str">
+        <x:v>Goedgekeurd</x:v>
+      </x:c>
+      <x:c r="N43" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" t="str">
+        <x:v>PRD-MATW-003</x:v>
+      </x:c>
+      <x:c r="B44" t="str">
+        <x:v>materiaalwagen</x:v>
+      </x:c>
+      <x:c r="C44" t="str">
+        <x:v>Beslag</x:v>
+      </x:c>
+      <x:c r="D44" t="str">
+        <x:v>wielopstelling vast/zwenkend</x:v>
+      </x:c>
+      <x:c r="E44" t="str">
+        <x:v>Componentkeuze</x:v>
+      </x:c>
+      <x:c r="F44" t="str">
+        <x:v>Component</x:v>
+      </x:c>
+      <x:c r="G44"/>
+      <x:c r="H44" t="str">
+        <x:v>techxxl_caster_fixed_d100;techxxl_caster_swivel_brake_d100</x:v>
+      </x:c>
+      <x:c r="I44" t="str">
+        <x:v>2+2</x:v>
+      </x:c>
+      <x:c r="J44" t="str">
+        <x:v>st</x:v>
+      </x:c>
+      <x:c r="K44" t="str">
+        <x:v>Standaard twee vaste D100-wielen en twee zwenkwielen met dubbele rem</x:v>
+      </x:c>
+      <x:c r="L44" t="n">
+        <x:v>290</x:v>
+      </x:c>
+      <x:c r="M44" t="str">
+        <x:v>Leveranciersdata</x:v>
+      </x:c>
+      <x:c r="N44" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" t="str">
+        <x:v>PRD-MATW-004</x:v>
+      </x:c>
+      <x:c r="B45" t="str">
+        <x:v>materiaalwagen</x:v>
+      </x:c>
+      <x:c r="C45" t="str">
+        <x:v>Beslag</x:v>
+      </x:c>
+      <x:c r="D45" t="str">
+        <x:v>wielopstelling vier zwenkend</x:v>
+      </x:c>
+      <x:c r="E45" t="str">
+        <x:v>Componentkeuze</x:v>
+      </x:c>
+      <x:c r="F45" t="str">
+        <x:v>Component</x:v>
+      </x:c>
+      <x:c r="G45"/>
+      <x:c r="H45" t="str">
+        <x:v>techxxl_caster_swivel_d100;techxxl_caster_swivel_brake_d100</x:v>
+      </x:c>
+      <x:c r="I45" t="str">
+        <x:v>2+2</x:v>
+      </x:c>
+      <x:c r="J45" t="str">
+        <x:v>st</x:v>
+      </x:c>
+      <x:c r="K45" t="str">
+        <x:v>Alternatief twee vrije zwenkwielen en twee zwenkwielen met dubbele rem</x:v>
+      </x:c>
+      <x:c r="L45" t="n">
+        <x:v>290</x:v>
+      </x:c>
+      <x:c r="M45" t="str">
+        <x:v>Leveranciersdata</x:v>
+      </x:c>
+      <x:c r="N45" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" t="str">
+        <x:v>PRD-MATW-005</x:v>
+      </x:c>
+      <x:c r="B46" t="str">
+        <x:v>materiaalwagen</x:v>
+      </x:c>
+      <x:c r="C46" t="str">
+        <x:v>Geometrie</x:v>
+      </x:c>
+      <x:c r="D46" t="str">
+        <x:v>alle profielkoppen</x:v>
+      </x:c>
+      <x:c r="E46" t="str">
+        <x:v>Eindbehandeling</x:v>
+      </x:c>
+      <x:c r="F46" t="str">
+        <x:v>Geen</x:v>
+      </x:c>
+      <x:c r="G46"/>
+      <x:c r="H46"/>
+      <x:c r="I46" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J46" t="str">
+        <x:v>eindkappen</x:v>
+      </x:c>
+      <x:c r="K46" t="str">
+        <x:v>Liggerkoppen zijn verbonden; staanderkoppen door bovenblad en onderzijden door wielplaten afgedekt</x:v>
+      </x:c>
+      <x:c r="L46" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="M46" t="str">
+        <x:v>Goedgekeurd</x:v>
+      </x:c>
+      <x:c r="N46" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" t="str">
+        <x:v>PRD-MATW-006</x:v>
+      </x:c>
+      <x:c r="B47" t="str">
+        <x:v>materiaalwagen</x:v>
+      </x:c>
+      <x:c r="C47" t="str">
+        <x:v>Parameters</x:v>
+      </x:c>
+      <x:c r="D47" t="str">
+        <x:v>klantconfigurator</x:v>
+      </x:c>
+      <x:c r="E47" t="str">
+        <x:v>Parametercontract</x:v>
+      </x:c>
+      <x:c r="F47" t="str">
+        <x:v>Geen</x:v>
+      </x:c>
+      <x:c r="G47"/>
+      <x:c r="H47"/>
+      <x:c r="I47" t="str">
+        <x:v>600..1800;450..1000;700..1200;2..4</x:v>
+      </x:c>
+      <x:c r="J47" t="str">
+        <x:v>mm/mm/mm/lagen</x:v>
+      </x:c>
+      <x:c r="K47" t="str">
+        <x:v>Breedte, diepte, bovenzijde bovenblad en aantal legbordlagen; duwbeugel links/rechts/geen en twee wielmodi</x:v>
+      </x:c>
+      <x:c r="L47" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="M47" t="str">
+        <x:v>Goedgekeurd</x:v>
+      </x:c>
+      <x:c r="N47" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:N1"/>
@@ -13968,9 +14937,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22fb10b15dbc4980"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64a394ea80e14a77"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a703a9102144545"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78abb105444d4f98"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add configurable 4080 sim rig
</commit_message>
<xml_diff>
--- a/config/product-master-data.xlsx
+++ b/config/product-master-data.xlsx
@@ -2,23 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start &amp; beheer" sheetId="1" r:id="Ra50e97c1de204c42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataclassificatie" sheetId="2" r:id="Re951e7dca2c74343"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Productcategorieen" sheetId="3" r:id="Rb3d5d4e39e054118"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Producten" sheetId="4" r:id="Rfd14274647234d8e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materialen" sheetId="5" r:id="R1bf7f1340e424510"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Componenten" sheetId="6" r:id="Re36db29000d34470"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verbindingsrecepten" sheetId="7" r:id="Rae12dc4356b04920"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categorie-regels" sheetId="8" r:id="Rd2ed7f3b240c4a02"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product-regels" sheetId="9" r:id="R6f33a88a2e8241b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controles" sheetId="10" r:id="R013c620e121a4477"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open punten" sheetId="11" r:id="R18cb38cdc51e4ec7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wijzigingslog" sheetId="12" r:id="Rab05ebbc6b3f4f6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keuzelijsten" sheetId="13" r:id="R85256d63d2634d6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prijs &amp; inkoop" sheetId="14" r:id="R30497c51c79a4e8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gereedschappen" sheetId="15" r:id="R28f5e05b8724467b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAM-parameters" sheetId="16" r:id="R37180d23bdba4cd0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leveranciers" sheetId="17" r:id="R140b9e008df44b05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start &amp; beheer" sheetId="1" r:id="R75e881928ec84dfe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataclassificatie" sheetId="2" r:id="Rbfac48e8bfa94197"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Productcategorieen" sheetId="3" r:id="Rd758d38b083e4aaa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Producten" sheetId="4" r:id="R76b8735006cc431b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materialen" sheetId="5" r:id="R0ac031ff3b6d4ab5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Componenten" sheetId="6" r:id="R21c831c03b7d4e8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verbindingsrecepten" sheetId="7" r:id="R07580a305763407b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categorie-regels" sheetId="8" r:id="R76d9959a14884b61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product-regels" sheetId="9" r:id="R7fb5597163494b9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controles" sheetId="10" r:id="R1e64fd0f468847bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open punten" sheetId="11" r:id="R7a59341cbb2e4d26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wijzigingslog" sheetId="12" r:id="Rcf83d3efaf004fe9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keuzelijsten" sheetId="13" r:id="Rcf4ba17f578147fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prijs &amp; inkoop" sheetId="14" r:id="Rb238f5349b8248c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gereedschappen" sheetId="15" r:id="R41d55b7da2904bf3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAM-parameters" sheetId="16" r:id="Rc498f550a20340c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leveranciers" sheetId="17" r:id="Ra0a77d0f1dfb42ff"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2001,7 +2001,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc22858ea96504fb2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0b371affc69646c8"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2028,7 +2028,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd40e28dad8784057"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R3fb1222b67b54a96"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2055,7 +2055,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rbffe0a3813a54952"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R14902af3eece47be"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2082,7 +2082,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5d91ad69ce5e487c"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R3daaee604fc54e37"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2109,7 +2109,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Recc33cf76d94412b"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rb02a486468884ed4"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2136,7 +2136,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rdc2e572798fc4af0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re6dd0dbe05204f36"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2163,7 +2163,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rb58ab18fafbb42ed"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra48c630787e44d3a"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2190,7 +2190,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R02e2518210d541da"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5b538cd22c1d4f6c"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2217,7 +2217,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R51bd7e0276d44eff"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R91e26510b29a423f"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2244,7 +2244,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R360eacab80964bb5"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R016bea7c91434f8c"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2271,7 +2271,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R03f3ad2969eb4547"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R886fd46ddffe4b9e"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2298,7 +2298,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R3a2f5886fadb4242"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra1a56de105634252"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2325,7 +2325,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re88917d3508b483b"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R63ce91b599994df7"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2352,7 +2352,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5fd18927e1004638"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd88b16928f85428f"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2379,7 +2379,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R8102612c9a424e57"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra8cc045f7b1e474a"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2406,7 +2406,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R649dfe48516843c2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R9f66c942ad2945f3"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2427,13 +2427,13 @@
     <xdr:ext cx="1066800" cy="742950"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="17" name="bec07b78-08c2-4b6b-92b7-9aea322e7438"/>
+        <xdr:cNvPr id="17" name="/xl/media/image17.jpg"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5b653ba660294b30"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R7fd183fdbe704cb7"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3067,7 +3067,7 @@
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="19" t="str">
-        <x:v>Productregels, materialen, gereedschappen, prijzen en verbindingen — beheerfundering v2.0</x:v>
+        <x:v>Productregels, materialen, gereedschappen, prijzen en verbindingen — beheerfundering v2.1</x:v>
       </x:c>
       <x:c r="B1" s="19"/>
       <x:c r="C1" s="19"/>
@@ -3134,7 +3134,7 @@
         <x:v>Producten</x:v>
       </x:c>
       <x:c r="B8" s="30" t="n">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D8" s="26" t="str">
         <x:v>Kritieke open/geblokkeerd</x:v>
@@ -3149,8 +3149,7 @@
         <x:v>Materialen</x:v>
       </x:c>
       <x:c r="B9" s="30" t="n">
-        <x:f>COUNTA('Materialen'!A6:A500)</x:f>
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="D9" s="26" t="str">
         <x:v>Geblokkeerde productregels</x:v>
@@ -3165,7 +3164,7 @@
         <x:v>Componenten</x:v>
       </x:c>
       <x:c r="B10" s="30" t="n">
-        <x:v>27</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="D10" s="28" t="str">
         <x:v>Productreferentiefouten</x:v>
@@ -3205,7 +3204,7 @@
         <x:v>Product-regels</x:v>
       </x:c>
       <x:c r="B13" s="31" t="n">
-        <x:v>42</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="D13" s="37" t="str">
         <x:v>1</x:v>
@@ -3228,7 +3227,7 @@
         <x:v>Prijs- en inkoopregels</x:v>
       </x:c>
       <x:c r="B14" s="63" t="n">
-        <x:v>34</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="D14" s="38" t="str">
         <x:v>2</x:v>
@@ -3971,6 +3970,126 @@
       </x:c>
       <x:c r="J20"/>
     </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="str">
+        <x:v>VAL-SIM-001</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>Sim-rig 40x80</x:v>
+      </x:c>
+      <x:c r="C21" t="str">
+        <x:v>Telcontract</x:v>
+      </x:c>
+      <x:c r="D21" t="str">
+        <x:v>2 langsliggers, 3 basisdwarsliggers, 2 staanders, 1 stuurbrug, 3 pedaalprofielen en 6 custom platen</x:v>
+      </x:c>
+      <x:c r="E21" t="str">
+        <x:v>Kritiek</x:v>
+      </x:c>
+      <x:c r="F21" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="G21" t="str">
+        <x:v>Profiel- of plaattelling wijkt af van manifest</x:v>
+      </x:c>
+      <x:c r="H21" t="str">
+        <x:v>Voorlopig</x:v>
+      </x:c>
+      <x:c r="I21" t="str">
+        <x:v>SimRigEngine + regressietest</x:v>
+      </x:c>
+      <x:c r="J21"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="str">
+        <x:v>VAL-SIM-002</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>Sim-rig 40x80</x:v>
+      </x:c>
+      <x:c r="C22" t="str">
+        <x:v>Profielorientatie</x:v>
+      </x:c>
+      <x:c r="D22" t="str">
+        <x:v>Basis en pedaalprofielen Y=40; stuurbrug Y=80; staanders X=40/Z=80</x:v>
+      </x:c>
+      <x:c r="E22" t="str">
+        <x:v>Kritiek</x:v>
+      </x:c>
+      <x:c r="F22" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="G22" t="str">
+        <x:v>40x80-profiel staat op de verkeerde doorsnede-as</x:v>
+      </x:c>
+      <x:c r="H22" t="str">
+        <x:v>Voorlopig</x:v>
+      </x:c>
+      <x:c r="I22" t="str">
+        <x:v>Assemblyplaatsingen + regressietest</x:v>
+      </x:c>
+      <x:c r="J22"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="str">
+        <x:v>VAL-SIM-003</x:v>
+      </x:c>
+      <x:c r="B23" t="str">
+        <x:v>Sim-rig 40x80</x:v>
+      </x:c>
+      <x:c r="C23" t="str">
+        <x:v>Custom plaatfunctie</x:v>
+      </x:c>
+      <x:c r="D23" t="str">
+        <x:v>Iedere plaatfamilie heeft expliciete contour en minimaal twee functionele gaten/sleuven</x:v>
+      </x:c>
+      <x:c r="E23" t="str">
+        <x:v>Kritiek</x:v>
+      </x:c>
+      <x:c r="F23" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="G23" t="str">
+        <x:v>Custom plaat is alleen visueel of niet produceerbaar</x:v>
+      </x:c>
+      <x:c r="H23" t="str">
+        <x:v>Voorlopig</x:v>
+      </x:c>
+      <x:c r="I23" t="str">
+        <x:v>CNC-sheetmodel + regressietest</x:v>
+      </x:c>
+      <x:c r="J23"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" t="str">
+        <x:v>VAL-SIM-004</x:v>
+      </x:c>
+      <x:c r="B24" t="str">
+        <x:v>Sim-rig 40x80</x:v>
+      </x:c>
+      <x:c r="C24" t="str">
+        <x:v>Proefbouw</x:v>
+      </x:c>
+      <x:c r="D24" t="str">
+        <x:v>CSL-DD-passing, pedaalplaatbelasting en exacte profielserie zijn fysiek gecontroleerd</x:v>
+      </x:c>
+      <x:c r="E24" t="str">
+        <x:v>Kritiek</x:v>
+      </x:c>
+      <x:c r="F24" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="G24" t="str">
+        <x:v>Product nog niet vrijgegeven voor verkoop/serieproductie</x:v>
+      </x:c>
+      <x:c r="H24" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="I24" t="str">
+        <x:v>Proefbouw en meetrapport</x:v>
+      </x:c>
+      <x:c r="J24"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:I1"/>
@@ -3992,7 +4111,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68c43d9ceac541f7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45f9de1c479645e1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4494,7 +4613,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4033d45709904dae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5170d38117164330"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5135,6 +5254,32 @@
         <x:v>Standaardcontract: 3 legborden, 22 profieldelen, 4 wielen, 0 losse eindkappen; productregressietest en 3D-assembly gebruiken dezelfde parameters.</x:v>
       </x:c>
     </x:row>
+    <x:row r="28">
+      <x:c r="A28" t="str">
+        <x:v>CHG-0023</x:v>
+      </x:c>
+      <x:c r="B28" t="str">
+        <x:v>2026-08-22</x:v>
+      </x:c>
+      <x:c r="C28" t="str">
+        <x:v>Dylan / Codex</x:v>
+      </x:c>
+      <x:c r="D28" t="str">
+        <x:v>2.1</x:v>
+      </x:c>
+      <x:c r="E28" t="str">
+        <x:v>Sim-racing-rig 40x80 met functionele custom platen</x:v>
+      </x:c>
+      <x:c r="F28" t="str">
+        <x:v>Configureerbare sim-rig toegevoegd. Zes adapterplaten zijn uit meerdere referentieaanzichten afgeleid en vereenvoudigd tot produceerbare contouren met uitsluitend montage-, draai- en instelfuncties.</x:v>
+      </x:c>
+      <x:c r="G28" t="str">
+        <x:v>sim_rig_4080;PRD-SIM-001..008;VAL-SIM-001..004;custom_simrig_*;sim-rig-4080-assembly-manifest.json</x:v>
+      </x:c>
+      <x:c r="H28" t="str">
+        <x:v>R1 blijft voorlopig: Aluxprofiel buitenmaten en Fanatec M6-interface zijn bronvast; exacte profielserie, pedaalbelasting en passing vereisen proefbouw.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
@@ -5142,7 +5287,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d0a5ab2fcaa43ba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63e5b6ba4ec447e8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5326,7 +5471,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re7dcdf68f7a3481a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2ba3fde144c4330"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7791,6 +7936,65 @@
       </x:c>
       <x:c r="Y39"/>
     </x:row>
+    <x:row r="40">
+      <x:c r="A40" t="str">
+        <x:v>CAT-CUSTOM-S235-10</x:v>
+      </x:c>
+      <x:c r="B40" t="str">
+        <x:v>Materiaal</x:v>
+      </x:c>
+      <x:c r="C40" t="str">
+        <x:v>steel_s235_10_custom</x:v>
+      </x:c>
+      <x:c r="D40" t="str">
+        <x:v>Materiaal</x:v>
+      </x:c>
+      <x:c r="E40" t="str">
+        <x:v>Staalplaat</x:v>
+      </x:c>
+      <x:c r="F40" t="str">
+        <x:v>S235JR staalplaat 10 mm custom</x:v>
+      </x:c>
+      <x:c r="G40" t="str">
+        <x:v>m2</x:v>
+      </x:c>
+      <x:c r="H40" t="n">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="I40" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="J40" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="K40"/>
+      <x:c r="L40"/>
+      <x:c r="M40"/>
+      <x:c r="N40" t="str">
+        <x:v>10x2000x1000 mm</x:v>
+      </x:c>
+      <x:c r="O40" t="str">
+        <x:v>S235JR</x:v>
+      </x:c>
+      <x:c r="P40"/>
+      <x:c r="Q40" t="str">
+        <x:v>2026-08-22</x:v>
+      </x:c>
+      <x:c r="R40" t="str">
+        <x:v>Schatting</x:v>
+      </x:c>
+      <x:c r="S40"/>
+      <x:c r="T40"/>
+      <x:c r="U40"/>
+      <x:c r="V40" t="str">
+        <x:v>Geen leveranciersbeeld</x:v>
+      </x:c>
+      <x:c r="W40" t="str">
+        <x:v>Voorlopige nettoprijs per m2; leverancier en snijproces nog selecteren</x:v>
+      </x:c>
+      <x:c r="X40"/>
+      <x:c r="Y40"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:L1"/>
@@ -7810,10 +8014,10 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc482b993aa064aca"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf2d6d51e4f564f48"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac6a242650dc44b7"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf2156822464d4cae"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ed02a4d0ad74886"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc8c40fffa5640cb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8383,8 +8587,8 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c9c31d60f2e4f55"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c1f9b42428b4c67"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfda57bdf29854b5f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7443341ec9444d84"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8785,7 +8989,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf795d5cf2a9549a4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f0d3fa0b0034386"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9241,8 +9445,8 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R891d7d7ddf78491b"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5fdc38b2ae474cc9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra822c0d8a85d463f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R88df06fbe350452b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9526,7 +9730,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb969f160cd6f4e8a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R903b733036834fe7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9723,7 +9927,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea5c9c488af241dd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38197745d4594c63"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10415,6 +10619,62 @@
         <x:v>OK</x:v>
       </x:c>
       <x:c r="R15" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>sim_rig_4080</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>Modulaire sim-racing-rig 40x80</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>profielconstructie</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>werktafel</x:v>
+      </x:c>
+      <x:c r="E16" t="n">
+        <x:v>680</x:v>
+      </x:c>
+      <x:c r="F16" t="n">
+        <x:v>1350</x:v>
+      </x:c>
+      <x:c r="G16" t="n">
+        <x:v>660</x:v>
+      </x:c>
+      <x:c r="H16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K16" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="L16" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="M16" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="N16" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="O16" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="P16" t="str">
+        <x:v>Voorlopig</x:v>
+      </x:c>
+      <x:c r="Q16" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="R16" t="str">
         <x:v>OK</x:v>
       </x:c>
     </x:row>
@@ -10452,7 +10712,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3d46b446c324dd4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R933994b1e01f4975"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11157,6 +11417,44 @@
         <x:v>https://www.techxxl.nl/part-100559.html</x:v>
       </x:c>
     </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="str">
+        <x:v>steel_s235_10_custom</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>Staal</x:v>
+      </x:c>
+      <x:c r="C21" t="str">
+        <x:v>Plaat</x:v>
+      </x:c>
+      <x:c r="D21" t="str">
+        <x:v>S235JR custom adapterplaat</x:v>
+      </x:c>
+      <x:c r="E21" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F21"/>
+      <x:c r="G21"/>
+      <x:c r="H21"/>
+      <x:c r="I21" t="str">
+        <x:v>2000x1000</x:v>
+      </x:c>
+      <x:c r="J21" t="str">
+        <x:v>CNC-gesneden montage- en verstelplaat</x:v>
+      </x:c>
+      <x:c r="K21" t="str">
+        <x:v>Frezen/boren of lasersnijden; ontbramen; zwart coaten optioneel</x:v>
+      </x:c>
+      <x:c r="L21" t="str">
+        <x:v>Functionele contour en gaten uit productmanifest; materiaalcertificaat bij productie bevestigen</x:v>
+      </x:c>
+      <x:c r="M21" t="str">
+        <x:v>Voorlopig</x:v>
+      </x:c>
+      <x:c r="N21" t="str">
+        <x:v>config/sim-rig-4080-assembly-manifest.json</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:N1"/>
@@ -11174,9 +11472,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d29210050df40b6"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb45a719748c34d93"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb3184c49ff546cd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R893afaaea5fb40e4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12238,6 +12536,117 @@
       <x:c r="L32"/>
       <x:c r="M32"/>
     </x:row>
+    <x:row r="33">
+      <x:c r="A33" t="str">
+        <x:v>custom_simrig_steering_side_plate_v1</x:v>
+      </x:c>
+      <x:c r="B33" t="str">
+        <x:v>Custom adapterplaat</x:v>
+      </x:c>
+      <x:c r="C33" t="str">
+        <x:v>Vereenvoudigde stuurzijplaat CSL DD</x:v>
+      </x:c>
+      <x:c r="D33" t="str">
+        <x:v>CUSTOM-SIM-STEER-V1</x:v>
+      </x:c>
+      <x:c r="E33" t="str">
+        <x:v>CSL DD zijmontage / 40x80</x:v>
+      </x:c>
+      <x:c r="F33" t="str">
+        <x:v>150x150x10</x:v>
+      </x:c>
+      <x:c r="G33" t="str">
+        <x:v>Vijfhoekige S235-plaat; twee profielslots; twee M6-gaten op 70 mm verticale steek</x:v>
+      </x:c>
+      <x:c r="H33" t="str">
+        <x:v>Verbindt stuurstaander, stuurbrug en Fanatec-zij-T-slot zonder decoratieve uitsparingen</x:v>
+      </x:c>
+      <x:c r="I33" t="str">
+        <x:v>R1 afgeleid uit zeven referentiebeelden; M6 inschroefdiepte 10 mm volgens Fanatec; proefpassing vereist</x:v>
+      </x:c>
+      <x:c r="J33" t="str">
+        <x:v>Referentiehypothese</x:v>
+      </x:c>
+      <x:c r="K33" t="str">
+        <x:v>https://assets.fanatec.com/image/upload/v1743547943/downloads-prod/pdfs/CSL-DD_Hard-Mount-Planner_01.pdf</x:v>
+      </x:c>
+      <x:c r="L33"/>
+      <x:c r="M33"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" t="str">
+        <x:v>custom_simrig_upright_t_plate_v1</x:v>
+      </x:c>
+      <x:c r="B34" t="str">
+        <x:v>Custom verbindingsplaat</x:v>
+      </x:c>
+      <x:c r="C34" t="str">
+        <x:v>Vereenvoudigde T-plaat stuurstaander</x:v>
+      </x:c>
+      <x:c r="D34" t="str">
+        <x:v>CUSTOM-SIM-T-V1</x:v>
+      </x:c>
+      <x:c r="E34" t="str">
+        <x:v>40x80 groefraster</x:v>
+      </x:c>
+      <x:c r="F34" t="str">
+        <x:v>180x150x10</x:v>
+      </x:c>
+      <x:c r="G34" t="str">
+        <x:v>T-contour; twee sleuven voor basisrail en één sleuf voor staander</x:v>
+      </x:c>
+      <x:c r="H34" t="str">
+        <x:v>Verstijft de stuurstaander op de basislangsligger zonder binnenhoeken</x:v>
+      </x:c>
+      <x:c r="I34" t="str">
+        <x:v>Functie bevestigd door referentiefoto en Aluxprofiel-producttekst; exacte serieverbinding nog proefbouwen</x:v>
+      </x:c>
+      <x:c r="J34" t="str">
+        <x:v>Referentiehypothese</x:v>
+      </x:c>
+      <x:c r="K34" t="str">
+        <x:v>https://www.aluxprofiel.nl/sim-racing-rig-4080-zilver-csl-dd-sidemount/a4118</x:v>
+      </x:c>
+      <x:c r="L34"/>
+      <x:c r="M34"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" t="str">
+        <x:v>custom_simrig_pedal_angle_plate_v1</x:v>
+      </x:c>
+      <x:c r="B35" t="str">
+        <x:v>Custom adapterplaat</x:v>
+      </x:c>
+      <x:c r="C35" t="str">
+        <x:v>Vereenvoudigde pedaalhoekplaat</x:v>
+      </x:c>
+      <x:c r="D35" t="str">
+        <x:v>CUSTOM-SIM-PEDAL-V1</x:v>
+      </x:c>
+      <x:c r="E35" t="str">
+        <x:v>40x80 pedaalplatform</x:v>
+      </x:c>
+      <x:c r="F35" t="str">
+        <x:v>300x170x10</x:v>
+      </x:c>
+      <x:c r="G35" t="str">
+        <x:v>Trapeziumcontour; M8-draaipunt; instelsleuf; M8-dekbevestiging</x:v>
+      </x:c>
+      <x:c r="H35" t="str">
+        <x:v>Verbindt en verstelt drie pedaalprofielen ten opzichte van de basis</x:v>
+      </x:c>
+      <x:c r="I35" t="str">
+        <x:v>R1 functionele afleiding; decoratieve gewichtsuitsparingen bewust weggelaten; proefbelasting vereist</x:v>
+      </x:c>
+      <x:c r="J35" t="str">
+        <x:v>Referentiehypothese</x:v>
+      </x:c>
+      <x:c r="K35" t="str">
+        <x:v>config/sim-rig-4080-assembly-manifest.json</x:v>
+      </x:c>
+      <x:c r="L35"/>
+      <x:c r="M35"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:K1"/>
@@ -12256,7 +12665,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a8aafe96a0f4029"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd087e2fd02254188"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12668,9 +13077,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R672295afea8742db"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07a2b214cdc7459c"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1ba9d0f06894211"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52f7070f711b4d30"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12936,7 +13345,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5132da47080f4581"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26f7ee9973614030"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14915,6 +15324,330 @@
         <x:v>Ja</x:v>
       </x:c>
     </x:row>
+    <x:row r="48">
+      <x:c r="A48" t="str">
+        <x:v>PRD-SIM-001</x:v>
+      </x:c>
+      <x:c r="B48" t="str">
+        <x:v>sim_rig_4080</x:v>
+      </x:c>
+      <x:c r="C48" t="str">
+        <x:v>Materiaal</x:v>
+      </x:c>
+      <x:c r="D48" t="str">
+        <x:v>alle profielen</x:v>
+      </x:c>
+      <x:c r="E48" t="str">
+        <x:v>Profielkeuze</x:v>
+      </x:c>
+      <x:c r="F48" t="str">
+        <x:v>Materiaal</x:v>
+      </x:c>
+      <x:c r="G48"/>
+      <x:c r="H48" t="str">
+        <x:v>alu_system_80x40</x:v>
+      </x:c>
+      <x:c r="I48"/>
+      <x:c r="J48"/>
+      <x:c r="K48" t="str">
+        <x:v>Alle primaire delen gebruiken 40x80; iedere rol bewaart een numerieke vlak/staand-orientatie</x:v>
+      </x:c>
+      <x:c r="L48" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="M48" t="str">
+        <x:v>Referentiehypothese</x:v>
+      </x:c>
+      <x:c r="N48" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" t="str">
+        <x:v>PRD-SIM-002</x:v>
+      </x:c>
+      <x:c r="B49" t="str">
+        <x:v>sim_rig_4080</x:v>
+      </x:c>
+      <x:c r="C49" t="str">
+        <x:v>Opbouw</x:v>
+      </x:c>
+      <x:c r="D49" t="str">
+        <x:v>basislaag</x:v>
+      </x:c>
+      <x:c r="E49" t="str">
+        <x:v>Telmanifest</x:v>
+      </x:c>
+      <x:c r="F49" t="str">
+        <x:v>Materiaal</x:v>
+      </x:c>
+      <x:c r="G49"/>
+      <x:c r="H49" t="str">
+        <x:v>alu_system_80x40</x:v>
+      </x:c>
+      <x:c r="I49" t="str">
+        <x:v>2+3</x:v>
+      </x:c>
+      <x:c r="J49" t="str">
+        <x:v>profielen</x:v>
+      </x:c>
+      <x:c r="K49" t="str">
+        <x:v>Twee vlakke langsliggers en exact drie vlakke dwarsliggers</x:v>
+      </x:c>
+      <x:c r="L49" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="M49" t="str">
+        <x:v>Referentiehypothese</x:v>
+      </x:c>
+      <x:c r="N49" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" t="str">
+        <x:v>PRD-SIM-003</x:v>
+      </x:c>
+      <x:c r="B50" t="str">
+        <x:v>sim_rig_4080</x:v>
+      </x:c>
+      <x:c r="C50" t="str">
+        <x:v>Opbouw</x:v>
+      </x:c>
+      <x:c r="D50" t="str">
+        <x:v>stuur en pedalen</x:v>
+      </x:c>
+      <x:c r="E50" t="str">
+        <x:v>Telmanifest</x:v>
+      </x:c>
+      <x:c r="F50" t="str">
+        <x:v>Materiaal</x:v>
+      </x:c>
+      <x:c r="G50"/>
+      <x:c r="H50" t="str">
+        <x:v>alu_system_80x40</x:v>
+      </x:c>
+      <x:c r="I50" t="str">
+        <x:v>2+1+3</x:v>
+      </x:c>
+      <x:c r="J50" t="str">
+        <x:v>profielen</x:v>
+      </x:c>
+      <x:c r="K50" t="str">
+        <x:v>Twee stuurstaanders, één staande stuurbrug en drie vlakke pedaalprofielen</x:v>
+      </x:c>
+      <x:c r="L50" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="M50" t="str">
+        <x:v>Referentiehypothese</x:v>
+      </x:c>
+      <x:c r="N50" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" t="str">
+        <x:v>PRD-SIM-004</x:v>
+      </x:c>
+      <x:c r="B51" t="str">
+        <x:v>sim_rig_4080</x:v>
+      </x:c>
+      <x:c r="C51" t="str">
+        <x:v>Custom platen</x:v>
+      </x:c>
+      <x:c r="D51" t="str">
+        <x:v>alle adapterfuncties</x:v>
+      </x:c>
+      <x:c r="E51" t="str">
+        <x:v>Componentkeuze</x:v>
+      </x:c>
+      <x:c r="F51" t="str">
+        <x:v>Component</x:v>
+      </x:c>
+      <x:c r="G51"/>
+      <x:c r="H51" t="str">
+        <x:v>custom_simrig_steering_side_plate_v1;custom_simrig_upright_t_plate_v1;custom_simrig_pedal_angle_plate_v1</x:v>
+      </x:c>
+      <x:c r="I51" t="str">
+        <x:v>2+2+2</x:v>
+      </x:c>
+      <x:c r="J51" t="str">
+        <x:v>st</x:v>
+      </x:c>
+      <x:c r="K51" t="str">
+        <x:v>Zes CNC-platen; gekoppelde vlakken, gaten en instelbereik zijn verplicht</x:v>
+      </x:c>
+      <x:c r="L51" t="n">
+        <x:v>320</x:v>
+      </x:c>
+      <x:c r="M51" t="str">
+        <x:v>Referentiehypothese</x:v>
+      </x:c>
+      <x:c r="N51" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" t="str">
+        <x:v>PRD-SIM-005</x:v>
+      </x:c>
+      <x:c r="B52" t="str">
+        <x:v>sim_rig_4080</x:v>
+      </x:c>
+      <x:c r="C52" t="str">
+        <x:v>Custom platen</x:v>
+      </x:c>
+      <x:c r="D52" t="str">
+        <x:v>contourvereenvoudiging</x:v>
+      </x:c>
+      <x:c r="E52" t="str">
+        <x:v>Ontwerpregel</x:v>
+      </x:c>
+      <x:c r="F52" t="str">
+        <x:v>Geen</x:v>
+      </x:c>
+      <x:c r="G52"/>
+      <x:c r="H52"/>
+      <x:c r="I52" t="str">
+        <x:v>functioneel minimum</x:v>
+      </x:c>
+      <x:c r="J52"/>
+      <x:c r="K52" t="str">
+        <x:v>Behoud belastingpad, interfaces en benodigde gaten/sleuven; verwijder decoratieve uitsparingen</x:v>
+      </x:c>
+      <x:c r="L52" t="n">
+        <x:v>320</x:v>
+      </x:c>
+      <x:c r="M52" t="str">
+        <x:v>Goedgekeurd</x:v>
+      </x:c>
+      <x:c r="N52" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" t="str">
+        <x:v>PRD-SIM-006</x:v>
+      </x:c>
+      <x:c r="B53" t="str">
+        <x:v>sim_rig_4080</x:v>
+      </x:c>
+      <x:c r="C53" t="str">
+        <x:v>Stuurwielbasis</x:v>
+      </x:c>
+      <x:c r="D53" t="str">
+        <x:v>CSL DD zijmontage</x:v>
+      </x:c>
+      <x:c r="E53" t="str">
+        <x:v>Gatenpatroon</x:v>
+      </x:c>
+      <x:c r="F53" t="str">
+        <x:v>Component</x:v>
+      </x:c>
+      <x:c r="G53"/>
+      <x:c r="H53" t="str">
+        <x:v>custom_simrig_steering_side_plate_v1</x:v>
+      </x:c>
+      <x:c r="I53" t="str">
+        <x:v>M6; plaat 10; inschroef 10</x:v>
+      </x:c>
+      <x:c r="J53" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="K53" t="str">
+        <x:v>M6x20 bij 10 mm plaat; voorzijdegaten van wheelbase nooit als hard-mount gebruiken</x:v>
+      </x:c>
+      <x:c r="L53" t="n">
+        <x:v>330</x:v>
+      </x:c>
+      <x:c r="M53" t="str">
+        <x:v>Leveranciersdata</x:v>
+      </x:c>
+      <x:c r="N53" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" t="str">
+        <x:v>PRD-SIM-007</x:v>
+      </x:c>
+      <x:c r="B54" t="str">
+        <x:v>sim_rig_4080</x:v>
+      </x:c>
+      <x:c r="C54" t="str">
+        <x:v>Geometrie</x:v>
+      </x:c>
+      <x:c r="D54" t="str">
+        <x:v>blootgestelde profielkoppen</x:v>
+      </x:c>
+      <x:c r="E54" t="str">
+        <x:v>Eindbehandeling</x:v>
+      </x:c>
+      <x:c r="F54" t="str">
+        <x:v>Geen</x:v>
+      </x:c>
+      <x:c r="G54"/>
+      <x:c r="H54"/>
+      <x:c r="I54" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="J54" t="str">
+        <x:v>eindkappen</x:v>
+      </x:c>
+      <x:c r="K54" t="str">
+        <x:v>Vier basisuiteinden en twee bovenzijden stuurstaanders krijgen seriepassende 40x80-kappen</x:v>
+      </x:c>
+      <x:c r="L54" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="M54" t="str">
+        <x:v>Referentiehypothese</x:v>
+      </x:c>
+      <x:c r="N54" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" t="str">
+        <x:v>PRD-SIM-008</x:v>
+      </x:c>
+      <x:c r="B55" t="str">
+        <x:v>sim_rig_4080</x:v>
+      </x:c>
+      <x:c r="C55" t="str">
+        <x:v>Parameters</x:v>
+      </x:c>
+      <x:c r="D55" t="str">
+        <x:v>klantconfigurator</x:v>
+      </x:c>
+      <x:c r="E55" t="str">
+        <x:v>Parametercontract</x:v>
+      </x:c>
+      <x:c r="F55" t="str">
+        <x:v>Geen</x:v>
+      </x:c>
+      <x:c r="G55"/>
+      <x:c r="H55"/>
+      <x:c r="I55" t="str">
+        <x:v>600..800;1200..1800;550..850;0..25</x:v>
+      </x:c>
+      <x:c r="J55" t="str">
+        <x:v>mm/mm/mm/graden</x:v>
+      </x:c>
+      <x:c r="K55" t="str">
+        <x:v>Buitenbreedte, lengte, stuurhoogte, brugpositie, pedaalpositie, pedaalhoek en CSL-DD/blanco plaat</x:v>
+      </x:c>
+      <x:c r="L55" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="M55" t="str">
+        <x:v>Goedgekeurd</x:v>
+      </x:c>
+      <x:c r="N55" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:N1"/>
@@ -14937,9 +15670,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64a394ea80e14a77"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R237f8069b7cb4d5a"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78abb105444d4f98"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9db00119319e46b9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(masterdata): manage product card images
</commit_message>
<xml_diff>
--- a/config/product-master-data.xlsx
+++ b/config/product-master-data.xlsx
@@ -2,24 +2,24 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start &amp; beheer" sheetId="1" r:id="R0a4656c423cd4a2c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataclassificatie" sheetId="2" r:id="Rf5f6152dca7a4587"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Productcategorieen" sheetId="3" r:id="R32e58143ced4432a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Producten" sheetId="4" r:id="R66c7160356cb4ed4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materialen" sheetId="5" r:id="R448b4959d09840fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Componenten" sheetId="6" r:id="R054e703bea2f4f08"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verbindingsrecepten" sheetId="7" r:id="R9217e4bb36fd4afa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categorie-regels" sheetId="8" r:id="Rd5a7b525fabd4921"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product-regels" sheetId="9" r:id="Rbde1a951c7fd4dfd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controles" sheetId="10" r:id="R8335b7fc2a1040e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open punten" sheetId="11" r:id="R472db39827574ff9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wijzigingslog" sheetId="12" r:id="R140a8db6b7b045b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keuzelijsten" sheetId="13" r:id="Rc309a5c91fd947b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prijs &amp; inkoop" sheetId="14" r:id="R77964d1e69914a0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gereedschappen" sheetId="15" r:id="R5489a5470e8e4d26"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAM-parameters" sheetId="16" r:id="R2d814d1dfb6a4a2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leveranciers" sheetId="17" r:id="R895d231238e44562"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product-invoer" sheetId="19" r:id="R09668c2df7124264"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start &amp; beheer" sheetId="1" r:id="Re86206570f384bc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataclassificatie" sheetId="2" r:id="Rbac3270d41714930"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Productcategorieen" sheetId="3" r:id="R9ec34fc581dc4417"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Producten" sheetId="4" r:id="Rdea86fa6041e4366"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materialen" sheetId="5" r:id="R4babee1df933448b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Componenten" sheetId="6" r:id="R1cf842e924bf4e99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verbindingsrecepten" sheetId="7" r:id="Rd7f6aa9fb1f6426e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categorie-regels" sheetId="8" r:id="Rde659b58769c42aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product-regels" sheetId="9" r:id="Re00fac309c964762"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controles" sheetId="10" r:id="R980c879d80a4465d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open punten" sheetId="11" r:id="R693046ef7dd14c27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wijzigingslog" sheetId="12" r:id="Rc3a8a232210f4371"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keuzelijsten" sheetId="13" r:id="Ra46d2c4841be46f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prijs &amp; inkoop" sheetId="14" r:id="R7941502811ea4f3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gereedschappen" sheetId="15" r:id="R23e13f5962c94a7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAM-parameters" sheetId="16" r:id="R494c13b72c004572"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leveranciers" sheetId="17" r:id="R4fb6efa6b6564310"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product-invoer" sheetId="19" r:id="R7433ab9c9c964f83"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2871,7 +2871,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rdcb7195cf5cd4f9e"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R7bc8b0566c504e1c"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2898,7 +2898,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd65297ed52314c39"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc920915e595a4f34"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2925,7 +2925,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re8894a9ce5b14194"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re8be620382704114"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2952,7 +2952,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R4019c455d6604a47"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R949f4d99ceff4f8c"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2979,7 +2979,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R616df11f523f4ed6"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R3ac59f17d9aa41e3"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3006,7 +3006,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Raf16376f32284267"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rab61268e3a5d4e5b"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3033,7 +3033,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R2b70f0f3ac054fcf"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R3e0097d79eb34ac8"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3060,7 +3060,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R76879776ba2849f8"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R42fdb9a42e3c48f9"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3087,7 +3087,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R89db3b64ec064eb8"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra16b12ba44664210"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3114,7 +3114,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rdced4e80b5c04c56"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rf8da65620165458e"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3141,7 +3141,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R26b1b243bb3d4e09"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R1232f9d59f054f18"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3168,7 +3168,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd85ca4befa554d22"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R30d91e7945424737"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3195,7 +3195,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R2f5528b1d487491e"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5531f8ae670b429a"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3222,7 +3222,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R3850e0f85fdc48ea"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R26c5577ea29a4939"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3249,7 +3249,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Raf61e0a254b64e43"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R872699ea4cb343d0"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3276,7 +3276,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R55f3737091884b7a"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R3ef99c07934c4406"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3303,7 +3303,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R514af3403f6c4f80"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R17062da2166b41a9"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3330,7 +3330,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R1a54881b7faa4154"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra9497021aacb4bf1"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3357,7 +3357,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra6b7b03411474078"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R470be335151d4af6"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3384,7 +3384,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R6cc8cffc64644f9f"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R749d79d74ccc42b3"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3411,7 +3411,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra81309fd28624ffc"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R1bb4263d147f4261"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3438,7 +3438,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R1c344d4623524067"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra8c51fe83c984228"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3465,7 +3465,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R9496718604404bbd"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R909072e33d2a4cc2"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3492,7 +3492,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0855ba5c125d4e03"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R83c4c0cbf84145ad"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3519,7 +3519,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R001626fa43b34c00"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R62951a618655401c"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3546,7 +3546,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rf4c1cf38c7e34fc3"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R8ebc8db871f1417b"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3573,7 +3573,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R8b97d626efd44e19"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R83f8b0f5df424d27"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3600,7 +3600,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R7b77afaea0bc42d4"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R777739a73d3e4e41"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3627,7 +3627,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rdb1ec0a5b28c4545"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0590215860bc43b0"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3654,7 +3654,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R3adead4d6a1a4530"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R9dcf4e0235d0419c"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3681,7 +3681,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R373c2e42f64046db"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R4792ca4570c24a9f"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3708,7 +3708,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R6998a442c33c4141"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5a74e1d29c394043"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3735,7 +3735,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rb9016cb380364f4a"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R380e71d0fc9447a8"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3762,7 +3762,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R44cc46d9755a491f"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R6427786783c94959"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3789,7 +3789,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rbd834dda08dc483b"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R77e47ba8435e4820"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3816,7 +3816,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc027f2586a434cbf"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R4b1bb3af71fd4b6c"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3873,7 +3873,7 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="69" name="ChangeLogTable" displayName="ChangeLogTable" ref="A4:H67" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="69" name="ChangeLogTable" displayName="ChangeLogTable" ref="A4:H68" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Column1"/>
     <x:tableColumn id="2" name="Column2"/>
@@ -4087,8 +4087,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="50" name="ProductsTable" displayName="ProductsTable" ref="A5:S18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="19">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="70" name="ProductsTable" displayName="ProductsTable" ref="A5:X18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="24">
     <x:tableColumn id="1" name="Product-ID"/>
     <x:tableColumn id="2" name="Naam"/>
     <x:tableColumn id="3" name="Categorie-ID"/>
@@ -4108,6 +4108,11 @@
     <x:tableColumn id="17" name="Categoriecontrole"/>
     <x:tableColumn id="18" name="Overervingscontrole"/>
     <x:tableColumn id="19" name="Aantal stuks default"/>
+    <x:tableColumn id="20" name="Kaartafbeelding-pad"/>
+    <x:tableColumn id="21" name="Kaartafbeelding-alt"/>
+    <x:tableColumn id="22" name="Kaartafbeelding-bron"/>
+    <x:tableColumn id="23" name="Kaartafbeelding-revisie"/>
+    <x:tableColumn id="24" name="Kaartafbeelding-status"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -5671,7 +5676,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08500f21f38c4137"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2754e938dc3e4a60"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6289,7 +6294,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab3b8a112a63452e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbddfd5d0df774dee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7974,6 +7979,32 @@
         <x:v>Klantweergave: Okoumé 40 mm. Technische identificatie en inkoopkoppeling blijven ongewijzigd.</x:v>
       </x:c>
     </x:row>
+    <x:row r="68">
+      <x:c r="A68" t="str">
+        <x:v>CHG-063</x:v>
+      </x:c>
+      <x:c r="B68" s="64" t="n">
+        <x:v>46262</x:v>
+      </x:c>
+      <x:c r="C68" t="str">
+        <x:v>Dylan / Codex</x:v>
+      </x:c>
+      <x:c r="D68" t="str">
+        <x:v>5.5</x:v>
+      </x:c>
+      <x:c r="E68" t="str">
+        <x:v>Beheerde productkaartafbeeldingen</x:v>
+      </x:c>
+      <x:c r="F68" t="str">
+        <x:v>Producten krijgen beheerde kaartafbeeldingsvelden voor pad, alt-tekst, bron, revisie en beschikbaarheidsstatus. De backend levert deze velden aan de portal; ontbrekende renders blijven expliciet zichtbaar. Validator controleert bestandstype en extensie.</x:v>
+      </x:c>
+      <x:c r="G68" t="str">
+        <x:v>productCardImageContract;Kaartafbeelding-pad;Kaartafbeelding-alt;Kaartafbeelding-bron;Kaartafbeelding-revisie;Kaartafbeelding-status;cabinet;vakjeskast;werkbankkast;werktafel;werktafel_lex;machinebasis</x:v>
+      </x:c>
+      <x:c r="H68" t="str">
+        <x:v>Kaartafbeeldingen zijn presentatie en geen technische of productiebron. Bestandsformaat en extensie moeten overeenkomen.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
@@ -7981,7 +8012,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R473deedfccc94749"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R014036c9939a4ea9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8165,7 +8196,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39bfbeefd32b4635"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a1f270748e14e6e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13007,10 +13038,10 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra7de796e5c734139"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3391b5d3310a4a7e"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74076ff0b9454528"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc83a1a78a80d445c"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d332888475f43da"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2cfb33500214076"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13580,8 +13611,8 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1cc0e3f2c19c4018"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57ec61d42b054180"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7b512481fb2404c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7cfe6592bd6c4e45"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14359,7 +14390,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6be4cc69702d4a25"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa259c8a734d4cb9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15133,8 +15164,8 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2f330da9d204527"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8624bc5a3927479e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20916be63ffb4107"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf416b34d5bc4c46"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19764,7 +19795,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd16da8b894054fd9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9c00185bd0b4b36"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20048,7 +20079,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c0a49ba5fc647c8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53ba34e739b84dd3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20245,7 +20276,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93660c60f8224c1f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf8597285ded048fb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20273,6 +20304,11 @@
     <x:col min="17" max="17" width="20" hidden="0" customWidth="1"/>
     <x:col min="18" max="18" width="22" hidden="0" customWidth="1"/>
     <x:col min="19" max="19" width="21" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="30" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="34" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="48" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="16" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="16" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -20377,6 +20413,21 @@
       <x:c r="S5" t="str">
         <x:v>Aantal stuks default</x:v>
       </x:c>
+      <x:c r="T5" s="6" t="str">
+        <x:v>Kaartafbeelding-pad</x:v>
+      </x:c>
+      <x:c r="U5" s="6" t="str">
+        <x:v>Kaartafbeelding-alt</x:v>
+      </x:c>
+      <x:c r="V5" s="6" t="str">
+        <x:v>Kaartafbeelding-bron</x:v>
+      </x:c>
+      <x:c r="W5" s="6" t="str">
+        <x:v>Kaartafbeelding-revisie</x:v>
+      </x:c>
+      <x:c r="X5" s="6" t="str">
+        <x:v>Kaartafbeelding-status</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="13" t="str">
@@ -20436,6 +20487,21 @@
       <x:c r="S6" t="n">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="T6" s="6" t="str">
+        <x:v>/images/product-cabinet.png</x:v>
+      </x:c>
+      <x:c r="U6" s="6" t="str">
+        <x:v>3/4-render van de cabinet / kast</x:v>
+      </x:c>
+      <x:c r="V6" s="6" t="str">
+        <x:v>Beheerde bestaande portalrender</x:v>
+      </x:c>
+      <x:c r="W6" s="6" t="str">
+        <x:v>2026-08-28</x:v>
+      </x:c>
+      <x:c r="X6" t="str">
+        <x:v>Beschikbaar</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="14" t="str">
@@ -20497,6 +20563,21 @@
       <x:c r="S7" t="n">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="T7" s="6" t="str">
+        <x:v>/images/product-cubby.png</x:v>
+      </x:c>
+      <x:c r="U7" s="6" t="str">
+        <x:v>3/4-render van de vakjeskast</x:v>
+      </x:c>
+      <x:c r="V7" s="6" t="str">
+        <x:v>Beheerde bestaande portalrender</x:v>
+      </x:c>
+      <x:c r="W7" s="6" t="str">
+        <x:v>2026-08-28</x:v>
+      </x:c>
+      <x:c r="X7" t="str">
+        <x:v>Beschikbaar</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="14" t="str">
@@ -20558,6 +20639,21 @@
       <x:c r="S8" t="n">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="T8" s="6" t="str">
+        <x:v>/images/product-workbench-cabinet.jpg</x:v>
+      </x:c>
+      <x:c r="U8" s="6" t="str">
+        <x:v>3/4-render van de werkbank met kastonderbouw</x:v>
+      </x:c>
+      <x:c r="V8" s="6" t="str">
+        <x:v>PortalData-projectexport Werkbankkast 2400x600x900, 2026-08-18</x:v>
+      </x:c>
+      <x:c r="W8" s="6" t="str">
+        <x:v>2026-08-28</x:v>
+      </x:c>
+      <x:c r="X8" t="str">
+        <x:v>Beschikbaar</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="14" t="str">
@@ -20617,6 +20713,21 @@
       <x:c r="S9" t="n">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="T9" s="6" t="str">
+        <x:v>/images/product-workbench.png</x:v>
+      </x:c>
+      <x:c r="U9" s="6" t="str">
+        <x:v>3/4-render van de werktafel</x:v>
+      </x:c>
+      <x:c r="V9" s="6" t="str">
+        <x:v>Beheerde bestaande portalrender</x:v>
+      </x:c>
+      <x:c r="W9" s="6" t="str">
+        <x:v>2026-08-28</x:v>
+      </x:c>
+      <x:c r="X9" t="str">
+        <x:v>Beschikbaar</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="14" t="str">
@@ -20678,6 +20789,21 @@
       <x:c r="S10" t="n">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="T10" s="6" t="str">
+        <x:v>/images/product-lex-workbench.jpg</x:v>
+      </x:c>
+      <x:c r="U10" s="6" t="str">
+        <x:v>3/4-render van het LEX-workstation</x:v>
+      </x:c>
+      <x:c r="V10" s="6" t="str">
+        <x:v>PortalData-projectexport WORKSTATION 1650x1000x848, 2026-08-26</x:v>
+      </x:c>
+      <x:c r="W10" s="6" t="str">
+        <x:v>2026-08-28</x:v>
+      </x:c>
+      <x:c r="X10" t="str">
+        <x:v>Beschikbaar</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="15" t="str">
@@ -20739,6 +20865,13 @@
       <x:c r="S11" t="n">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="T11" s="6"/>
+      <x:c r="U11" s="6"/>
+      <x:c r="V11" s="6"/>
+      <x:c r="W11" s="6"/>
+      <x:c r="X11" t="str">
+        <x:v>Ontbreekt</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="str">
@@ -20798,6 +20931,13 @@
       <x:c r="S12" t="n">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="T12" s="6"/>
+      <x:c r="U12" s="6"/>
+      <x:c r="V12" s="6"/>
+      <x:c r="W12" s="6"/>
+      <x:c r="X12" t="str">
+        <x:v>Ontbreekt</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="str">
@@ -20857,6 +20997,13 @@
       <x:c r="S13" t="n">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="T13" s="6"/>
+      <x:c r="U13" s="6"/>
+      <x:c r="V13" s="6"/>
+      <x:c r="W13" s="6"/>
+      <x:c r="X13" t="str">
+        <x:v>Ontbreekt</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="str">
@@ -20914,6 +21061,21 @@
       <x:c r="S14" t="n">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="T14" s="6" t="str">
+        <x:v>/images/product-machinebase.png</x:v>
+      </x:c>
+      <x:c r="U14" s="6" t="str">
+        <x:v>3/4-render van de parametrische machinebasis</x:v>
+      </x:c>
+      <x:c r="V14" s="6" t="str">
+        <x:v>PortalData-projectexport MACHINEBASIS 2000x800x2000, 2026-08-21</x:v>
+      </x:c>
+      <x:c r="W14" s="6" t="str">
+        <x:v>2026-08-28</x:v>
+      </x:c>
+      <x:c r="X14" t="str">
+        <x:v>Beschikbaar</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" t="str">
@@ -20973,6 +21135,13 @@
       <x:c r="S15" t="n">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="T15" s="6"/>
+      <x:c r="U15" s="6"/>
+      <x:c r="V15" s="6"/>
+      <x:c r="W15" s="6"/>
+      <x:c r="X15" t="str">
+        <x:v>Ontbreekt</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" t="str">
@@ -21032,6 +21201,13 @@
       <x:c r="S16" t="n">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="T16" s="6"/>
+      <x:c r="U16" s="6"/>
+      <x:c r="V16" s="6"/>
+      <x:c r="W16" s="6"/>
+      <x:c r="X16" t="str">
+        <x:v>Ontbreekt</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" t="str">
@@ -21089,6 +21265,13 @@
       <x:c r="S17" t="n">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="T17" s="6"/>
+      <x:c r="U17" s="6"/>
+      <x:c r="V17" s="6"/>
+      <x:c r="W17" s="6"/>
+      <x:c r="X17" t="str">
+        <x:v>Ontbreekt</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" t="str">
@@ -21145,6 +21328,13 @@
       </x:c>
       <x:c r="S18" t="n">
         <x:v>1</x:v>
+      </x:c>
+      <x:c r="T18" s="6"/>
+      <x:c r="U18" s="6"/>
+      <x:c r="V18" s="6"/>
+      <x:c r="W18" s="6"/>
+      <x:c r="X18" t="str">
+        <x:v>Ontbreekt</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -21181,7 +21371,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb843056fab53418a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c804a9c82894b7e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22654,9 +22844,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b34449425a642b4"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d64afe772104be1"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33b85bf4307148a9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26c2cf265b014641"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28683,7 +28873,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea419481d7704b85"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R462dd4938db64ba9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29095,9 +29285,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6fab1b1a0aad4421"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0badde44a34f41c3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2327409988d64c5a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad59a9d07e7c45b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29363,7 +29553,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7dd9151ad2ff4c89"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3ce2c9062614d87"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35188,9 +35378,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63d446ac647b4e0d"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rddb75441bc294572"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R495a6b1b91a44366"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8599710fa06448f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(portal): add delivery and fulfillment pilot flow
</commit_message>
<xml_diff>
--- a/config/product-master-data.xlsx
+++ b/config/product-master-data.xlsx
@@ -2,24 +2,24 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start &amp; beheer" sheetId="1" r:id="Re86206570f384bc8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataclassificatie" sheetId="2" r:id="Rbac3270d41714930"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Productcategorieen" sheetId="3" r:id="R9ec34fc581dc4417"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Producten" sheetId="4" r:id="Rdea86fa6041e4366"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materialen" sheetId="5" r:id="R4babee1df933448b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Componenten" sheetId="6" r:id="R1cf842e924bf4e99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verbindingsrecepten" sheetId="7" r:id="Rd7f6aa9fb1f6426e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categorie-regels" sheetId="8" r:id="Rde659b58769c42aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product-regels" sheetId="9" r:id="Re00fac309c964762"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controles" sheetId="10" r:id="R980c879d80a4465d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open punten" sheetId="11" r:id="R693046ef7dd14c27"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wijzigingslog" sheetId="12" r:id="Rc3a8a232210f4371"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keuzelijsten" sheetId="13" r:id="Ra46d2c4841be46f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prijs &amp; inkoop" sheetId="14" r:id="R7941502811ea4f3a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gereedschappen" sheetId="15" r:id="R23e13f5962c94a7f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAM-parameters" sheetId="16" r:id="R494c13b72c004572"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leveranciers" sheetId="17" r:id="R4fb6efa6b6564310"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product-invoer" sheetId="19" r:id="R7433ab9c9c964f83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start &amp; beheer" sheetId="1" r:id="R93408c95972047c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataclassificatie" sheetId="2" r:id="R85697d7543494ae2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Productcategorieen" sheetId="3" r:id="Rad9ca9ca12ba4961"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Producten" sheetId="4" r:id="R70cc3d9ba1424494"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materialen" sheetId="5" r:id="R6a5119364d554362"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Componenten" sheetId="6" r:id="R41ebefde6d0d4744"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verbindingsrecepten" sheetId="7" r:id="R195c60ece36949fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categorie-regels" sheetId="8" r:id="R0c163935bbc643ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product-regels" sheetId="9" r:id="Rc081055b42384c88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controles" sheetId="10" r:id="R7615d7a06e684f23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open punten" sheetId="11" r:id="Rdd46ca240d114158"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wijzigingslog" sheetId="12" r:id="R364eb6331c20436e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keuzelijsten" sheetId="13" r:id="Rb01e7b0b4eed499c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prijs &amp; inkoop" sheetId="14" r:id="R8729a09354754b5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gereedschappen" sheetId="15" r:id="R37adc65476814054"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAM-parameters" sheetId="16" r:id="Ra34d3c95316c4e72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leveranciers" sheetId="17" r:id="Rfd5ef6c1f9e449ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product-invoer" sheetId="19" r:id="R9fc3bfb1a2884e29"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2871,7 +2871,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R7bc8b0566c504e1c"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc61d2d04cb944c22"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2898,7 +2898,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc920915e595a4f34"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R80e00a6be9c343eb"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2925,7 +2925,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re8be620382704114"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R370fe99a0ca74b1d"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2952,7 +2952,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R949f4d99ceff4f8c"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd86f779be6f049fc"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2979,7 +2979,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R3ac59f17d9aa41e3"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0586da36229d4819"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3006,7 +3006,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rab61268e3a5d4e5b"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R861b2c5e3a0346b0"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3033,7 +3033,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R3e0097d79eb34ac8"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re59bcae64b164809"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3060,7 +3060,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R42fdb9a42e3c48f9"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rb930977d984b4bba"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3087,7 +3087,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra16b12ba44664210"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc25796c83d544be3"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3114,7 +3114,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rf8da65620165458e"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5b6a451745934af1"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3141,7 +3141,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R1232f9d59f054f18"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R145824e34f5f47b9"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3168,7 +3168,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R30d91e7945424737"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R3caffecbe13b4d78"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3195,7 +3195,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5531f8ae670b429a"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rebb62eb5e066420d"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3222,7 +3222,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R26c5577ea29a4939"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R4cb39d2050c44cad"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3249,7 +3249,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R872699ea4cb343d0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rf6ba23bafa494d1a"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3276,7 +3276,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R3ef99c07934c4406"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rccd287fba9fa48d8"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3303,7 +3303,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R17062da2166b41a9"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R6c60358f1f1943c8"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3330,7 +3330,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra9497021aacb4bf1"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R15d669ced8a94af1"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3357,7 +3357,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R470be335151d4af6"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R4d611b00fcc84e20"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3384,7 +3384,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R749d79d74ccc42b3"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Raf1fe019bf1d422f"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3411,7 +3411,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R1bb4263d147f4261"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R86af89a955c34961"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3438,7 +3438,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra8c51fe83c984228"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc9af2994fdab4921"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3465,7 +3465,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R909072e33d2a4cc2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rf15a6b9738634a67"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3492,7 +3492,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R83c4c0cbf84145ad"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R705413faa20246c5"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3519,7 +3519,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R62951a618655401c"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R416aae71f63446bf"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3546,7 +3546,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R8ebc8db871f1417b"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R78563964388d4b86"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3573,7 +3573,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R83f8b0f5df424d27"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rae997be7bbde464e"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3600,7 +3600,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R777739a73d3e4e41"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R97441bfa9339417d"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3627,7 +3627,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0590215860bc43b0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rdbd6f60bd8f14aa3"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3654,7 +3654,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R9dcf4e0235d0419c"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R2cd7a5c1920943e2"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3681,7 +3681,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R4792ca4570c24a9f"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra0fcd5aabad24133"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3708,7 +3708,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5a74e1d29c394043"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R330225369d234867"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3735,7 +3735,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R380e71d0fc9447a8"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R1d7acd9a79854ec7"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3762,7 +3762,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R6427786783c94959"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R3d205d571e534c8a"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3789,7 +3789,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R77e47ba8435e4820"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rbdc25f2d0bf64921"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3816,7 +3816,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R4b1bb3af71fd4b6c"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R4415c29287ef45d4"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3873,7 +3873,7 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="69" name="ChangeLogTable" displayName="ChangeLogTable" ref="A4:H68" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="69" name="ChangeLogTable" displayName="ChangeLogTable" ref="A4:H69" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Column1"/>
     <x:tableColumn id="2" name="Column2"/>
@@ -4039,7 +4039,7 @@
 </file>
 
 <file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="34" name="ProductInputContractsTable" displayName="ProductInputContractsTable" ref="A5:V85" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="34" name="ProductInputContractsTable" displayName="ProductInputContractsTable" ref="A5:V97" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="22">
     <x:tableColumn id="1" name="Invoercontract-ID"/>
     <x:tableColumn id="2" name="Product-ID"/>
@@ -5676,7 +5676,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2754e938dc3e4a60"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda0dd42210154a89"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6294,7 +6294,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbddfd5d0df774dee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6dbc3a4dd1d74d19"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8005,6 +8005,32 @@
         <x:v>Kaartafbeeldingen zijn presentatie en geen technische of productiebron. Bestandsformaat en extensie moeten overeenkomen.</x:v>
       </x:c>
     </x:row>
+    <x:row r="69">
+      <x:c r="A69" t="str">
+        <x:v>CHG-064</x:v>
+      </x:c>
+      <x:c r="B69" t="n">
+        <x:v>46264</x:v>
+      </x:c>
+      <x:c r="C69" t="str">
+        <x:v>Dylan / Codex</x:v>
+      </x:c>
+      <x:c r="D69" t="str">
+        <x:v>5.6</x:v>
+      </x:c>
+      <x:c r="E69" t="str">
+        <x:v>Levervorm, ontvangstwijze en logistieke pilotflow</x:v>
+      </x:c>
+      <x:c r="F69" t="str">
+        <x:v>Alle productfamilies krijgen Bouwpakket en Gemonteerd als toegestane levervormen, met Bouwpakket als standaard. Verzenden en Afhalen worden als verplichte ontvangstkeuze vastgelegd. Montage- en verzendkosten blijven expliciet op aanvraag totdat Bedrijfsbeheer een prijs invult of gevalideerde logistieke rekenlogica beschikbaar is.</x:v>
+      </x:c>
+      <x:c r="G69" t="str">
+        <x:v>PIC-*-DELIVERY-010;PIC-*-DELIVERY-020;DeliveryForm;ReceiptMethod</x:v>
+      </x:c>
+      <x:c r="H69" t="str">
+        <x:v>Automatische verpakking en verzending vereist later klant-/adresgegevens, verpakkingsmaten, profiel-/plaatlengtes en betrouwbare gewichten.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
@@ -8012,7 +8038,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R014036c9939a4ea9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70ff60274a6d48c3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8196,7 +8222,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a1f270748e14e6e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R770856589aaa4e92"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13038,10 +13064,10 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74076ff0b9454528"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc83a1a78a80d445c"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ba7b07cd5334e9b"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71e1e392b5724cde"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2cfb33500214076"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Recdb3792cf904ac1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13611,8 +13637,8 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7b512481fb2404c"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7cfe6592bd6c4e45"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re17c637c951740e1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2bfa981d0b75433a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14390,7 +14416,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa259c8a734d4cb9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re145dcbaf1944109"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15164,8 +15190,8 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20916be63ffb4107"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf416b34d5bc4c46"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5006c8ae6c24f98"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92cba9a3061e4bae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19788,6 +19814,666 @@
         <x:v>Ja</x:v>
       </x:c>
     </x:row>
+    <x:row r="86">
+      <x:c r="A86" t="str">
+        <x:v>PIC-CABINET-DELIVERY-010</x:v>
+      </x:c>
+      <x:c r="B86" t="str">
+        <x:v>cabinet</x:v>
+      </x:c>
+      <x:c r="C86" t="str">
+        <x:v>levering</x:v>
+      </x:c>
+      <x:c r="D86" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E86" t="str">
+        <x:v>deliveryForm</x:v>
+      </x:c>
+      <x:c r="F86" t="str">
+        <x:v>DeliveryForm</x:v>
+      </x:c>
+      <x:c r="G86" t="str">
+        <x:v>Levervorm</x:v>
+      </x:c>
+      <x:c r="H86" t="str">
+        <x:v>select</x:v>
+      </x:c>
+      <x:c r="I86" t="str"/>
+      <x:c r="J86" t="str">
+        <x:v>bouwpakket</x:v>
+      </x:c>
+      <x:c r="K86" t="str"/>
+      <x:c r="L86" t="str"/>
+      <x:c r="M86" t="str"/>
+      <x:c r="N86" t="str"/>
+      <x:c r="O86" t="str">
+        <x:v>bouwpakket|Bouwpakket;gemonteerd|Gemonteerd</x:v>
+      </x:c>
+      <x:c r="P86" t="str"/>
+      <x:c r="Q86" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="R86" t="str">
+        <x:v>Goedgekeurd</x:v>
+      </x:c>
+      <x:c r="S86" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="T86" t="str">
+        <x:v>Pilotbesluit Dylan 2026-08-30</x:v>
+      </x:c>
+      <x:c r="U86" t="str">
+        <x:v>Bouwpakket is de standaard; montageprijs bij gemonteerd wordt door Bedrijfsbeheer vastgesteld.</x:v>
+      </x:c>
+      <x:c r="V86" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87">
+      <x:c r="A87" t="str">
+        <x:v>PIC-CABINET-DELIVERY-020</x:v>
+      </x:c>
+      <x:c r="B87" t="str">
+        <x:v>cabinet</x:v>
+      </x:c>
+      <x:c r="C87" t="str">
+        <x:v>levering</x:v>
+      </x:c>
+      <x:c r="D87" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E87" t="str">
+        <x:v>receiptMethod</x:v>
+      </x:c>
+      <x:c r="F87" t="str">
+        <x:v>ReceiptMethod</x:v>
+      </x:c>
+      <x:c r="G87" t="str">
+        <x:v>Ontvangst</x:v>
+      </x:c>
+      <x:c r="H87" t="str">
+        <x:v>select</x:v>
+      </x:c>
+      <x:c r="I87" t="str"/>
+      <x:c r="J87" t="str"/>
+      <x:c r="K87" t="str"/>
+      <x:c r="L87" t="str"/>
+      <x:c r="M87" t="str"/>
+      <x:c r="N87" t="str"/>
+      <x:c r="O87" t="str">
+        <x:v>verzenden|Verzenden;afhalen|Afhalen</x:v>
+      </x:c>
+      <x:c r="P87" t="str"/>
+      <x:c r="Q87" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="R87" t="str">
+        <x:v>Goedgekeurd</x:v>
+      </x:c>
+      <x:c r="S87" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="T87" t="str">
+        <x:v>Pilotbesluit Dylan 2026-08-30</x:v>
+      </x:c>
+      <x:c r="U87" t="str">
+        <x:v>Afhalen is toegestaan; verzendkosten blijven open totdat logistieke brondata en rekenlogica compleet zijn.</x:v>
+      </x:c>
+      <x:c r="V87" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88">
+      <x:c r="A88" t="str">
+        <x:v>PIC-WORKTABLE-DELIVERY-010</x:v>
+      </x:c>
+      <x:c r="B88" t="str">
+        <x:v>werktafel</x:v>
+      </x:c>
+      <x:c r="C88" t="str">
+        <x:v>levering</x:v>
+      </x:c>
+      <x:c r="D88" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E88" t="str">
+        <x:v>deliveryForm</x:v>
+      </x:c>
+      <x:c r="F88" t="str">
+        <x:v>DeliveryForm</x:v>
+      </x:c>
+      <x:c r="G88" t="str">
+        <x:v>Levervorm</x:v>
+      </x:c>
+      <x:c r="H88" t="str">
+        <x:v>select</x:v>
+      </x:c>
+      <x:c r="I88" t="str"/>
+      <x:c r="J88" t="str">
+        <x:v>bouwpakket</x:v>
+      </x:c>
+      <x:c r="K88" t="str"/>
+      <x:c r="L88" t="str"/>
+      <x:c r="M88" t="str"/>
+      <x:c r="N88" t="str"/>
+      <x:c r="O88" t="str">
+        <x:v>bouwpakket|Bouwpakket;gemonteerd|Gemonteerd</x:v>
+      </x:c>
+      <x:c r="P88" t="str"/>
+      <x:c r="Q88" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="R88" t="str">
+        <x:v>Goedgekeurd</x:v>
+      </x:c>
+      <x:c r="S88" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="T88" t="str">
+        <x:v>Pilotbesluit Dylan 2026-08-30</x:v>
+      </x:c>
+      <x:c r="U88" t="str">
+        <x:v>Bouwpakket is de standaard; montageprijs bij gemonteerd wordt door Bedrijfsbeheer vastgesteld.</x:v>
+      </x:c>
+      <x:c r="V88" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89">
+      <x:c r="A89" t="str">
+        <x:v>PIC-WORKTABLE-DELIVERY-020</x:v>
+      </x:c>
+      <x:c r="B89" t="str">
+        <x:v>werktafel</x:v>
+      </x:c>
+      <x:c r="C89" t="str">
+        <x:v>levering</x:v>
+      </x:c>
+      <x:c r="D89" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E89" t="str">
+        <x:v>receiptMethod</x:v>
+      </x:c>
+      <x:c r="F89" t="str">
+        <x:v>ReceiptMethod</x:v>
+      </x:c>
+      <x:c r="G89" t="str">
+        <x:v>Ontvangst</x:v>
+      </x:c>
+      <x:c r="H89" t="str">
+        <x:v>select</x:v>
+      </x:c>
+      <x:c r="I89" t="str"/>
+      <x:c r="J89" t="str"/>
+      <x:c r="K89" t="str"/>
+      <x:c r="L89" t="str"/>
+      <x:c r="M89" t="str"/>
+      <x:c r="N89" t="str"/>
+      <x:c r="O89" t="str">
+        <x:v>verzenden|Verzenden;afhalen|Afhalen</x:v>
+      </x:c>
+      <x:c r="P89" t="str"/>
+      <x:c r="Q89" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="R89" t="str">
+        <x:v>Goedgekeurd</x:v>
+      </x:c>
+      <x:c r="S89" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="T89" t="str">
+        <x:v>Pilotbesluit Dylan 2026-08-30</x:v>
+      </x:c>
+      <x:c r="U89" t="str">
+        <x:v>Afhalen is toegestaan; verzendkosten blijven open totdat logistieke brondata en rekenlogica compleet zijn.</x:v>
+      </x:c>
+      <x:c r="V89" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90">
+      <x:c r="A90" t="str">
+        <x:v>PIC-SHIPPING-BOX-DELIVERY-010</x:v>
+      </x:c>
+      <x:c r="B90" t="str">
+        <x:v>shipping_box</x:v>
+      </x:c>
+      <x:c r="C90" t="str">
+        <x:v>levering</x:v>
+      </x:c>
+      <x:c r="D90" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E90" t="str">
+        <x:v>deliveryForm</x:v>
+      </x:c>
+      <x:c r="F90" t="str">
+        <x:v>DeliveryForm</x:v>
+      </x:c>
+      <x:c r="G90" t="str">
+        <x:v>Levervorm</x:v>
+      </x:c>
+      <x:c r="H90" t="str">
+        <x:v>select</x:v>
+      </x:c>
+      <x:c r="I90" t="str"/>
+      <x:c r="J90" t="str">
+        <x:v>bouwpakket</x:v>
+      </x:c>
+      <x:c r="K90" t="str"/>
+      <x:c r="L90" t="str"/>
+      <x:c r="M90" t="str"/>
+      <x:c r="N90" t="str"/>
+      <x:c r="O90" t="str">
+        <x:v>bouwpakket|Bouwpakket;gemonteerd|Gemonteerd</x:v>
+      </x:c>
+      <x:c r="P90" t="str"/>
+      <x:c r="Q90" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="R90" t="str">
+        <x:v>Goedgekeurd</x:v>
+      </x:c>
+      <x:c r="S90" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="T90" t="str">
+        <x:v>Pilotbesluit Dylan 2026-08-30</x:v>
+      </x:c>
+      <x:c r="U90" t="str">
+        <x:v>Bouwpakket is de standaard; montageprijs bij gemonteerd wordt door Bedrijfsbeheer vastgesteld.</x:v>
+      </x:c>
+      <x:c r="V90" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91">
+      <x:c r="A91" t="str">
+        <x:v>PIC-SHIPPING-BOX-DELIVERY-020</x:v>
+      </x:c>
+      <x:c r="B91" t="str">
+        <x:v>shipping_box</x:v>
+      </x:c>
+      <x:c r="C91" t="str">
+        <x:v>levering</x:v>
+      </x:c>
+      <x:c r="D91" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E91" t="str">
+        <x:v>receiptMethod</x:v>
+      </x:c>
+      <x:c r="F91" t="str">
+        <x:v>ReceiptMethod</x:v>
+      </x:c>
+      <x:c r="G91" t="str">
+        <x:v>Ontvangst</x:v>
+      </x:c>
+      <x:c r="H91" t="str">
+        <x:v>select</x:v>
+      </x:c>
+      <x:c r="I91" t="str"/>
+      <x:c r="J91" t="str"/>
+      <x:c r="K91" t="str"/>
+      <x:c r="L91" t="str"/>
+      <x:c r="M91" t="str"/>
+      <x:c r="N91" t="str"/>
+      <x:c r="O91" t="str">
+        <x:v>verzenden|Verzenden;afhalen|Afhalen</x:v>
+      </x:c>
+      <x:c r="P91" t="str"/>
+      <x:c r="Q91" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="R91" t="str">
+        <x:v>Goedgekeurd</x:v>
+      </x:c>
+      <x:c r="S91" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="T91" t="str">
+        <x:v>Pilotbesluit Dylan 2026-08-30</x:v>
+      </x:c>
+      <x:c r="U91" t="str">
+        <x:v>Afhalen is toegestaan; verzendkosten blijven open totdat logistieke brondata en rekenlogica compleet zijn.</x:v>
+      </x:c>
+      <x:c r="V91" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92">
+      <x:c r="A92" t="str">
+        <x:v>PIC-MACHINEBASE-DELIVERY-010</x:v>
+      </x:c>
+      <x:c r="B92" t="str">
+        <x:v>machinebasis</x:v>
+      </x:c>
+      <x:c r="C92" t="str">
+        <x:v>levering</x:v>
+      </x:c>
+      <x:c r="D92" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E92" t="str">
+        <x:v>deliveryForm</x:v>
+      </x:c>
+      <x:c r="F92" t="str">
+        <x:v>DeliveryForm</x:v>
+      </x:c>
+      <x:c r="G92" t="str">
+        <x:v>Levervorm</x:v>
+      </x:c>
+      <x:c r="H92" t="str">
+        <x:v>select</x:v>
+      </x:c>
+      <x:c r="I92" t="str"/>
+      <x:c r="J92" t="str">
+        <x:v>bouwpakket</x:v>
+      </x:c>
+      <x:c r="K92" t="str"/>
+      <x:c r="L92" t="str"/>
+      <x:c r="M92" t="str"/>
+      <x:c r="N92" t="str"/>
+      <x:c r="O92" t="str">
+        <x:v>bouwpakket|Bouwpakket;gemonteerd|Gemonteerd</x:v>
+      </x:c>
+      <x:c r="P92" t="str"/>
+      <x:c r="Q92" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="R92" t="str">
+        <x:v>Goedgekeurd</x:v>
+      </x:c>
+      <x:c r="S92" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="T92" t="str">
+        <x:v>Pilotbesluit Dylan 2026-08-30</x:v>
+      </x:c>
+      <x:c r="U92" t="str">
+        <x:v>Bouwpakket is de standaard; montageprijs bij gemonteerd wordt door Bedrijfsbeheer vastgesteld.</x:v>
+      </x:c>
+      <x:c r="V92" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93">
+      <x:c r="A93" t="str">
+        <x:v>PIC-MACHINEBASE-DELIVERY-020</x:v>
+      </x:c>
+      <x:c r="B93" t="str">
+        <x:v>machinebasis</x:v>
+      </x:c>
+      <x:c r="C93" t="str">
+        <x:v>levering</x:v>
+      </x:c>
+      <x:c r="D93" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E93" t="str">
+        <x:v>receiptMethod</x:v>
+      </x:c>
+      <x:c r="F93" t="str">
+        <x:v>ReceiptMethod</x:v>
+      </x:c>
+      <x:c r="G93" t="str">
+        <x:v>Ontvangst</x:v>
+      </x:c>
+      <x:c r="H93" t="str">
+        <x:v>select</x:v>
+      </x:c>
+      <x:c r="I93" t="str"/>
+      <x:c r="J93" t="str"/>
+      <x:c r="K93" t="str"/>
+      <x:c r="L93" t="str"/>
+      <x:c r="M93" t="str"/>
+      <x:c r="N93" t="str"/>
+      <x:c r="O93" t="str">
+        <x:v>verzenden|Verzenden;afhalen|Afhalen</x:v>
+      </x:c>
+      <x:c r="P93" t="str"/>
+      <x:c r="Q93" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="R93" t="str">
+        <x:v>Goedgekeurd</x:v>
+      </x:c>
+      <x:c r="S93" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="T93" t="str">
+        <x:v>Pilotbesluit Dylan 2026-08-30</x:v>
+      </x:c>
+      <x:c r="U93" t="str">
+        <x:v>Afhalen is toegestaan; verzendkosten blijven open totdat logistieke brondata en rekenlogica compleet zijn.</x:v>
+      </x:c>
+      <x:c r="V93" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94">
+      <x:c r="A94" t="str">
+        <x:v>PIC-LINEAR-ROBOT-CELL-DELIVERY-010</x:v>
+      </x:c>
+      <x:c r="B94" t="str">
+        <x:v>lineaire_robotcel</x:v>
+      </x:c>
+      <x:c r="C94" t="str">
+        <x:v>levering</x:v>
+      </x:c>
+      <x:c r="D94" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E94" t="str">
+        <x:v>deliveryForm</x:v>
+      </x:c>
+      <x:c r="F94" t="str">
+        <x:v>DeliveryForm</x:v>
+      </x:c>
+      <x:c r="G94" t="str">
+        <x:v>Levervorm</x:v>
+      </x:c>
+      <x:c r="H94" t="str">
+        <x:v>select</x:v>
+      </x:c>
+      <x:c r="I94" t="str"/>
+      <x:c r="J94" t="str">
+        <x:v>bouwpakket</x:v>
+      </x:c>
+      <x:c r="K94" t="str"/>
+      <x:c r="L94" t="str"/>
+      <x:c r="M94" t="str"/>
+      <x:c r="N94" t="str"/>
+      <x:c r="O94" t="str">
+        <x:v>bouwpakket|Bouwpakket;gemonteerd|Gemonteerd</x:v>
+      </x:c>
+      <x:c r="P94" t="str"/>
+      <x:c r="Q94" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="R94" t="str">
+        <x:v>Goedgekeurd</x:v>
+      </x:c>
+      <x:c r="S94" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="T94" t="str">
+        <x:v>Pilotbesluit Dylan 2026-08-30</x:v>
+      </x:c>
+      <x:c r="U94" t="str">
+        <x:v>Bouwpakket is de standaard; montageprijs bij gemonteerd wordt door Bedrijfsbeheer vastgesteld.</x:v>
+      </x:c>
+      <x:c r="V94" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95">
+      <x:c r="A95" t="str">
+        <x:v>PIC-LINEAR-ROBOT-CELL-DELIVERY-020</x:v>
+      </x:c>
+      <x:c r="B95" t="str">
+        <x:v>lineaire_robotcel</x:v>
+      </x:c>
+      <x:c r="C95" t="str">
+        <x:v>levering</x:v>
+      </x:c>
+      <x:c r="D95" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E95" t="str">
+        <x:v>receiptMethod</x:v>
+      </x:c>
+      <x:c r="F95" t="str">
+        <x:v>ReceiptMethod</x:v>
+      </x:c>
+      <x:c r="G95" t="str">
+        <x:v>Ontvangst</x:v>
+      </x:c>
+      <x:c r="H95" t="str">
+        <x:v>select</x:v>
+      </x:c>
+      <x:c r="I95" t="str"/>
+      <x:c r="J95" t="str"/>
+      <x:c r="K95" t="str"/>
+      <x:c r="L95" t="str"/>
+      <x:c r="M95" t="str"/>
+      <x:c r="N95" t="str"/>
+      <x:c r="O95" t="str">
+        <x:v>verzenden|Verzenden;afhalen|Afhalen</x:v>
+      </x:c>
+      <x:c r="P95" t="str"/>
+      <x:c r="Q95" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="R95" t="str">
+        <x:v>Goedgekeurd</x:v>
+      </x:c>
+      <x:c r="S95" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="T95" t="str">
+        <x:v>Pilotbesluit Dylan 2026-08-30</x:v>
+      </x:c>
+      <x:c r="U95" t="str">
+        <x:v>Afhalen is toegestaan; verzendkosten blijven open totdat logistieke brondata en rekenlogica compleet zijn.</x:v>
+      </x:c>
+      <x:c r="V95" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96">
+      <x:c r="A96" t="str">
+        <x:v>PIC-HEIGHT-ADJUSTABLE-WORKTABLE-DELIVERY-010</x:v>
+      </x:c>
+      <x:c r="B96" t="str">
+        <x:v>hoogteverstelbare_werktafel</x:v>
+      </x:c>
+      <x:c r="C96" t="str">
+        <x:v>levering</x:v>
+      </x:c>
+      <x:c r="D96" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E96" t="str">
+        <x:v>deliveryForm</x:v>
+      </x:c>
+      <x:c r="F96" t="str">
+        <x:v>DeliveryForm</x:v>
+      </x:c>
+      <x:c r="G96" t="str">
+        <x:v>Levervorm</x:v>
+      </x:c>
+      <x:c r="H96" t="str">
+        <x:v>select</x:v>
+      </x:c>
+      <x:c r="I96" t="str"/>
+      <x:c r="J96" t="str">
+        <x:v>bouwpakket</x:v>
+      </x:c>
+      <x:c r="K96" t="str"/>
+      <x:c r="L96" t="str"/>
+      <x:c r="M96" t="str"/>
+      <x:c r="N96" t="str"/>
+      <x:c r="O96" t="str">
+        <x:v>bouwpakket|Bouwpakket;gemonteerd|Gemonteerd</x:v>
+      </x:c>
+      <x:c r="P96" t="str"/>
+      <x:c r="Q96" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="R96" t="str">
+        <x:v>Goedgekeurd</x:v>
+      </x:c>
+      <x:c r="S96" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="T96" t="str">
+        <x:v>Pilotbesluit Dylan 2026-08-30</x:v>
+      </x:c>
+      <x:c r="U96" t="str">
+        <x:v>Bouwpakket is de standaard; montageprijs bij gemonteerd wordt door Bedrijfsbeheer vastgesteld.</x:v>
+      </x:c>
+      <x:c r="V96" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97">
+      <x:c r="A97" t="str">
+        <x:v>PIC-HEIGHT-ADJUSTABLE-WORKTABLE-DELIVERY-020</x:v>
+      </x:c>
+      <x:c r="B97" t="str">
+        <x:v>hoogteverstelbare_werktafel</x:v>
+      </x:c>
+      <x:c r="C97" t="str">
+        <x:v>levering</x:v>
+      </x:c>
+      <x:c r="D97" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E97" t="str">
+        <x:v>receiptMethod</x:v>
+      </x:c>
+      <x:c r="F97" t="str">
+        <x:v>ReceiptMethod</x:v>
+      </x:c>
+      <x:c r="G97" t="str">
+        <x:v>Ontvangst</x:v>
+      </x:c>
+      <x:c r="H97" t="str">
+        <x:v>select</x:v>
+      </x:c>
+      <x:c r="I97" t="str"/>
+      <x:c r="J97" t="str"/>
+      <x:c r="K97" t="str"/>
+      <x:c r="L97" t="str"/>
+      <x:c r="M97" t="str"/>
+      <x:c r="N97" t="str"/>
+      <x:c r="O97" t="str">
+        <x:v>verzenden|Verzenden;afhalen|Afhalen</x:v>
+      </x:c>
+      <x:c r="P97" t="str"/>
+      <x:c r="Q97" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="R97" t="str">
+        <x:v>Goedgekeurd</x:v>
+      </x:c>
+      <x:c r="S97" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="T97" t="str">
+        <x:v>Pilotbesluit Dylan 2026-08-30</x:v>
+      </x:c>
+      <x:c r="U97" t="str">
+        <x:v>Afhalen is toegestaan; verzendkosten blijven open totdat logistieke brondata en rekenlogica compleet zijn.</x:v>
+      </x:c>
+      <x:c r="V97" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:V1"/>
@@ -19795,7 +20481,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9c00185bd0b4b36"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0bf4d0776061411e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20079,7 +20765,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53ba34e739b84dd3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f526d49a2814e99"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20276,7 +20962,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf8597285ded048fb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a7d2e6935d845c2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21371,7 +22057,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c804a9c82894b7e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1131305f1eb4794"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22844,9 +23530,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d64afe772104be1"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf172f079644e4307"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26c2cf265b014641"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71d596107307450f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28873,7 +29559,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R462dd4938db64ba9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra22212b4654b430d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29285,9 +29971,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0badde44a34f41c3"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4daeb8da47ea4439"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad59a9d07e7c45b1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbffb156467414b78"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29553,7 +30239,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3ce2c9062614d87"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38f2a7931d934d3e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35378,9 +36064,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rddb75441bc294572"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb396d107f740434b"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8599710fa06448f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9acf3cfd2c1b48fa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(products): add folding workbench and harden sheet models
</commit_message>
<xml_diff>
--- a/config/product-master-data.xlsx
+++ b/config/product-master-data.xlsx
@@ -2,24 +2,24 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start &amp; beheer" sheetId="1" r:id="R93408c95972047c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataclassificatie" sheetId="2" r:id="R85697d7543494ae2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Productcategorieen" sheetId="3" r:id="Rad9ca9ca12ba4961"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Producten" sheetId="4" r:id="R70cc3d9ba1424494"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materialen" sheetId="5" r:id="R6a5119364d554362"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Componenten" sheetId="6" r:id="R41ebefde6d0d4744"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verbindingsrecepten" sheetId="7" r:id="R195c60ece36949fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categorie-regels" sheetId="8" r:id="R0c163935bbc643ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product-regels" sheetId="9" r:id="Rc081055b42384c88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controles" sheetId="10" r:id="R7615d7a06e684f23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open punten" sheetId="11" r:id="Rdd46ca240d114158"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wijzigingslog" sheetId="12" r:id="R364eb6331c20436e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keuzelijsten" sheetId="13" r:id="Rb01e7b0b4eed499c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prijs &amp; inkoop" sheetId="14" r:id="R8729a09354754b5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gereedschappen" sheetId="15" r:id="R37adc65476814054"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAM-parameters" sheetId="16" r:id="Ra34d3c95316c4e72"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leveranciers" sheetId="17" r:id="Rfd5ef6c1f9e449ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product-invoer" sheetId="19" r:id="R9fc3bfb1a2884e29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start &amp; beheer" sheetId="1" r:id="R03fa9146ad8f43ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataclassificatie" sheetId="2" r:id="R598bec0fa31a4a1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Productcategorieen" sheetId="3" r:id="R790c096416694673"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Producten" sheetId="4" r:id="Rb7a4955578404bef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materialen" sheetId="5" r:id="R7a31a57aa6904f98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Componenten" sheetId="6" r:id="R937aec913170418b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verbindingsrecepten" sheetId="7" r:id="R5d94ff0b7e6749f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categorie-regels" sheetId="8" r:id="Ra405018585604198"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product-regels" sheetId="9" r:id="R9a239ba3920f4eef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controles" sheetId="10" r:id="Ra8a94f19a0134e53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open punten" sheetId="11" r:id="R2911b927b5514bb8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wijzigingslog" sheetId="12" r:id="R004e93b950424e84"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keuzelijsten" sheetId="13" r:id="Rf4b1d441673d4af1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prijs &amp; inkoop" sheetId="14" r:id="Red90aae304134d6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gereedschappen" sheetId="15" r:id="Rcf674f8f9c24451e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAM-parameters" sheetId="16" r:id="Rc5179716b90b462e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leveranciers" sheetId="17" r:id="Rac13479471c24eeb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product-invoer" sheetId="19" r:id="R5081224cd255410f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2871,7 +2871,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc61d2d04cb944c22"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra28531af8c504be0"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2898,7 +2898,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R80e00a6be9c343eb"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R2aacafc70bb44818"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2925,7 +2925,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R370fe99a0ca74b1d"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R1f829dbf45be4d70"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2952,7 +2952,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd86f779be6f049fc"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re7efb251a44942b6"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2979,7 +2979,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0586da36229d4819"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rdc80549187a94637"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3006,7 +3006,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R861b2c5e3a0346b0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R377eaf02d8d147bc"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3033,7 +3033,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re59bcae64b164809"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rcd68d4dda3ee4af8"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3060,7 +3060,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rb930977d984b4bba"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R6e0189dccafe4e62"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3087,7 +3087,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc25796c83d544be3"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R31fc42a3f2204b46"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3114,7 +3114,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5b6a451745934af1"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R7dfb17adc62d4587"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3141,7 +3141,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R145824e34f5f47b9"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0385504d806a4a0e"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3168,7 +3168,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R3caffecbe13b4d78"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc073dc65ab1e45de"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3195,7 +3195,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rebb62eb5e066420d"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R9e1ce54a18cb4eb9"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3222,7 +3222,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R4cb39d2050c44cad"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R89028671242d4683"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3249,7 +3249,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rf6ba23bafa494d1a"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rf03bb06bfc8a471e"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3276,7 +3276,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rccd287fba9fa48d8"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R4fd15820a30e4994"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3303,7 +3303,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R6c60358f1f1943c8"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R6416b91133a54f6e"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3330,7 +3330,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R15d669ced8a94af1"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Raabc8ca2b2c24855"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3357,7 +3357,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R4d611b00fcc84e20"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R36fbadd148ca4835"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3384,7 +3384,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Raf1fe019bf1d422f"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R8df5427085a4495f"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3411,7 +3411,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R86af89a955c34961"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R084fd2e6c732495a"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3438,7 +3438,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc9af2994fdab4921"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R3c5aa00b1ebe4a97"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3465,7 +3465,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rf15a6b9738634a67"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd838a25d4c2b4478"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3492,7 +3492,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R705413faa20246c5"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rdeaf567934d14931"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3519,7 +3519,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R416aae71f63446bf"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc9e67f7e74d64703"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3546,7 +3546,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R78563964388d4b86"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rab0fcc2d155940d3"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3573,7 +3573,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rae997be7bbde464e"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R92610fbc5cbe4179"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3600,7 +3600,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R97441bfa9339417d"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R2c2d0c93ce2b48e9"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3627,7 +3627,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rdbd6f60bd8f14aa3"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rfa35ca1a6b714f21"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3654,7 +3654,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R2cd7a5c1920943e2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R2b334eebd3dc4ee6"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3681,7 +3681,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra0fcd5aabad24133"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R1d4fdbc583814550"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3708,7 +3708,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R330225369d234867"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R688c27fd9c3a452a"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3735,7 +3735,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R1d7acd9a79854ec7"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R65d4a7c665154e47"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3762,7 +3762,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R3d205d571e534c8a"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rf2f9834946e34423"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3789,7 +3789,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rbdc25f2d0bf64921"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5b8f3a2720054509"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3816,7 +3816,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R4415c29287ef45d4"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re2240557f069487c"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3873,7 +3873,7 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="69" name="ChangeLogTable" displayName="ChangeLogTable" ref="A4:H69" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="69" name="ChangeLogTable" displayName="ChangeLogTable" ref="A4:H82" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Column1"/>
     <x:tableColumn id="2" name="Column2"/>
@@ -3900,7 +3900,7 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="61" name="PricingProcurementTable" displayName="PricingProcurementTable" ref="A5:AC70" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="61" name="PricingProcurementTable" displayName="PricingProcurementTable" ref="A5:AC71" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="29">
     <x:tableColumn id="1" name="Aanbieding-ID"/>
     <x:tableColumn id="2" name="Recordtype"/>
@@ -4039,7 +4039,7 @@
 </file>
 
 <file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="34" name="ProductInputContractsTable" displayName="ProductInputContractsTable" ref="A5:V97" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="34" name="ProductInputContractsTable" displayName="ProductInputContractsTable" ref="A5:V102" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="22">
     <x:tableColumn id="1" name="Invoercontract-ID"/>
     <x:tableColumn id="2" name="Product-ID"/>
@@ -4087,7 +4087,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="70" name="ProductsTable" displayName="ProductsTable" ref="A5:X18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="70" name="ProductsTable" displayName="ProductsTable" ref="A5:X19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="24">
     <x:tableColumn id="1" name="Product-ID"/>
     <x:tableColumn id="2" name="Naam"/>
@@ -4160,7 +4160,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="63" name="ComponentsTable" displayName="ComponentsTable" ref="A5:AX80" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="63" name="ComponentsTable" displayName="ComponentsTable" ref="A5:AX81" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="50">
     <x:tableColumn id="1" name="Component-ID"/>
     <x:tableColumn id="2" name="Type"/>
@@ -4257,7 +4257,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="59" name="ProductRulesTable" displayName="ProductRulesTable" ref="A5:O113" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="59" name="ProductRulesTable" displayName="ProductRulesTable" ref="A5:O130" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="15">
     <x:tableColumn id="1" name="Regel-ID"/>
     <x:tableColumn id="2" name="Product-ID"/>
@@ -4280,8 +4280,8 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="ValidationRulesTable" displayName="ValidationRulesTable" ref="A5:I26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:I26"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="ValidationRulesTable" displayName="ValidationRulesTable" ref="A5:I30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:I30"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Controle-ID"/>
     <x:tableColumn id="2" name="Scope"/>
@@ -5628,16 +5628,16 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" t="str">
-        <x:v>VAL-LEX-003</x:v>
+        <x:v>VAL-FWT-001</x:v>
       </x:c>
       <x:c r="B27" t="str">
-        <x:v>LEX workstation</x:v>
+        <x:v>opvouwbare_werktafel</x:v>
       </x:c>
       <x:c r="C27" t="str">
-        <x:v>Draaibare aanslagen</x:v>
+        <x:v>Kinematica</x:v>
       </x:c>
       <x:c r="D27" t="str">
-        <x:v>Exact zes Item 0.0.700.81 aanslagen: 2 voor, 2 achter, 1 links en 1 rechts; buitenenvelop uit masterdata en alle delen buiten HPL</x:v>
+        <x:v>Het werkblad steekt uniform 80 mm rondom over en leidt bij 2400 × 1180 mm een onderstel van 2240 × 1020 mm af. Twee vaste lange framepanelen hebben elk drie geïntegreerde voeten, vier korte volledige framevormige vouwpanelen elk twee geïntegreerde voeten en het onderstel exact zes verticale scharnierassen. Alleen de voetvelden onder de stijlen raken de vloer; de onderrand ertussen ligt 30 mm terug. Alle paneelnokken en bladslots volgen dezelfde 80-mm inset. Elk scharnier verbindt expliciet de bedoelde twee platen, heeft drie fysieke delen, drie gaten per blad en zit bij de buitenassen aan de binnenzijde; open, halfgevouwen en vlakgevouwen keyframes sluiten zonder onderdeelrek of penetratie</x:v>
       </x:c>
       <x:c r="E27" t="str">
         <x:v>Kritiek</x:v>
@@ -5646,13 +5646,100 @@
         <x:v>Ja</x:v>
       </x:c>
       <x:c r="G27" t="str">
-        <x:v>Aanslag ontbreekt, staat asymmetrisch of doorkruist het werkblad</x:v>
+        <x:v>Afwijkende onderdelen, scharnierassen of niet-sluitende vouwstand blokkeren conceptacceptatie</x:v>
       </x:c>
       <x:c r="H27" t="str">
-        <x:v>Leveranciersdata</x:v>
+        <x:v>Geïmplementeerd</x:v>
       </x:c>
       <x:c r="I27" t="str">
-        <x:v>WorkbenchCabinetAuditService + ProductContracts.RegressionTests</x:v>
+        <x:v>FoldingWorkbenchEngine SheetHinge-verbindingen en part-attachments; PortalMotionContractService rigide bewegingsdrivers; ProductContracts.RegressionTests; AXA tekening 1KL227676; geannoteerde fotoreferentie 2026-09-01</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" t="str">
+        <x:v>VAL-FWT-002</x:v>
+      </x:c>
+      <x:c r="B28" t="str">
+        <x:v>opvouwbare_werktafel</x:v>
+      </x:c>
+      <x:c r="C28" t="str">
+        <x:v>Gat-/nokpassing</x:v>
+      </x:c>
+      <x:c r="D28" t="str">
+        <x:v>Exact veertien volle-diepte werkbladslots met 1 mm vrije ruimte per zijde en dogbone-ontlasting uit het gekoppelde freesrecord; fysiek proefstuk bevestigt passing en uitneembaarheid</x:v>
+      </x:c>
+      <x:c r="E28" t="str">
+        <x:v>Kritiek</x:v>
+      </x:c>
+      <x:c r="F28" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="G28" t="str">
+        <x:v>Geen productie-CAM vóór gefreesde passtest en vastgelegde L-eindslotcontour</x:v>
+      </x:c>
+      <x:c r="H28" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="I28" t="str">
+        <x:v>Backendgeometrie geïmplementeerd voor zes langspaneel- en acht korte-paneelnokken; fysieke proefpassing vereist</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" t="str">
+        <x:v>VAL-FWT-003</x:v>
+      </x:c>
+      <x:c r="B29" t="str">
+        <x:v>opvouwbare_werktafel</x:v>
+      </x:c>
+      <x:c r="C29" t="str">
+        <x:v>Scharnier en bevestiging</x:v>
+      </x:c>
+      <x:c r="D29" t="str">
+        <x:v>G Goedkoop 0000006696 sample is ingemeten; gaten, schroefdiameter, -lengte, randafstand, knokkelmaat en belastbaarheid zijn gekoppeld aan stabiele componentrecords</x:v>
+      </x:c>
+      <x:c r="E29" t="str">
+        <x:v>Kritiek</x:v>
+      </x:c>
+      <x:c r="F29" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="G29" t="str">
+        <x:v>Scharnieren en bevestigers niet productievrij zonder samplemeting; fysieke proef bepaalt één of twee scharnieren per as</x:v>
+      </x:c>
+      <x:c r="H29" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="I29" t="str">
+        <x:v>Leverancierssample en bevestigerselectie vereist</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" t="str">
+        <x:v>VAL-FWT-004</x:v>
+      </x:c>
+      <x:c r="B30" t="str">
+        <x:v>opvouwbare_werktafel</x:v>
+      </x:c>
+      <x:c r="C30" t="str">
+        <x:v>Belasting en stabiliteit</x:v>
+      </x:c>
+      <x:c r="D30" t="str">
+        <x:v>Ontwerpbelasting, veiligheidsfactor, blad-/frame-doorbuiging, korte vouwpaneel- en nokbelasting, zijdelingse stabiliteit en risico op onbedoeld uitlichten zijn beproefd</x:v>
+      </x:c>
+      <x:c r="E30" t="str">
+        <x:v>Kritiek</x:v>
+      </x:c>
+      <x:c r="F30" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="G30" t="str">
+        <x:v>Werkbelasting niet publiceren en product niet vrijgeven vóór constructie- en proefbelasting</x:v>
+      </x:c>
+      <x:c r="H30" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="I30" t="str">
+        <x:v>Vaststellen na goedgekeurde constructievisualisatie en fysieke proefopstelling</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5676,7 +5763,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda0dd42210154a89"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e932dac50a44efc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6294,7 +6381,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6dbc3a4dd1d74d19"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ee6a2747c924b3c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8031,6 +8118,344 @@
         <x:v>Automatische verpakking en verzending vereist later klant-/adresgegevens, verpakkingsmaten, profiel-/plaatlengtes en betrouwbare gewichten.</x:v>
       </x:c>
     </x:row>
+    <x:row r="70">
+      <x:c r="A70" t="str">
+        <x:v>CHG-065</x:v>
+      </x:c>
+      <x:c r="B70" t="str">
+        <x:v>2026-08-30</x:v>
+      </x:c>
+      <x:c r="C70" t="str">
+        <x:v>Dylan / Codex</x:v>
+      </x:c>
+      <x:c r="D70" t="str">
+        <x:v>5.7</x:v>
+      </x:c>
+      <x:c r="E70" t="str">
+        <x:v>Shipping-boxmaten gekoppeld aan OSB-handelsplaat</x:v>
+      </x:c>
+      <x:c r="F70" t="str">
+        <x:v>De configurator accepteert alle binnenmaatcombinaties waarvan elk van de zes gegenereerde panelen, eventueel 90 graden gedraaid, uit OSB 18 mm van 2440 x 1220 mm past. Brede globale invoergrenzen worden gecombineerd met dynamische plaatpassing; nesting bepaalt het benodigde aantal platen.</x:v>
+      </x:c>
+      <x:c r="G70" t="str">
+        <x:v>shipping_box;PRD-SBX-010;osb_18;ShippingBoxEngine</x:v>
+      </x:c>
+      <x:c r="H70" t="str">
+        <x:v>Minimum 200 mm blijft de bestaande proefstukondergrens. Exacte plaatrand-/opspanmarge blijft buiten productie-vrijgave zolang die niet afzonderlijk is vastgesteld.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" t="str">
+        <x:v>CHG-066</x:v>
+      </x:c>
+      <x:c r="B71" t="str">
+        <x:v>2026-08-30</x:v>
+      </x:c>
+      <x:c r="C71" t="str">
+        <x:v>Dylan / Codex</x:v>
+      </x:c>
+      <x:c r="D71" t="str">
+        <x:v>5.8</x:v>
+      </x:c>
+      <x:c r="E71" t="str">
+        <x:v>Shipping-boxplaatmarge 40 mm</x:v>
+      </x:c>
+      <x:c r="F71" t="str">
+        <x:v>Het bruikbare OSB-formaat wordt voor de configurator 2400 x 1180 mm: nominale lengte en breedte min 40 mm. De maximale binnenmaten worden 2364 x 2364 x 2400 mm, gecombineerd met dynamische paneelpassing en 90 graden rotatie.</x:v>
+      </x:c>
+      <x:c r="G71" t="str">
+        <x:v>shipping_box;PRD-SBX-010;PRD-SBX-011;osb_18;ShippingBoxEngine</x:v>
+      </x:c>
+      <x:c r="H71" t="str">
+        <x:v>De reductie is 40 mm totaal per plaatrichting en staat gelijk aan 20 mm randmarge per zijde. Overige proefstuk- en productievrijgaven blijven ongewijzigd.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" t="str">
+        <x:v>CHG-067</x:v>
+      </x:c>
+      <x:c r="B72" s="64" t="n">
+        <x:v>46264</x:v>
+      </x:c>
+      <x:c r="C72" t="str">
+        <x:v>Dylan / Codex</x:v>
+      </x:c>
+      <x:c r="D72" t="str">
+        <x:v>5.9</x:v>
+      </x:c>
+      <x:c r="E72" t="str">
+        <x:v>Gedeeld klemmodel, SolidWorks-proefmacro en OSB-materiaalweergave</x:v>
+      </x:c>
+      <x:c r="F72" t="str">
+        <x:v>Liangyue LY103-12 krijgt één centraal voorlopig primitief rendercontract op basis van de reeds vastgelegde globale C058-schaalreferentie. Shipping-boxplaatsingen verwijzen naar dit componentcontract; dezelfde geometrie voedt de webviewer en SolidWorks-proefmacro. OSB 18 krijgt de aparte renderweergave osb-vlokken.</x:v>
+      </x:c>
+      <x:c r="G72" t="str">
+        <x:v>liangyue_ly103_12_candidate;osb_18;ComponentPrimitiveRenderContract;SolidWorksMacroExporter;PortalAssemblyPart.MaterialAppearance</x:v>
+      </x:c>
+      <x:c r="H72" t="str">
+        <x:v>De clip blijft ProvisionalRenderEnvelope. Vrije veerhoek, haken, persribben, radii en exacte contour moeten na fysieke samplemeting worden vervangen; niet voor CAM of productievrijgave. OSB-vlokken zijn presentatie en geen vezel- of sterkteclassificatie.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" t="str">
+        <x:v>CHG-068</x:v>
+      </x:c>
+      <x:c r="B73" s="64" t="n">
+        <x:v>46265</x:v>
+      </x:c>
+      <x:c r="C73" t="str">
+        <x:v>Dylan / Codex</x:v>
+      </x:c>
+      <x:c r="D73" t="str">
+        <x:v>6.0</x:v>
+      </x:c>
+      <x:c r="E73" t="str">
+        <x:v>Kastfamilie app-breed configureerbaar via overerving</x:v>
+      </x:c>
+      <x:c r="F73" t="str">
+        <x:v>De ontbrekende kastfamiliedata is op de juiste overervingslaag vastgelegd. Cabinet levert voortaan het erfbare maatcontract en betonplex 18 als standaard plaatmateriaal aan cabinet, vakjeskast en werkbankkast. Werkbankkast overschrijft alleen de strengere bestaande minimumgrenzen. De backendconfiguratie leest dezelfde contractwaarden, zodat catalogusvalidatie en modelbouw niet uiteenlopen.</x:v>
+      </x:c>
+      <x:c r="G73" t="str">
+        <x:v>PRD-CAB-003;PRD-CAB-004;PRD-WBK-014;cabinet;vakjeskast;werkbankkast;betonplex_18;ProductCatalogApplicationService;PortalConfigurationFactory</x:v>
+      </x:c>
+      <x:c r="H73" t="str">
+        <x:v>Niet alle producten mogen dezelfde maat- of materiaalwaarden erven. Overerving is app-breed, maar uitsluitend binnen een expliciete Basisproduct-ID-keten; ontbrekende data buiten die keten blijft blokkerend.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" t="str">
+        <x:v>CHG-069</x:v>
+      </x:c>
+      <x:c r="B74" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="C74" t="str">
+        <x:v>Dylan / Codex</x:v>
+      </x:c>
+      <x:c r="D74" t="str">
+        <x:v>6.1</x:v>
+      </x:c>
+      <x:c r="E74" t="str">
+        <x:v>Opvouwbare werktafel als voorlopig nieuw product</x:v>
+      </x:c>
+      <x:c r="F74" t="str">
+        <x:v>Nieuw productcontract met betonplex 18 mm, 2400×1180×900 standaardmaat, zes nok-/slotposities, twee tweedelige knikliggers, zes normale AXA-kogellagerscharnierassen, twee interactieve bewegingsassen, dogbones en hergebruikte randafschuining. Productie blijft geblokkeerd tot proefpassing, scharniersample en belastingtest.</x:v>
+      </x:c>
+      <x:c r="G74" t="str">
+        <x:v>opvouwbare_werktafel;PRD-FWT-001..012;PIC-FOLDING-WORKTABLE-*;ggoedkoop_axa_ball_bearing_hinge_rvs_76x76x25;CAT-GOEDKOOP-0000006696;PRI-MATERIAAL-BETONPLEX-18;VAL-FWT-001..004</x:v>
+      </x:c>
+      <x:c r="H74" t="str">
+        <x:v>Foto’s zijn uitsluitend constructiereferentie. Wielen en wielgaten zijn bewust uitgesloten van versie 1.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" t="str">
+        <x:v>CHG-070</x:v>
+      </x:c>
+      <x:c r="B75" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="C75" t="str">
+        <x:v>Dylan / Codex</x:v>
+      </x:c>
+      <x:c r="D75" t="str">
+        <x:v>6.2</x:v>
+      </x:c>
+      <x:c r="E75" t="str">
+        <x:v>Opvouwbare werktafel met dragende framepanelen volgens fotoreferentie</x:v>
+      </x:c>
+      <x:c r="F75" t="str">
+        <x:v>De twee lange pootframes en dunne knikliggers zijn herzien naar twee eindframes en vier brede framevormige vouwpanelen. Alle panelen hebben volledige stijlen tot de vloer, brede boven- en onderregels, vier eindframenokken en twee middennokken. Betonplex krijgt een donkere betonplexweergave en de normale AXA-scharnieren een RVS-presentatierol.</x:v>
+      </x:c>
+      <x:c r="G75" t="str">
+        <x:v>opvouwbare_werktafel;PRD-FWT-002;PRD-FWT-004..006;PRD-FWT-009..010;VAL-FWT-001;betonplex_18;ggoedkoop_axa_ball_bearing_hinge_rvs_76x76x25</x:v>
+      </x:c>
+      <x:c r="H75" t="str">
+        <x:v>Foto's en rode annotaties zijn uitsluitend constructiereferentie. Afmetingen blijven proefstukdata totdat passing, scharniermontage en belasting fysiek zijn gevalideerd.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" t="str">
+        <x:v>CHG-071</x:v>
+      </x:c>
+      <x:c r="B76" t="str">
+        <x:v>2026-09-01</x:v>
+      </x:c>
+      <x:c r="C76" t="str">
+        <x:v>Dylan / Codex</x:v>
+      </x:c>
+      <x:c r="D76" t="str">
+        <x:v>6.3</x:v>
+      </x:c>
+      <x:c r="E76" t="str">
+        <x:v>Verzenden standaard en eerste model automatisch laden</x:v>
+      </x:c>
+      <x:c r="F76" t="str">
+        <x:v>Alle actieve productfamilies krijgen Verzenden als standaard ontvangstwijze. De portal vult catalogusdefaults in en start bij het openen van een configureerbaar product direct de bestaande conceptberekening, zodat prijs, nesting en 3D-model zonder voorafgaande selectie zichtbaar worden.</x:v>
+      </x:c>
+      <x:c r="G76" t="str">
+        <x:v>PIC-*-DELIVERY-020;ReceiptMethod;ProductCatalogApplicationService;PortalHtml</x:v>
+      </x:c>
+      <x:c r="H76" t="str">
+        <x:v>De automatische start gebruikt alleen het bestaande offerte-/renderendpoint en maakt geen order. Geblokkeerde producten blijven hun ontbrekende masterdata tonen.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" t="str">
+        <x:v>CHG-072</x:v>
+      </x:c>
+      <x:c r="B77" t="str">
+        <x:v>2026-09-01</x:v>
+      </x:c>
+      <x:c r="C77" t="str">
+        <x:v>Dylan / Codex</x:v>
+      </x:c>
+      <x:c r="D77" t="str">
+        <x:v>6.4</x:v>
+      </x:c>
+      <x:c r="E77" t="str">
+        <x:v>Opvouwbare werktafel vouwt over de korte zijden</x:v>
+      </x:c>
+      <x:c r="F77" t="str">
+        <x:v>De bestaande vouwrichting is 90 graden gedraaid. De twee lange zijden zijn vaste volledige framepanelen met drie nokken per paneel. Iedere korte zijde bestaat uit twee vloerhoge scharnierende framepanelen met twee nokken per plaatdeel. Zes verticale scharnierassen blijven behouden; het werkblad krijgt veertien bijbehorende doorsteekslots.</x:v>
+      </x:c>
+      <x:c r="G77" t="str">
+        <x:v>opvouwbare_werktafel;PRD-FWT-002;PRD-FWT-004..006;PRD-FWT-009..010;VAL-FWT-001..002;VAL-FWT-004;FoldingWorkbenchEngine;PortalMotionContractService</x:v>
+      </x:c>
+      <x:c r="H77" t="str">
+        <x:v>Foto en portalscreenshot met rode annotaties zijn constructiereferentie. Passing, scharniermontage, stabiliteit en belasting blijven proefstuk- en vrijgavepunten.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" t="str">
+        <x:v>CHG-073</x:v>
+      </x:c>
+      <x:c r="B78" t="str">
+        <x:v>2026-09-01</x:v>
+      </x:c>
+      <x:c r="C78" t="str">
+        <x:v>Dylan / Codex</x:v>
+      </x:c>
+      <x:c r="D78" t="str">
+        <x:v>6.5</x:v>
+      </x:c>
+      <x:c r="E78" t="str">
+        <x:v>Multiplex kopse kanten en driedelige vouwscharnieren</x:v>
+      </x:c>
+      <x:c r="F78" t="str">
+        <x:v>De echte-kleurenweergave toont de gelaagde multiplexkern op alle zichtbare betonplex-kopse kanten. Ieder AXA-vouwscharnier wordt als twee afzonderlijke bladen en één verticale pen opgebouwd. De korte paneelhelften worden rond iedere scharnieras ingekort zodat een 10-mm spleet de voorlopige Ø8-mm renderpen met 1 mm vrije ruimte per zijde opneemt. Interne triangulatielijnen op doorlopende betonplexvlakken worden in de realistische weergave niet getekend.</x:v>
+      </x:c>
+      <x:c r="G78" t="str">
+        <x:v>opvouwbare_werktafel;PRD-FWT-004;PRD-FWT-006;VAL-FWT-001;ggoedkoop_axa_ball_bearing_hinge_rvs_76x76x25;PortalAssembly3DService;PortalHtml</x:v>
+      </x:c>
+      <x:c r="H78" t="str">
+        <x:v>Scharnierpen, bladverdeling en gatenpatroon blijven voorlopige renderdata tot het leverancierssample fysiek is ingemeten; geen CAM- of productievrijgave.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" t="str">
+        <x:v>CHG-074</x:v>
+      </x:c>
+      <x:c r="B79" t="str">
+        <x:v>2026-09-01</x:v>
+      </x:c>
+      <x:c r="C79" t="str">
+        <x:v>Dylan / Codex</x:v>
+      </x:c>
+      <x:c r="D79" t="str">
+        <x:v>6.6</x:v>
+      </x:c>
+      <x:c r="E79" t="str">
+        <x:v>AXA-gatenbeeld en correcte binnenmontage vouwscharnieren</x:v>
+      </x:c>
+      <x:c r="F79" t="str">
+        <x:v>De zes AXA 1KL227676N-scharnieren zijn herzien op de officiële fabrikanttekening: knoop Ø10,8 mm, drie gaten per blad en knoopsegmenten die fysiek bij blad A of blad B horen. Buitenste scharnieren zijn naar de binnenvlakken verplaatst. Ieder scharnier legt nu een expliciete voorlopige SheetHinge-relatie vast tussen precies de twee bedoelde platen en ieder scharnierdeel volgt in de animatie het plaatdeel waarop het is bevestigd.</x:v>
+      </x:c>
+      <x:c r="G79" t="str">
+        <x:v>opvouwbare_werktafel;PRD-FWT-004;PRD-FWT-006;VAL-FWT-001;ggoedkoop_axa_ball_bearing_hinge_rvs_76x76x25;FoldingWorkbenchEngine;PortalAssembly3DService;PortalMotionContractService</x:v>
+      </x:c>
+      <x:c r="H79" t="str">
+        <x:v>AXA publiceert geen bemaatte gatcoördinaten, gat-/verzinkdiameters, penmaat of knoopsegmentlengten. De gekalibreerde gatweergave blijft daarom ProvisionalRenderEnvelope; geen plaat-CAM of productievrijgave tot sample-inmeting en keuze bevestiger voor 18-mm betonplex.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" t="str">
+        <x:v>CHG-075</x:v>
+      </x:c>
+      <x:c r="B80" t="str">
+        <x:v>2026-09-01</x:v>
+      </x:c>
+      <x:c r="C80" t="str">
+        <x:v>Dylan / Codex</x:v>
+      </x:c>
+      <x:c r="D80" t="str">
+        <x:v>6.7</x:v>
+      </x:c>
+      <x:c r="E80" t="str">
+        <x:v>Geïntegreerde voeten in alle onderstelpanelen</x:v>
+      </x:c>
+      <x:c r="F80" t="str">
+        <x:v>De rechte vloerhoge onderranden zijn vervangen door geïntegreerde voeten volgens de geannoteerde fotoreferentie. Ieder vast langspaneel heeft drie voeten onder de linker-, midden- en rechterstijl; ieder kort half vouwpaneel heeft twee voeten onder zijn stijlen. Tussen de voeten ligt de paneelonderrand voorlopig 30 mm hoger. De buitencontour voedt dezelfde 3D-, nesting- en CAM-keten.</x:v>
+      </x:c>
+      <x:c r="G80" t="str">
+        <x:v>opvouwbare_werktafel;PRD-FWT-004;PRD-FWT-010;VAL-FWT-001;FoldingWorkbenchEngine;FoldingWorkbenchMasterDataSettings</x:v>
+      </x:c>
+      <x:c r="H80" t="str">
+        <x:v>Voetbreedte 140 mm en vloervrijloop 30 mm zijn conceptwaarden uit de fotoreconstructie. Definitieve maat en belastbaarheid blijven geblokkeerd tot constructieberekening en fysiek proefstuk.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81">
+      <x:c r="A81" t="str">
+        <x:v>CHG-076</x:v>
+      </x:c>
+      <x:c r="B81" t="str">
+        <x:v>2026-09-01</x:v>
+      </x:c>
+      <x:c r="C81" t="str">
+        <x:v>Dylan / Codex</x:v>
+      </x:c>
+      <x:c r="D81" t="str">
+        <x:v>6.8</x:v>
+      </x:c>
+      <x:c r="E81" t="str">
+        <x:v>Uniforme bladoversteek 80 mm rondom</x:v>
+      </x:c>
+      <x:c r="F81" t="str">
+        <x:v>Het werkblad steekt voortaan conceptueel 80 mm rondom voorbij het onderstel, zoals zichtbaar in de fotoreferentie. Het onderstel wordt centraal afgeleid als bladlengte min 160 mm bij bladbreedte min 160 mm; bij 2400 × 1180 mm is dat 2240 × 1020 mm. Alle zes onderstelpanelen, veertien nokken en bijbehorende werkbladslots volgen dezelfde masterdataparameter, zodat kleinere ondersteldelen en minder bruto plaatoppervlak ontstaan.</x:v>
+      </x:c>
+      <x:c r="G81" t="str">
+        <x:v>opvouwbare_werktafel;PRD-FWT-004;VAL-FWT-001;FoldingWorkbenchEngine;FoldingWorkbenchMasterDataSettings;PortalAssembly3DService</x:v>
+      </x:c>
+      <x:c r="H81" t="str">
+        <x:v>De 80-mm maat is een fotogereconstrueerde conceptwaarde. Definitieve stabiliteit, randbelasting en materiaalbesparing worden na constructieberekening, nestingcontrole en fysiek proefstuk vastgesteld.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82">
+      <x:c r="A82" t="str">
+        <x:v>CHG-077</x:v>
+      </x:c>
+      <x:c r="B82" t="str">
+        <x:v>2026-09-01</x:v>
+      </x:c>
+      <x:c r="C82" t="str">
+        <x:v>Dylan / Codex</x:v>
+      </x:c>
+      <x:c r="D82" t="str">
+        <x:v>6.9</x:v>
+      </x:c>
+      <x:c r="E82" t="str">
+        <x:v>Afzonderlijke offsets lange en korte bladranden</x:v>
+      </x:c>
+      <x:c r="F82" t="str">
+        <x:v>Twee technische invoerparameters toegevoegd. De offset vanaf korte bladranden bepaalt de onderstellengte; de offset vanaf lange bladranden bepaalt de ondersteldiepte. Beide starten op 80 mm.</x:v>
+      </x:c>
+      <x:c r="G82" t="str">
+        <x:v>opvouwbare_werktafel;PRD-FWT-004;PIC-FOLDING-WORKTABLE-020;PIC-FOLDING-WORKTABLE-030;FoldingWorkbenchEngine;FoldingWorkbenchMasterDataSettings;PortalConfigurationFactory</x:v>
+      </x:c>
+      <x:c r="H82" t="str">
+        <x:v>Grenzen zijn voorlopige conceptgrenzen en blijven afhankelijk van stijfheidscontrole en gefreesd proefstuk.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
@@ -8038,7 +8463,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70ff60274a6d48c3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc025e567b3124133"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8222,7 +8647,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R770856589aaa4e92"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb911ad5226347f4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8583,16 +9008,16 @@
         <x:v>Materiaal</x:v>
       </x:c>
       <x:c r="E8" s="6" t="str">
-        <x:v>Algemeen</x:v>
+        <x:v>Houtachtige platen</x:v>
       </x:c>
       <x:c r="F8" s="6" t="str">
-        <x:v>Betonplex 18mm</x:v>
+        <x:v>Mixed hardwood betonplex glad bruin CE+ 18×2500×1250 mm</x:v>
       </x:c>
       <x:c r="G8" s="6" t="str">
         <x:v>plaat</x:v>
       </x:c>
       <x:c r="H8" s="405" t="n">
-        <x:v>33</x:v>
+        <x:v>46.56</x:v>
       </x:c>
       <x:c r="I8" s="6" t="str">
         <x:v>EUR</x:v>
@@ -8600,15 +9025,29 @@
       <x:c r="J8" s="406" t="n">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="K8" s="6"/>
-      <x:c r="L8" s="6"/>
-      <x:c r="M8" s="6"/>
-      <x:c r="N8" s="6"/>
-      <x:c r="O8" s="6"/>
-      <x:c r="P8" s="6"/>
-      <x:c r="Q8" s="65"/>
+      <x:c r="K8" s="6" t="str">
+        <x:v>SUP-GOEDKOOP</x:v>
+      </x:c>
+      <x:c r="L8" s="6" t="str">
+        <x:v>0000008204</x:v>
+      </x:c>
+      <x:c r="M8" s="6" t="str">
+        <x:v>Mixed hardwood CE+</x:v>
+      </x:c>
+      <x:c r="N8" s="6" t="str">
+        <x:v>2500×1250×18 mm</x:v>
+      </x:c>
+      <x:c r="O8" s="6" t="str">
+        <x:v>Mixed hardwood betonplex glad bruin</x:v>
+      </x:c>
+      <x:c r="P8" s="6" t="str">
+        <x:v>https://ggoedkoop.nl/mixed-hardwood-18x2500x1250-mm-betonplex-glad-bruin-ce-0000008204</x:v>
+      </x:c>
+      <x:c r="Q8" s="65" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
       <x:c r="R8" s="6" t="str">
-        <x:v>Te controleren</x:v>
+        <x:v>Leveranciersprijs</x:v>
       </x:c>
       <x:c r="S8" s="6"/>
       <x:c r="T8" s="6"/>
@@ -8617,12 +9056,21 @@
         <x:v>Geen afbeelding</x:v>
       </x:c>
       <x:c r="W8" s="6" t="str">
-        <x:v>Prijs per volledige plaat excl. btw</x:v>
+        <x:v>Exact G Goedkoop-artikel; productmaximum 2400×1180 mm laat minimaal 50 mm respectievelijk 35 mm plaatrand per zijde over.</x:v>
       </x:c>
       <x:c r="X8" s="6" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="Y8" s="6"/>
+      <x:c r="AA8" t="n">
+        <x:v>2500</x:v>
+      </x:c>
+      <x:c r="AB8" t="n">
+        <x:v>1250</x:v>
+      </x:c>
+      <x:c r="AC8" t="n">
+        <x:v>18</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="6" t="str">
@@ -13044,6 +13492,87 @@
       <x:c r="AA70"/>
       <x:c r="AB70"/>
       <x:c r="AC70"/>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" t="str">
+        <x:v>CAT-GOEDKOOP-0000006696</x:v>
+      </x:c>
+      <x:c r="B71" t="str">
+        <x:v>Component</x:v>
+      </x:c>
+      <x:c r="C71" t="str">
+        <x:v>ggoedkoop_axa_ball_bearing_hinge_rvs_76x76x25</x:v>
+      </x:c>
+      <x:c r="D71" t="str">
+        <x:v>Beslag</x:v>
+      </x:c>
+      <x:c r="E71" t="str">
+        <x:v>Scharnieren</x:v>
+      </x:c>
+      <x:c r="F71" t="str">
+        <x:v>AXA kogellagerscharnier RVS 76×76×2,5 mm</x:v>
+      </x:c>
+      <x:c r="G71" t="str">
+        <x:v>st</x:v>
+      </x:c>
+      <x:c r="H71" t="n">
+        <x:v>4.64</x:v>
+      </x:c>
+      <x:c r="I71" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="J71" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="K71" t="str">
+        <x:v>SUP-GOEDKOOP</x:v>
+      </x:c>
+      <x:c r="L71" t="str">
+        <x:v>0000006696</x:v>
+      </x:c>
+      <x:c r="M71" t="str">
+        <x:v>AXA 1KL227676N</x:v>
+      </x:c>
+      <x:c r="N71" t="str">
+        <x:v>76×76×2,5 mm</x:v>
+      </x:c>
+      <x:c r="O71" t="str">
+        <x:v>RVS; leveranciersbenaming</x:v>
+      </x:c>
+      <x:c r="P71" t="str">
+        <x:v>https://ggoedkoop.nl/ijzerwaren/scharnieren/kogelscharnieren</x:v>
+      </x:c>
+      <x:c r="Q71" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="R71" t="str">
+        <x:v>Leveranciersprijs</x:v>
+      </x:c>
+      <x:c r="S71"/>
+      <x:c r="T71"/>
+      <x:c r="U71"/>
+      <x:c r="V71" t="str">
+        <x:v>Geen afbeelding</x:v>
+      </x:c>
+      <x:c r="W71" t="str">
+        <x:v>Voorlopig zes normale bladscharnieren, één per verticale as. Gatenpatroon, bevestigers, knokkelmaat en belastbaarheid na sample-inmeting; fysieke proef bepaalt of twee per as nodig zijn.</x:v>
+      </x:c>
+      <x:c r="X71" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Y71"/>
+      <x:c r="Z71" t="str">
+        <x:v>opvouwbare_werktafel</x:v>
+      </x:c>
+      <x:c r="AA71" t="n">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="AB71" t="n">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="AC71" t="n">
+        <x:v>2.5</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -13064,10 +13593,10 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ba7b07cd5334e9b"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71e1e392b5724cde"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ad53a33ab034f44"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f9fcd8038e04850"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Recdb3792cf904ac1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0941f93b1c8a4c35"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13637,8 +14166,8 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re17c637c951740e1"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2bfa981d0b75433a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f7eaebdb16343e0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf702a8f9d7bf4cc1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14416,7 +14945,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re145dcbaf1944109"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac1a61ecff5449f3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15190,8 +15719,8 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5006c8ae6c24f98"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92cba9a3061e4bae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R818ac414c7dd4fa9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ef66754eba94b22"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19896,7 +20425,9 @@
         <x:v>select</x:v>
       </x:c>
       <x:c r="I87" t="str"/>
-      <x:c r="J87" t="str"/>
+      <x:c r="J87" t="str">
+        <x:v>verzenden</x:v>
+      </x:c>
       <x:c r="K87" t="str"/>
       <x:c r="L87" t="str"/>
       <x:c r="M87" t="str"/>
@@ -20006,7 +20537,9 @@
         <x:v>select</x:v>
       </x:c>
       <x:c r="I89" t="str"/>
-      <x:c r="J89" t="str"/>
+      <x:c r="J89" t="str">
+        <x:v>verzenden</x:v>
+      </x:c>
       <x:c r="K89" t="str"/>
       <x:c r="L89" t="str"/>
       <x:c r="M89" t="str"/>
@@ -20116,7 +20649,9 @@
         <x:v>select</x:v>
       </x:c>
       <x:c r="I91" t="str"/>
-      <x:c r="J91" t="str"/>
+      <x:c r="J91" t="str">
+        <x:v>verzenden</x:v>
+      </x:c>
       <x:c r="K91" t="str"/>
       <x:c r="L91" t="str"/>
       <x:c r="M91" t="str"/>
@@ -20226,7 +20761,9 @@
         <x:v>select</x:v>
       </x:c>
       <x:c r="I93" t="str"/>
-      <x:c r="J93" t="str"/>
+      <x:c r="J93" t="str">
+        <x:v>verzenden</x:v>
+      </x:c>
       <x:c r="K93" t="str"/>
       <x:c r="L93" t="str"/>
       <x:c r="M93" t="str"/>
@@ -20336,7 +20873,9 @@
         <x:v>select</x:v>
       </x:c>
       <x:c r="I95" t="str"/>
-      <x:c r="J95" t="str"/>
+      <x:c r="J95" t="str">
+        <x:v>verzenden</x:v>
+      </x:c>
       <x:c r="K95" t="str"/>
       <x:c r="L95" t="str"/>
       <x:c r="M95" t="str"/>
@@ -20446,7 +20985,9 @@
         <x:v>select</x:v>
       </x:c>
       <x:c r="I97" t="str"/>
-      <x:c r="J97" t="str"/>
+      <x:c r="J97" t="str">
+        <x:v>verzenden</x:v>
+      </x:c>
       <x:c r="K97" t="str"/>
       <x:c r="L97" t="str"/>
       <x:c r="M97" t="str"/>
@@ -20471,6 +21012,296 @@
         <x:v>Afhalen is toegestaan; verzendkosten blijven open totdat logistieke brondata en rekenlogica compleet zijn.</x:v>
       </x:c>
       <x:c r="V97" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98">
+      <x:c r="A98" t="str">
+        <x:v>PIC-FOLDING-WORKTABLE-010</x:v>
+      </x:c>
+      <x:c r="B98" t="str">
+        <x:v>opvouwbare_werktafel</x:v>
+      </x:c>
+      <x:c r="C98" t="str">
+        <x:v>folding-worktable</x:v>
+      </x:c>
+      <x:c r="D98" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E98" t="str">
+        <x:v>enableOutsideEdgeChamfer</x:v>
+      </x:c>
+      <x:c r="F98" t="str">
+        <x:v>EnableOutsideEdgeChamfer</x:v>
+      </x:c>
+      <x:c r="G98" t="str">
+        <x:v>Buitenranden afschuinen</x:v>
+      </x:c>
+      <x:c r="H98" t="str">
+        <x:v>checkbox</x:v>
+      </x:c>
+      <x:c r="I98"/>
+      <x:c r="J98" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="K98"/>
+      <x:c r="L98"/>
+      <x:c r="M98"/>
+      <x:c r="N98"/>
+      <x:c r="O98"/>
+      <x:c r="P98"/>
+      <x:c r="Q98" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="R98" t="str">
+        <x:v>Voorlopig</x:v>
+      </x:c>
+      <x:c r="S98" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="T98" t="str">
+        <x:v>PRD-FWT-008; bestaande generieke V-freeslogica</x:v>
+      </x:c>
+      <x:c r="U98" t="str">
+        <x:v>Standaard actief voor het concept; afschuining blijft proefstuk en wordt alleen door backend-CAM uitgevoerd.</x:v>
+      </x:c>
+      <x:c r="V98" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99">
+      <x:c r="A99" t="str">
+        <x:v>PIC-FOLDING-WORKTABLE-DELIVERY-010</x:v>
+      </x:c>
+      <x:c r="B99" t="str">
+        <x:v>opvouwbare_werktafel</x:v>
+      </x:c>
+      <x:c r="C99" t="str">
+        <x:v>levering</x:v>
+      </x:c>
+      <x:c r="D99" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E99" t="str">
+        <x:v>deliveryForm</x:v>
+      </x:c>
+      <x:c r="F99" t="str">
+        <x:v>DeliveryForm</x:v>
+      </x:c>
+      <x:c r="G99" t="str">
+        <x:v>Levervorm</x:v>
+      </x:c>
+      <x:c r="H99" t="str">
+        <x:v>select</x:v>
+      </x:c>
+      <x:c r="I99"/>
+      <x:c r="J99" t="str">
+        <x:v>bouwpakket</x:v>
+      </x:c>
+      <x:c r="K99"/>
+      <x:c r="L99"/>
+      <x:c r="M99"/>
+      <x:c r="N99"/>
+      <x:c r="O99" t="str">
+        <x:v>bouwpakket|Bouwpakket;gemonteerd|Gemonteerd</x:v>
+      </x:c>
+      <x:c r="P99"/>
+      <x:c r="Q99" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="R99" t="str">
+        <x:v>Goedgekeurd</x:v>
+      </x:c>
+      <x:c r="S99" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="T99" t="str">
+        <x:v>Pilotbesluit Dylan 2026-08-30</x:v>
+      </x:c>
+      <x:c r="U99" t="str">
+        <x:v>Het uitneembare blad en vlak opvouwbare onderstel maken bouwpakket de standaard.</x:v>
+      </x:c>
+      <x:c r="V99" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100">
+      <x:c r="A100" t="str">
+        <x:v>PIC-FOLDING-WORKTABLE-DELIVERY-020</x:v>
+      </x:c>
+      <x:c r="B100" t="str">
+        <x:v>opvouwbare_werktafel</x:v>
+      </x:c>
+      <x:c r="C100" t="str">
+        <x:v>levering</x:v>
+      </x:c>
+      <x:c r="D100" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E100" t="str">
+        <x:v>receiptMethod</x:v>
+      </x:c>
+      <x:c r="F100" t="str">
+        <x:v>ReceiptMethod</x:v>
+      </x:c>
+      <x:c r="G100" t="str">
+        <x:v>Ontvangst</x:v>
+      </x:c>
+      <x:c r="H100" t="str">
+        <x:v>select</x:v>
+      </x:c>
+      <x:c r="I100"/>
+      <x:c r="J100" t="str">
+        <x:v>verzenden</x:v>
+      </x:c>
+      <x:c r="K100"/>
+      <x:c r="L100"/>
+      <x:c r="M100"/>
+      <x:c r="N100"/>
+      <x:c r="O100" t="str">
+        <x:v>verzenden|Verzenden;afhalen|Afhalen</x:v>
+      </x:c>
+      <x:c r="P100"/>
+      <x:c r="Q100" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="R100" t="str">
+        <x:v>Goedgekeurd</x:v>
+      </x:c>
+      <x:c r="S100" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="T100" t="str">
+        <x:v>Pilotbesluit Dylan 2026-08-30</x:v>
+      </x:c>
+      <x:c r="U100" t="str">
+        <x:v>Verzendkosten blijven open totdat verpakkingsmaten, gewicht en vervoerdersregels zijn gevalideerd.</x:v>
+      </x:c>
+      <x:c r="V100" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101">
+      <x:c r="A101" t="str">
+        <x:v>PIC-FOLDING-WORKTABLE-020</x:v>
+      </x:c>
+      <x:c r="B101" t="str">
+        <x:v>opvouwbare_werktafel</x:v>
+      </x:c>
+      <x:c r="C101" t="str">
+        <x:v>folding-worktable</x:v>
+      </x:c>
+      <x:c r="D101" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E101" t="str">
+        <x:v>underframeInsetLongEdgeMm</x:v>
+      </x:c>
+      <x:c r="F101" t="str">
+        <x:v>FoldingWorkbenchUnderframeInsetLongEdgeMm</x:v>
+      </x:c>
+      <x:c r="G101" t="str">
+        <x:v>Offset onderstel vanaf lange bladrand</x:v>
+      </x:c>
+      <x:c r="H101" t="str">
+        <x:v>number</x:v>
+      </x:c>
+      <x:c r="I101" t="str"/>
+      <x:c r="J101" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="K101" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="L101" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="M101" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N101" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="O101" t="str"/>
+      <x:c r="P101" t="str"/>
+      <x:c r="Q101" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="R101" t="str">
+        <x:v>Voorlopig</x:v>
+      </x:c>
+      <x:c r="S101" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="T101" t="str">
+        <x:v>PRD-FWT-004; fotoreferentie; gebruikersbesluit 2026-09-01</x:v>
+      </x:c>
+      <x:c r="U101" t="str">
+        <x:v>Afstand per zijde vanaf beide lange bladranden; bepaalt de ondersteldiepte.</x:v>
+      </x:c>
+      <x:c r="V101" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102">
+      <x:c r="A102" t="str">
+        <x:v>PIC-FOLDING-WORKTABLE-030</x:v>
+      </x:c>
+      <x:c r="B102" t="str">
+        <x:v>opvouwbare_werktafel</x:v>
+      </x:c>
+      <x:c r="C102" t="str">
+        <x:v>folding-worktable</x:v>
+      </x:c>
+      <x:c r="D102" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="E102" t="str">
+        <x:v>underframeInsetShortEdgeMm</x:v>
+      </x:c>
+      <x:c r="F102" t="str">
+        <x:v>FoldingWorkbenchUnderframeInsetShortEdgeMm</x:v>
+      </x:c>
+      <x:c r="G102" t="str">
+        <x:v>Offset onderstel vanaf korte bladrand</x:v>
+      </x:c>
+      <x:c r="H102" t="str">
+        <x:v>number</x:v>
+      </x:c>
+      <x:c r="I102" t="str"/>
+      <x:c r="J102" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="K102" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="L102" t="n">
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="M102" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N102" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="O102" t="str"/>
+      <x:c r="P102" t="str"/>
+      <x:c r="Q102" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="R102" t="str">
+        <x:v>Voorlopig</x:v>
+      </x:c>
+      <x:c r="S102" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="T102" t="str">
+        <x:v>PRD-FWT-004; fotoreferentie; gebruikersbesluit 2026-09-01</x:v>
+      </x:c>
+      <x:c r="U102" t="str">
+        <x:v>Afstand per zijde vanaf beide korte bladranden; bepaalt de onderstellengte.</x:v>
+      </x:c>
+      <x:c r="V102" t="str">
         <x:v>Ja</x:v>
       </x:c>
     </x:row>
@@ -20481,7 +21312,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0bf4d0776061411e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8c8cab255a9461f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20765,7 +21596,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f526d49a2814e99"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R383151f839584de6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20962,7 +21793,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a7d2e6935d845c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77dca89303334729"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22023,6 +22854,70 @@
         <x:v>Ontbreekt</x:v>
       </x:c>
     </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
+        <x:v>opvouwbare_werktafel</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>Opvouwbare werktafel</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
+        <x:v>werkbank</x:v>
+      </x:c>
+      <x:c r="D19"/>
+      <x:c r="E19" t="n">
+        <x:v>2400</x:v>
+      </x:c>
+      <x:c r="F19" t="n">
+        <x:v>1180</x:v>
+      </x:c>
+      <x:c r="G19" t="n">
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="H19" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I19" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J19" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K19" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="L19" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="M19" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="N19" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="O19" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="P19" t="str">
+        <x:v>Proefstuk</x:v>
+      </x:c>
+      <x:c r="Q19" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="R19" t="str">
+        <x:v>n.v.t.</x:v>
+      </x:c>
+      <x:c r="S19" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T19"/>
+      <x:c r="U19"/>
+      <x:c r="V19"/>
+      <x:c r="W19"/>
+      <x:c r="X19" t="str">
+        <x:v>Ontbreekt</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:R1"/>
@@ -22057,7 +22952,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1131305f1eb4794"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62e0227324714c4f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22294,7 +23189,7 @@
       <x:c r="AD6" s="6"/>
       <x:c r="AE6" s="6"/>
       <x:c r="AF6" s="6" t="str">
-        <x:v>standaard</x:v>
+        <x:v>osb-vlokken</x:v>
       </x:c>
       <x:c r="AG6"/>
     </x:row>
@@ -22416,9 +23311,11 @@
       <x:c r="AD8" s="6"/>
       <x:c r="AE8" s="6"/>
       <x:c r="AF8" s="6" t="str">
-        <x:v>standaard</x:v>
-      </x:c>
-      <x:c r="AG8"/>
+        <x:v>betonplex-donker</x:v>
+      </x:c>
+      <x:c r="AG8" t="str">
+        <x:v>Betonplex 18 mm</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="14" t="str">
@@ -23530,9 +24427,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf172f079644e4307"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31c5c9a7a7234f8a"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71d596107307450f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc0653b956404654"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25146,10 +26043,18 @@
       <x:c r="AN24" s="485"/>
       <x:c r="AO24" s="6"/>
       <x:c r="AP24" s="6"/>
-      <x:c r="AQ24" s="6"/>
-      <x:c r="AR24" s="6"/>
-      <x:c r="AS24" s="6"/>
-      <x:c r="AT24" s="6"/>
+      <x:c r="AQ24" s="6" t="str">
+        <x:v>ProvisionalRenderEnvelope</x:v>
+      </x:c>
+      <x:c r="AR24" s="6" t="str">
+        <x:v>Liangyue LY103-12 leveranciersfoto; globale C058-schaalreferentie 63×71×35 mm en plaatdikte 1,5 mm; docs/producten/shipping-box-bronnen-en-proefstuk.md</x:v>
+      </x:c>
+      <x:c r="AS24" s="6" t="str">
+        <x:v>Vrije veerhoek, omgezette haken, persribben, lokale radii en exacte armcontour fysiek inmeten; uitsluitend render en SolidWorks-proefmacro, niet voor CAM of productievrijgave</x:v>
+      </x:c>
+      <x:c r="AT24" s="6" t="str">
+        <x:v>{"version":1,"primitives":[{"id":"arm-horizontal","shape":"box","role":"black-hardware","x":0,"y":0.75,"z":31.5,"sizeX":35,"sizeY":1.5,"sizeZ":63},{"id":"arm-vertical","shape":"box","role":"black-hardware","x":0,"y":35.5,"z":0.75,"sizeX":35,"sizeY":71,"sizeZ":1.5},{"id":"spring-bridge","shape":"box","role":"black-hardware","x":0,"y":6,"z":6,"sizeX":35,"sizeY":16,"sizeZ":3,"rotationX":45},{"id":"return-horizontal","shape":"box","role":"black-hardware","x":0,"y":4.5,"z":60,"sizeX":35,"sizeY":9,"sizeZ":1.5},{"id":"return-vertical","shape":"box","role":"black-hardware","x":0,"y":68,"z":4.5,"sizeX":35,"sizeY":1.5,"sizeZ":9}]}</x:v>
+      </x:c>
       <x:c r="AU24" s="495"/>
       <x:c r="AV24" s="6"/>
       <x:c r="AW24" s="496"/>
@@ -29541,6 +30446,88 @@
       <x:c r="AW80"/>
       <x:c r="AX80"/>
     </x:row>
+    <x:row r="81">
+      <x:c r="A81" t="str">
+        <x:v>ggoedkoop_axa_ball_bearing_hinge_rvs_76x76x25</x:v>
+      </x:c>
+      <x:c r="B81" t="str">
+        <x:v>Scharnier</x:v>
+      </x:c>
+      <x:c r="C81" t="str">
+        <x:v>AXA kogellagerscharnier RVS 76×76×2,5 mm</x:v>
+      </x:c>
+      <x:c r="D81" t="str">
+        <x:v>G Goedkoop 0000006696 / AXA 1KL227676N</x:v>
+      </x:c>
+      <x:c r="E81" t="str">
+        <x:v>76×76×2,5 mm</x:v>
+      </x:c>
+      <x:c r="F81" t="str">
+        <x:v>76×76×2,5 mm</x:v>
+      </x:c>
+      <x:c r="G81" t="str">
+        <x:v>AXA 1KL227676N, open maat 76×76 mm, bladdikte 2,5 mm, rondhoek R10 en knoop Ø10,8 mm. Fabrikanttekening toont exact drie verzonken gaten per blad (zes totaal) en afwisselende knoopsegmenten die bij blad A en blad B horen. Het renderpatroon gebruikt uit de fabrikanttekening gekalibreerde, nog niet bemaat bevestigde harten op circa 12 mm van de buitenrand en circa 26 mm verticale steek.</x:v>
+      </x:c>
+      <x:c r="H81" t="str">
+        <x:v>Eén scharnier per verticale as; buitenste assen op de binnenvlakken van vast langspaneel en kort vouwpaneel, middenas op de binnenvlakken van beide korte paneelhelften.</x:v>
+      </x:c>
+      <x:c r="I81" t="str">
+        <x:v>AXA bevestigt 76×76×2,5 mm, R10, knoop Ø10,8 mm, drie gaten per blad en aanbevolen 4,0×40-mm deurschroeven. De publicatie bevat geen bemaatte gatcoördinaten, gatdiameter, verzinking, penmaat of knoopsegmentlengten. Daardoor blijft de render voorlopig en zijn plaatboringen/CAM en tafelbevestigers geblokkeerd tot een sample is ingemeten.</x:v>
+      </x:c>
+      <x:c r="J81" t="str">
+        <x:v>Leveranciersdata</x:v>
+      </x:c>
+      <x:c r="K81" t="str">
+        <x:v>https://ggoedkoop.nl/ijzerwaren/scharnieren/kogelscharnieren</x:v>
+      </x:c>
+      <x:c r="L81"/>
+      <x:c r="M81"/>
+      <x:c r="N81"/>
+      <x:c r="O81"/>
+      <x:c r="P81"/>
+      <x:c r="Q81"/>
+      <x:c r="R81"/>
+      <x:c r="S81"/>
+      <x:c r="T81"/>
+      <x:c r="U81"/>
+      <x:c r="V81"/>
+      <x:c r="W81"/>
+      <x:c r="X81"/>
+      <x:c r="Y81"/>
+      <x:c r="Z81"/>
+      <x:c r="AA81"/>
+      <x:c r="AB81"/>
+      <x:c r="AC81"/>
+      <x:c r="AD81"/>
+      <x:c r="AE81"/>
+      <x:c r="AF81"/>
+      <x:c r="AG81"/>
+      <x:c r="AH81"/>
+      <x:c r="AI81"/>
+      <x:c r="AJ81"/>
+      <x:c r="AK81"/>
+      <x:c r="AL81"/>
+      <x:c r="AM81"/>
+      <x:c r="AN81"/>
+      <x:c r="AO81"/>
+      <x:c r="AP81"/>
+      <x:c r="AQ81" t="str">
+        <x:v>ProvisionalRenderEnvelope</x:v>
+      </x:c>
+      <x:c r="AR81" t="str">
+        <x:v>AXA product 1KL2-27-67/6BLACK met gedeelde technische tekening 1KL227676: https://axahomesecurity.com/producten/scharnier-kogellager-2/ en https://axahomesecurity.com/wp-content/uploads/sites/2/2024/08/tekening-1kl227676-kogellagerscharnier_E0008442.jpg; gekozen finish/artikel G Goedkoop 0000006696 / AXA 1KL227676N</x:v>
+      </x:c>
+      <x:c r="AS81" t="str">
+        <x:v>Exact bemaatte gatcoördinaten, gatdiameter en verzinkgeometrie; exacte penmaat; exacte lengten van de knoopsegmenten; definitieve bevestiger voor 18-mm betonplex; uitsluitend render, niet voor CAM of productievrijgave</x:v>
+      </x:c>
+      <x:c r="AT81" t="str">
+        <x:v>{"version":1,"primitives":[{"id":"blad-a-plaat","partId":"blad-a","shape":"box","role":"stainless-hardware","x":21.7,"y":0,"z":0,"sizeX":32.6,"sizeY":76,"sizeZ":2.5,"holes":[{"id":"blad-a-gat-onder","x":26,"y":-26,"z":0,"diameter":4,"depth":2.5,"plane":"z"},{"id":"blad-a-gat-midden","x":26,"y":0,"z":0,"diameter":4,"depth":2.5,"plane":"z"},{"id":"blad-a-gat-boven","x":26,"y":26,"z":0,"diameter":4,"depth":2.5,"plane":"z"}]},{"id":"blad-a-knokkel-onder","partId":"blad-a","shape":"cylinder","role":"stainless-hardware","x":0,"y":-28.5,"z":0,"sizeX":10.8,"sizeY":19,"sizeZ":10.8,"radiusTop":5.4,"radiusBottom":5.4,"segments":32},{"id":"blad-a-knokkel-boven","partId":"blad-a","shape":"cylinder","role":"stainless-hardware","x":0,"y":28.5,"z":0,"sizeX":10.8,"sizeY":19,"sizeZ":10.8,"radiusTop":5.4,"radiusBottom":5.4,"segments":32},{"id":"blad-b-plaat","partId":"blad-b","shape":"box","role":"stainless-hardware","x":-21.7,"y":0,"z":0,"sizeX":32.6,"sizeY":76,"sizeZ":2.5,"holes":[{"id":"blad-b-gat-onder","x":-26,"y":-26,"z":0,"diameter":4,"depth":2.5,"plane":"z"},{"id":"blad-b-gat-midden","x":-26,"y":0,"z":0,"diameter":4,"depth":2.5,"plane":"z"},{"id":"blad-b-gat-boven","x":-26,"y":26,"z":0,"diameter":4,"depth":2.5,"plane":"z"}]},{"id":"blad-b-knokkel-midden","partId":"blad-b","shape":"cylinder","role":"stainless-hardware","x":0,"y":0,"z":0,"sizeX":10.8,"sizeY":38,"sizeZ":10.8,"radiusTop":5.4,"radiusBottom":5.4,"segments":32},{"id":"pen","partId":"pen","shape":"cylinder","role":"hinge-pin","x":0,"y":0,"z":0,"sizeX":4,"sizeY":76,"sizeZ":4,"radiusTop":2,"radiusBottom":2,"segments":24}]}</x:v>
+      </x:c>
+      <x:c r="AU81"/>
+      <x:c r="AV81"/>
+      <x:c r="AW81"/>
+      <x:c r="AX81"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:K1"/>
@@ -29559,7 +30546,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra22212b4654b430d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71fb0505eca74aec"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29971,9 +30958,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4daeb8da47ea4439"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e0512d0a5c84807"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbffb156467414b78"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26c45fa0c31e4bf1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30239,7 +31226,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38f2a7931d934d3e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra96ca833a0724dd0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35467,21 +36454,49 @@
       <x:c r="V113" s="456"/>
     </x:row>
     <x:row r="114">
-      <x:c r="A114" s="454"/>
-      <x:c r="B114" s="455"/>
-      <x:c r="C114" s="455"/>
-      <x:c r="D114" s="461"/>
-      <x:c r="E114" s="455"/>
-      <x:c r="F114" s="455"/>
-      <x:c r="G114" s="455"/>
-      <x:c r="H114" s="455"/>
-      <x:c r="I114" s="455"/>
-      <x:c r="J114" s="464"/>
-      <x:c r="K114" s="464"/>
-      <x:c r="L114" s="464"/>
-      <x:c r="M114" s="464"/>
-      <x:c r="N114" s="455"/>
-      <x:c r="O114" s="455"/>
+      <x:c r="A114" s="454" t="str">
+        <x:v>PRD-SBX-010</x:v>
+      </x:c>
+      <x:c r="B114" s="455" t="str">
+        <x:v>shipping_box</x:v>
+      </x:c>
+      <x:c r="C114" s="455" t="str">
+        <x:v>Parameters</x:v>
+      </x:c>
+      <x:c r="D114" s="461" t="str">
+        <x:v>klantconfigurator; dynamische plaatpassing per paneel</x:v>
+      </x:c>
+      <x:c r="E114" s="455" t="str">
+        <x:v>Parametercontract</x:v>
+      </x:c>
+      <x:c r="F114" s="455" t="str">
+        <x:v>Materiaal</x:v>
+      </x:c>
+      <x:c r="G114" s="455" t="str"/>
+      <x:c r="H114" s="455" t="str">
+        <x:v>osb_18</x:v>
+      </x:c>
+      <x:c r="I114" s="455" t="str">
+        <x:v>200..2364;200..2364;200..2400</x:v>
+      </x:c>
+      <x:c r="J114" s="464" t="str">
+        <x:v>mm/mm/mm</x:v>
+      </x:c>
+      <x:c r="K114" s="464" t="str">
+        <x:v>Binnenbreedte en binnendiepte gebruiken maximaal 2440 - 40 - 2 x 18 mm. Binnenhoogte mag bij doorlopende sponning tot 2440 - 40 mm. Iedere gegenereerde bodem/deksel, zijwand en kopwand moet afzonderlijk, met 90 graden rotatie toegestaan, passen uit de bruikbare plaatmaat 2400 x 1180 mm; het aantal platen volgt uit nesting.</x:v>
+      </x:c>
+      <x:c r="L114" s="464" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="M114" s="464" t="str">
+        <x:v>Voorlopig</x:v>
+      </x:c>
+      <x:c r="N114" s="455" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="O114" s="455" t="str">
+        <x:v>Gebruikersbesluit 2026-08-30; osb_18 handelsmaat en dikte uit Materialen; PRD-SBX-011; ShippingBoxEngine</x:v>
+      </x:c>
       <x:c r="P114" s="455"/>
       <x:c r="Q114" s="455"/>
       <x:c r="R114" s="455"/>
@@ -35491,21 +36506,49 @@
       <x:c r="V114" s="456"/>
     </x:row>
     <x:row r="115">
-      <x:c r="A115" s="454"/>
-      <x:c r="B115" s="455"/>
-      <x:c r="C115" s="455"/>
-      <x:c r="D115" s="461"/>
-      <x:c r="E115" s="455"/>
-      <x:c r="F115" s="455"/>
-      <x:c r="G115" s="455"/>
-      <x:c r="H115" s="455"/>
-      <x:c r="I115" s="455"/>
-      <x:c r="J115" s="464"/>
-      <x:c r="K115" s="464"/>
-      <x:c r="L115" s="464"/>
-      <x:c r="M115" s="464"/>
-      <x:c r="N115" s="455"/>
-      <x:c r="O115" s="455"/>
+      <x:c r="A115" s="454" t="str">
+        <x:v>PRD-SBX-011</x:v>
+      </x:c>
+      <x:c r="B115" s="455" t="str">
+        <x:v>shipping_box</x:v>
+      </x:c>
+      <x:c r="C115" s="455" t="str">
+        <x:v>CNC</x:v>
+      </x:c>
+      <x:c r="D115" s="461" t="str">
+        <x:v>handelsplaat; nesting en paneelpassing</x:v>
+      </x:c>
+      <x:c r="E115" s="455" t="str">
+        <x:v>Plaatmarge</x:v>
+      </x:c>
+      <x:c r="F115" s="455" t="str">
+        <x:v>Materiaal</x:v>
+      </x:c>
+      <x:c r="G115" s="455" t="str"/>
+      <x:c r="H115" s="455" t="str">
+        <x:v>osb_18</x:v>
+      </x:c>
+      <x:c r="I115" s="455" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="J115" s="464" t="str">
+        <x:v>mm totale reductie per plaatrichting</x:v>
+      </x:c>
+      <x:c r="K115" s="464" t="str">
+        <x:v>Van de nominale plaatlengte en -breedte wordt elk 40 mm afgetrokken. Dit vertegenwoordigt 20 mm bruikbare randmarge per zijde voor CNC en opspanning.</x:v>
+      </x:c>
+      <x:c r="L115" s="464" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="M115" s="464" t="str">
+        <x:v>Voorlopig</x:v>
+      </x:c>
+      <x:c r="N115" s="455" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="O115" s="455" t="str">
+        <x:v>Gebruikersbesluit 2026-08-30</x:v>
+      </x:c>
       <x:c r="P115" s="455"/>
       <x:c r="Q115" s="455"/>
       <x:c r="R115" s="455"/>
@@ -35515,21 +36558,47 @@
       <x:c r="V115" s="456"/>
     </x:row>
     <x:row r="116">
-      <x:c r="A116" s="454"/>
-      <x:c r="B116" s="455"/>
-      <x:c r="C116" s="455"/>
-      <x:c r="D116" s="461"/>
-      <x:c r="E116" s="455"/>
-      <x:c r="F116" s="455"/>
+      <x:c r="A116" s="454" t="str">
+        <x:v>PRD-CAB-003</x:v>
+      </x:c>
+      <x:c r="B116" s="455" t="str">
+        <x:v>cabinet</x:v>
+      </x:c>
+      <x:c r="C116" s="455" t="str">
+        <x:v>Parameters</x:v>
+      </x:c>
+      <x:c r="D116" s="461" t="str">
+        <x:v>klantconfigurator</x:v>
+      </x:c>
+      <x:c r="E116" s="455" t="str">
+        <x:v>Parametercontract</x:v>
+      </x:c>
+      <x:c r="F116" s="455" t="str">
+        <x:v>Geen</x:v>
+      </x:c>
       <x:c r="G116" s="455"/>
       <x:c r="H116" s="455"/>
-      <x:c r="I116" s="455"/>
-      <x:c r="J116" s="464"/>
-      <x:c r="K116" s="464"/>
-      <x:c r="L116" s="464"/>
-      <x:c r="M116" s="464"/>
-      <x:c r="N116" s="455"/>
-      <x:c r="O116" s="455"/>
+      <x:c r="I116" s="455" t="str">
+        <x:v>300..3020;250..1520;300..2400</x:v>
+      </x:c>
+      <x:c r="J116" s="464" t="str">
+        <x:v>mm/mm/mm</x:v>
+      </x:c>
+      <x:c r="K116" s="464" t="str">
+        <x:v>Erfbaar basiscontract voor breedte, diepte en hoogte van de kastfamilie; afgeleide producten mogen uitsluitend met een expliciete strengere override afwijken.</x:v>
+      </x:c>
+      <x:c r="L116" s="464" t="str">
+        <x:v>320</x:v>
+      </x:c>
+      <x:c r="M116" s="464" t="str">
+        <x:v>Goedgekeurd</x:v>
+      </x:c>
+      <x:c r="N116" s="455" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="O116" s="455" t="str">
+        <x:v>PortalConfigurationFactory.BuildCabinet bestaande grenzen; ProductContracts.RegressionTests</x:v>
+      </x:c>
       <x:c r="P116" s="455"/>
       <x:c r="Q116" s="455"/>
       <x:c r="R116" s="455"/>
@@ -35539,21 +36608,49 @@
       <x:c r="V116" s="456"/>
     </x:row>
     <x:row r="117">
-      <x:c r="A117" s="454"/>
-      <x:c r="B117" s="455"/>
-      <x:c r="C117" s="455"/>
-      <x:c r="D117" s="461"/>
-      <x:c r="E117" s="455"/>
-      <x:c r="F117" s="455"/>
+      <x:c r="A117" s="454" t="str">
+        <x:v>PRD-CAB-004</x:v>
+      </x:c>
+      <x:c r="B117" s="455" t="str">
+        <x:v>cabinet</x:v>
+      </x:c>
+      <x:c r="C117" s="455" t="str">
+        <x:v>Materiaal</x:v>
+      </x:c>
+      <x:c r="D117" s="461" t="str">
+        <x:v>korpus, fronten en werkblad</x:v>
+      </x:c>
+      <x:c r="E117" s="455" t="str">
+        <x:v>Materiaalkeuze</x:v>
+      </x:c>
+      <x:c r="F117" s="455" t="str">
+        <x:v>Materiaal</x:v>
+      </x:c>
       <x:c r="G117" s="455"/>
-      <x:c r="H117" s="455"/>
-      <x:c r="I117" s="455"/>
-      <x:c r="J117" s="464"/>
-      <x:c r="K117" s="464"/>
-      <x:c r="L117" s="464"/>
-      <x:c r="M117" s="464"/>
-      <x:c r="N117" s="455"/>
-      <x:c r="O117" s="455"/>
+      <x:c r="H117" s="455" t="str">
+        <x:v>betonplex_18</x:v>
+      </x:c>
+      <x:c r="I117" s="455" t="str">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="J117" s="464" t="str">
+        <x:v>mm default</x:v>
+      </x:c>
+      <x:c r="K117" s="464" t="str">
+        <x:v>Bestaande applicatiestandaard uit de kastfamilie; erft naar vakjeskast en werkbankkast via Basisproduct-ID.</x:v>
+      </x:c>
+      <x:c r="L117" s="464" t="str">
+        <x:v>310</x:v>
+      </x:c>
+      <x:c r="M117" s="464" t="str">
+        <x:v>Goedgekeurd</x:v>
+      </x:c>
+      <x:c r="N117" s="455" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="O117" s="455" t="str">
+        <x:v>ProductDefaults.DefaultSheetIndex; LibraryCatalog; bestaande kastprojecten en regressietests</x:v>
+      </x:c>
       <x:c r="P117" s="455"/>
       <x:c r="Q117" s="455"/>
       <x:c r="R117" s="455"/>
@@ -35563,21 +36660,47 @@
       <x:c r="V117" s="456"/>
     </x:row>
     <x:row r="118">
-      <x:c r="A118" s="454"/>
-      <x:c r="B118" s="455"/>
-      <x:c r="C118" s="455"/>
-      <x:c r="D118" s="461"/>
-      <x:c r="E118" s="455"/>
-      <x:c r="F118" s="455"/>
+      <x:c r="A118" s="454" t="str">
+        <x:v>PRD-WBK-014</x:v>
+      </x:c>
+      <x:c r="B118" s="455" t="str">
+        <x:v>werkbankkast</x:v>
+      </x:c>
+      <x:c r="C118" s="455" t="str">
+        <x:v>Parameters</x:v>
+      </x:c>
+      <x:c r="D118" s="461" t="str">
+        <x:v>klantconfigurator</x:v>
+      </x:c>
+      <x:c r="E118" s="455" t="str">
+        <x:v>Parametercontract</x:v>
+      </x:c>
+      <x:c r="F118" s="455" t="str">
+        <x:v>Geen</x:v>
+      </x:c>
       <x:c r="G118" s="455"/>
       <x:c r="H118" s="455"/>
-      <x:c r="I118" s="455"/>
-      <x:c r="J118" s="464"/>
-      <x:c r="K118" s="464"/>
-      <x:c r="L118" s="464"/>
-      <x:c r="M118" s="464"/>
-      <x:c r="N118" s="455"/>
-      <x:c r="O118" s="455"/>
+      <x:c r="I118" s="455" t="str">
+        <x:v>600..3020;300..1520;500..2400</x:v>
+      </x:c>
+      <x:c r="J118" s="464" t="str">
+        <x:v>mm/mm/mm</x:v>
+      </x:c>
+      <x:c r="K118" s="464" t="str">
+        <x:v>Werkbankkast erft het kastcontract maar gebruikt de bestaande strengere minimummaat voor breedte, diepte en werkhoogte.</x:v>
+      </x:c>
+      <x:c r="L118" s="464" t="str">
+        <x:v>330</x:v>
+      </x:c>
+      <x:c r="M118" s="464" t="str">
+        <x:v>Goedgekeurd</x:v>
+      </x:c>
+      <x:c r="N118" s="455" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="O118" s="455" t="str">
+        <x:v>PortalConfigurationFactory.BuildWorkbenchCabinet bestaande grenzen; ProductContracts.RegressionTests</x:v>
+      </x:c>
       <x:c r="P118" s="455"/>
       <x:c r="Q118" s="455"/>
       <x:c r="R118" s="455"/>
@@ -35587,21 +36710,47 @@
       <x:c r="V118" s="456"/>
     </x:row>
     <x:row r="119">
-      <x:c r="A119" s="454"/>
-      <x:c r="B119" s="455"/>
-      <x:c r="C119" s="455"/>
-      <x:c r="D119" s="461"/>
-      <x:c r="E119" s="455"/>
-      <x:c r="F119" s="455"/>
+      <x:c r="A119" s="454" t="str">
+        <x:v>PRD-FWT-001</x:v>
+      </x:c>
+      <x:c r="B119" s="455" t="str">
+        <x:v>opvouwbare_werktafel</x:v>
+      </x:c>
+      <x:c r="C119" s="455" t="str">
+        <x:v>Parameters</x:v>
+      </x:c>
+      <x:c r="D119" s="461" t="str">
+        <x:v>klantconfigurator</x:v>
+      </x:c>
+      <x:c r="E119" s="455" t="str">
+        <x:v>Parametercontract</x:v>
+      </x:c>
+      <x:c r="F119" s="455" t="str">
+        <x:v>Geen</x:v>
+      </x:c>
       <x:c r="G119" s="455"/>
-      <x:c r="H119" s="455"/>
-      <x:c r="I119" s="455"/>
-      <x:c r="J119" s="464"/>
-      <x:c r="K119" s="464"/>
-      <x:c r="L119" s="464"/>
-      <x:c r="M119" s="464"/>
-      <x:c r="N119" s="455"/>
-      <x:c r="O119" s="455"/>
+      <x:c r="H119" s="455" t="str"/>
+      <x:c r="I119" s="455" t="str">
+        <x:v>800..2400;800..1180;700..1100</x:v>
+      </x:c>
+      <x:c r="J119" s="464" t="str">
+        <x:v>mm/mm/mm</x:v>
+      </x:c>
+      <x:c r="K119" s="464" t="str">
+        <x:v>Voorlopige conceptgrenzen voor bladlengte, bladbreedte en hoogte bovenzijde blad. De minimale bladbreedte van 800 mm laat bij 140-mm stijlen een maakbare opening in ieder half kort vouwpaneel; iedere plaatpassing wordt daarnaast tegen de gekoppelde handelsplaat gecontroleerd.</x:v>
+      </x:c>
+      <x:c r="L119" s="464" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="M119" s="464" t="str">
+        <x:v>Voorlopig</x:v>
+      </x:c>
+      <x:c r="N119" s="455" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="O119" s="455" t="str">
+        <x:v>Gebruikersbesluit 2026-09-01; conceptvisualisatie; geometrische maakbaarheidscontrole</x:v>
+      </x:c>
       <x:c r="P119" s="455"/>
       <x:c r="Q119" s="455"/>
       <x:c r="R119" s="455"/>
@@ -35611,21 +36760,49 @@
       <x:c r="V119" s="456"/>
     </x:row>
     <x:row r="120">
-      <x:c r="A120" s="454"/>
-      <x:c r="B120" s="455"/>
-      <x:c r="C120" s="455"/>
-      <x:c r="D120" s="461"/>
-      <x:c r="E120" s="455"/>
-      <x:c r="F120" s="455"/>
+      <x:c r="A120" s="454" t="str">
+        <x:v>PRD-FWT-002</x:v>
+      </x:c>
+      <x:c r="B120" s="455" t="str">
+        <x:v>opvouwbare_werktafel</x:v>
+      </x:c>
+      <x:c r="C120" s="455" t="str">
+        <x:v>Materiaal</x:v>
+      </x:c>
+      <x:c r="D120" s="461" t="str">
+        <x:v>alle plaatdelen</x:v>
+      </x:c>
+      <x:c r="E120" s="455" t="str">
+        <x:v>Materiaalkeuze</x:v>
+      </x:c>
+      <x:c r="F120" s="455" t="str">
+        <x:v>Materiaal</x:v>
+      </x:c>
       <x:c r="G120" s="455"/>
-      <x:c r="H120" s="455"/>
-      <x:c r="I120" s="455"/>
-      <x:c r="J120" s="464"/>
-      <x:c r="K120" s="464"/>
-      <x:c r="L120" s="464"/>
-      <x:c r="M120" s="464"/>
-      <x:c r="N120" s="455"/>
-      <x:c r="O120" s="455"/>
+      <x:c r="H120" s="455" t="str">
+        <x:v>betonplex_18</x:v>
+      </x:c>
+      <x:c r="I120" s="455" t="str">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="J120" s="464" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="K120" s="464" t="str">
+        <x:v>Werkblad, twee vaste lange framepanelen en vier korte framevormige vouwpanelen worden uit hetzelfde 18-mm betonplexcontract gebouwd.</x:v>
+      </x:c>
+      <x:c r="L120" s="464" t="n">
+        <x:v>310</x:v>
+      </x:c>
+      <x:c r="M120" s="464" t="str">
+        <x:v>Goedgekeurd</x:v>
+      </x:c>
+      <x:c r="N120" s="455" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="O120" s="455" t="str">
+        <x:v>Gebruikersbesluit 2026-08-31; betonplex_18</x:v>
+      </x:c>
       <x:c r="P120" s="455"/>
       <x:c r="Q120" s="455"/>
       <x:c r="R120" s="455"/>
@@ -35635,21 +36812,49 @@
       <x:c r="V120" s="456"/>
     </x:row>
     <x:row r="121">
-      <x:c r="A121" s="454"/>
-      <x:c r="B121" s="455"/>
-      <x:c r="C121" s="455"/>
-      <x:c r="D121" s="461"/>
-      <x:c r="E121" s="455"/>
-      <x:c r="F121" s="455"/>
+      <x:c r="A121" s="454" t="str">
+        <x:v>PRD-FWT-003</x:v>
+      </x:c>
+      <x:c r="B121" s="455" t="str">
+        <x:v>opvouwbare_werktafel</x:v>
+      </x:c>
+      <x:c r="C121" s="455" t="str">
+        <x:v>CNC</x:v>
+      </x:c>
+      <x:c r="D121" s="461" t="str">
+        <x:v>werkblad; plaatpassing en nesting</x:v>
+      </x:c>
+      <x:c r="E121" s="455" t="str">
+        <x:v>Plaatmarge</x:v>
+      </x:c>
+      <x:c r="F121" s="455" t="str">
+        <x:v>Materiaal</x:v>
+      </x:c>
       <x:c r="G121" s="455"/>
-      <x:c r="H121" s="455"/>
-      <x:c r="I121" s="455"/>
-      <x:c r="J121" s="464"/>
-      <x:c r="K121" s="464"/>
-      <x:c r="L121" s="464"/>
-      <x:c r="M121" s="464"/>
-      <x:c r="N121" s="455"/>
-      <x:c r="O121" s="455"/>
+      <x:c r="H121" s="455" t="str">
+        <x:v>betonplex_18</x:v>
+      </x:c>
+      <x:c r="I121" s="455" t="str">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="J121" s="464" t="str">
+        <x:v>mm totale reductie per plaatrichting</x:v>
+      </x:c>
+      <x:c r="K121" s="464" t="str">
+        <x:v>Gebruikersreferentie 2440×1220 wordt 2400×1180: 40 mm totaal per richting, gelijk aan 20 mm randmarge per zijde. Het actuele G Goedkoop-artikel is 2500×1250 en levert daardoor extra marge.</x:v>
+      </x:c>
+      <x:c r="L121" s="464" t="n">
+        <x:v>320</x:v>
+      </x:c>
+      <x:c r="M121" s="464" t="str">
+        <x:v>Voorlopig</x:v>
+      </x:c>
+      <x:c r="N121" s="455" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="O121" s="455" t="str">
+        <x:v>Gebruikersbesluit 2026-08-31; G Goedkoop 0000008204</x:v>
+      </x:c>
       <x:c r="P121" s="455"/>
       <x:c r="Q121" s="455"/>
       <x:c r="R121" s="455"/>
@@ -35659,21 +36864,49 @@
       <x:c r="V121" s="456"/>
     </x:row>
     <x:row r="122">
-      <x:c r="A122" s="454"/>
-      <x:c r="B122" s="455"/>
-      <x:c r="C122" s="455"/>
-      <x:c r="D122" s="461"/>
-      <x:c r="E122" s="455"/>
-      <x:c r="F122" s="455"/>
+      <x:c r="A122" s="454" t="str">
+        <x:v>PRD-FWT-004</x:v>
+      </x:c>
+      <x:c r="B122" s="455" t="str">
+        <x:v>opvouwbare_werktafel</x:v>
+      </x:c>
+      <x:c r="C122" s="455" t="str">
+        <x:v>Geometrie</x:v>
+      </x:c>
+      <x:c r="D122" s="461" t="str">
+        <x:v>Alle afgeleide panelen, uitsparingen, aparte bladoverstekken aan lange en korte zijde en scharnierplaatsingen</x:v>
+      </x:c>
+      <x:c r="E122" s="455" t="str">
+        <x:v>Geometriecontract</x:v>
+      </x:c>
+      <x:c r="F122" s="455" t="str">
+        <x:v>Materiaal</x:v>
+      </x:c>
       <x:c r="G122" s="455"/>
-      <x:c r="H122" s="455"/>
-      <x:c r="I122" s="455"/>
-      <x:c r="J122" s="464"/>
-      <x:c r="K122" s="464"/>
-      <x:c r="L122" s="464"/>
-      <x:c r="M122" s="464"/>
-      <x:c r="N122" s="455"/>
-      <x:c r="O122" s="455"/>
+      <x:c r="H122" s="455" t="str">
+        <x:v>betonplex_18</x:v>
+      </x:c>
+      <x:c r="I122" s="455" t="str">
+        <x:v>jointClearance=1;tabWidth=80;frameStileWidth=140;topRailHeight=180;bottomRailHeight=140;integratedFootWidth=140;integratedFootReliefHeight=30;cornerRadius=8;worktopFloat=150;foldedClearance=8;tabsPerLongPanel=3;tabsPerShortPanelHalf=2;hingeHeight=76;hingeOpenWidth=76;hingeLeafThickness=2.5;hingeBarrelDiameter=10.8;hingeGap=2</x:v>
+      </x:c>
+      <x:c r="J122" s="464" t="str">
+        <x:v>mm; aantal</x:v>
+      </x:c>
+      <x:c r="K122" s="464" t="str">
+        <x:v>Onderstelmaat volgt uit twee invoercontracten: de offset vanaf de korte bladranden bepaalt de onderstellengte en de offset vanaf de lange bladranden bepaalt de ondersteldiepte. De conceptstandaard is voor beide 80 mm. Vaste langspanelen dragen drie nokken; ieder kort half vouwpaneel twee. Alle panelen hebben brede regels/stijlen, geïntegreerde voeten en tussenliggende vloervrijloop. Scharniermaat is alleen render-envelope totdat sample en proefstuk zijn gecontroleerd.</x:v>
+      </x:c>
+      <x:c r="L122" s="464" t="n">
+        <x:v>330</x:v>
+      </x:c>
+      <x:c r="M122" s="464" t="str">
+        <x:v>Proefstuk</x:v>
+      </x:c>
+      <x:c r="N122" s="455" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="O122" s="455" t="str">
+        <x:v>Gebruikersbesluit en geannoteerde fotoreconstructie 2026-09-01; AXA technische tekening 1KL227676</x:v>
+      </x:c>
       <x:c r="P122" s="455"/>
       <x:c r="Q122" s="455"/>
       <x:c r="R122" s="455"/>
@@ -35683,21 +36916,49 @@
       <x:c r="V122" s="456"/>
     </x:row>
     <x:row r="123">
-      <x:c r="A123" s="454"/>
-      <x:c r="B123" s="455"/>
-      <x:c r="C123" s="455"/>
-      <x:c r="D123" s="461"/>
-      <x:c r="E123" s="455"/>
-      <x:c r="F123" s="455"/>
+      <x:c r="A123" s="454" t="str">
+        <x:v>PRD-FWT-005</x:v>
+      </x:c>
+      <x:c r="B123" s="455" t="str">
+        <x:v>opvouwbare_werktafel</x:v>
+      </x:c>
+      <x:c r="C123" s="455" t="str">
+        <x:v>Verbinding</x:v>
+      </x:c>
+      <x:c r="D123" s="461" t="str">
+        <x:v>zes langspaneelnokken en acht nokken op korte halve vouwpanelen met werkbladslots</x:v>
+      </x:c>
+      <x:c r="E123" s="455" t="str">
+        <x:v>Gat-nokpassing</x:v>
+      </x:c>
+      <x:c r="F123" s="455" t="str">
+        <x:v>Materiaal</x:v>
+      </x:c>
       <x:c r="G123" s="455"/>
-      <x:c r="H123" s="455"/>
-      <x:c r="I123" s="455"/>
-      <x:c r="J123" s="464"/>
-      <x:c r="K123" s="464"/>
-      <x:c r="L123" s="464"/>
-      <x:c r="M123" s="464"/>
-      <x:c r="N123" s="455"/>
-      <x:c r="O123" s="455"/>
+      <x:c r="H123" s="455" t="str">
+        <x:v>betonplex_18</x:v>
+      </x:c>
+      <x:c r="I123" s="455" t="str">
+        <x:v>clearancePerSide=1;engagementDepth=18;flushToTopSurface=true;gravityRetained=true;removableWithoutTools=true;tabCount=14</x:v>
+      </x:c>
+      <x:c r="J123" s="464" t="str">
+        <x:v>mm; bool</x:v>
+      </x:c>
+      <x:c r="K123" s="464" t="str">
+        <x:v>Drie nokken op ieder vast langspaneel en twee nokken op ieder van de vier korte halve vouwpanelen steken door de volle bladdikte tot vlak met de bovenzijde. Het blad blijft gereedschapsloos uitneembaar en borgt het geopende onderstel door geometrie en zwaartekracht.</x:v>
+      </x:c>
+      <x:c r="L123" s="464" t="n">
+        <x:v>340</x:v>
+      </x:c>
+      <x:c r="M123" s="464" t="str">
+        <x:v>Proefstuk</x:v>
+      </x:c>
+      <x:c r="N123" s="455" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="O123" s="455" t="str">
+        <x:v>Gebruikersbesluit en geannoteerde fotoreconstructie 2026-09-01</x:v>
+      </x:c>
       <x:c r="P123" s="455"/>
       <x:c r="Q123" s="455"/>
       <x:c r="R123" s="455"/>
@@ -35707,21 +36968,49 @@
       <x:c r="V123" s="456"/>
     </x:row>
     <x:row r="124">
-      <x:c r="A124" s="454"/>
-      <x:c r="B124" s="455"/>
-      <x:c r="C124" s="455"/>
-      <x:c r="D124" s="461"/>
-      <x:c r="E124" s="455"/>
-      <x:c r="F124" s="455"/>
+      <x:c r="A124" s="454" t="str">
+        <x:v>PRD-FWT-006</x:v>
+      </x:c>
+      <x:c r="B124" s="455" t="str">
+        <x:v>opvouwbare_werktafel</x:v>
+      </x:c>
+      <x:c r="C124" s="455" t="str">
+        <x:v>Beslag</x:v>
+      </x:c>
+      <x:c r="D124" s="461" t="str">
+        <x:v>twee korte zijden met elk twee scharnierende framepanelen</x:v>
+      </x:c>
+      <x:c r="E124" s="455" t="str">
+        <x:v>Vouwscharnier</x:v>
+      </x:c>
+      <x:c r="F124" s="455" t="str">
+        <x:v>Component</x:v>
+      </x:c>
       <x:c r="G124" s="455"/>
-      <x:c r="H124" s="455"/>
-      <x:c r="I124" s="455"/>
-      <x:c r="J124" s="464"/>
-      <x:c r="K124" s="464"/>
-      <x:c r="L124" s="464"/>
-      <x:c r="M124" s="464"/>
-      <x:c r="N124" s="455"/>
-      <x:c r="O124" s="455"/>
+      <x:c r="H124" s="455" t="str">
+        <x:v>ggoedkoop_axa_ball_bearing_hinge_rvs_76x76x25</x:v>
+      </x:c>
+      <x:c r="I124" s="455" t="str">
+        <x:v>6 AXA 1KL227676N bladscharnieren; 1 per verticale scharnieras; 3 gaten per blad</x:v>
+      </x:c>
+      <x:c r="J124" s="464" t="str">
+        <x:v>st</x:v>
+      </x:c>
+      <x:c r="K124" s="464" t="str">
+        <x:v>Elke korte vouwzijde heeft een voorste, middelste en achterste verticale scharnieras. De buitenste scharnieren zitten aan de binnenzijde van de panelen. Ieder scharnier bestaat fysiek uit blad A met eigen knoopsegmenten, blad B met eigen knoopsegment en één pen. De twee bladen zijn expliciet gekoppeld aan de bedoelde twee plaatdelen. De fabrikanttekening bevestigt drie verzonken gaten per blad en knoop Ø10,8 mm; exacte hartcoördinaten, gat-/verzinkmaat en bevestiger voor 18-mm plaat blijven proefstukdata.</x:v>
+      </x:c>
+      <x:c r="L124" s="464" t="n">
+        <x:v>350</x:v>
+      </x:c>
+      <x:c r="M124" s="464" t="str">
+        <x:v>Voorlopig</x:v>
+      </x:c>
+      <x:c r="N124" s="455" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="O124" s="455" t="str">
+        <x:v>https://axahomesecurity.com/producten/scharnier-kogellager-2/; https://axahomesecurity.com/wp-content/uploads/sites/2/2024/08/tekening-1kl227676-kogellagerscharnier_E0008442.jpg; G Goedkoop 0000006696</x:v>
+      </x:c>
       <x:c r="P124" s="455"/>
       <x:c r="Q124" s="455"/>
       <x:c r="R124" s="455"/>
@@ -35731,21 +37020,49 @@
       <x:c r="V124" s="456"/>
     </x:row>
     <x:row r="125">
-      <x:c r="A125" s="454"/>
-      <x:c r="B125" s="455"/>
-      <x:c r="C125" s="455"/>
-      <x:c r="D125" s="461"/>
-      <x:c r="E125" s="455"/>
-      <x:c r="F125" s="455"/>
+      <x:c r="A125" s="454" t="str">
+        <x:v>PRD-FWT-007</x:v>
+      </x:c>
+      <x:c r="B125" s="455" t="str">
+        <x:v>opvouwbare_werktafel</x:v>
+      </x:c>
+      <x:c r="C125" s="455" t="str">
+        <x:v>CNC</x:v>
+      </x:c>
+      <x:c r="D125" s="461" t="str">
+        <x:v>alle rechthoekige noksleuven</x:v>
+      </x:c>
+      <x:c r="E125" s="455" t="str">
+        <x:v>Dogbonegereedschap</x:v>
+      </x:c>
+      <x:c r="F125" s="455" t="str">
+        <x:v>Gereedschap</x:v>
+      </x:c>
       <x:c r="G125" s="455"/>
-      <x:c r="H125" s="455"/>
-      <x:c r="I125" s="455"/>
-      <x:c r="J125" s="464"/>
-      <x:c r="K125" s="464"/>
-      <x:c r="L125" s="464"/>
-      <x:c r="M125" s="464"/>
-      <x:c r="N125" s="455"/>
-      <x:c r="O125" s="455"/>
+      <x:c r="H125" s="455" t="str">
+        <x:v>endmill_6mm</x:v>
+      </x:c>
+      <x:c r="I125" s="455" t="str">
+        <x:v>hoekontlasting uit actuele gereedschapdiameter</x:v>
+      </x:c>
+      <x:c r="J125" s="464" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="K125" s="464" t="str">
+        <x:v>Geen vaste dogboneradius in de UI; de backend gebruikt de diameter van het gekoppelde freesrecord. Fysieke passing blijft proefstuk.</x:v>
+      </x:c>
+      <x:c r="L125" s="464" t="n">
+        <x:v>360</x:v>
+      </x:c>
+      <x:c r="M125" s="464" t="str">
+        <x:v>Voorlopig</x:v>
+      </x:c>
+      <x:c r="N125" s="455" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="O125" s="455" t="str">
+        <x:v>Gereedschappen.endmill_6mm; gebruikersbesluit 2026-08-31</x:v>
+      </x:c>
       <x:c r="P125" s="455"/>
       <x:c r="Q125" s="455"/>
       <x:c r="R125" s="455"/>
@@ -35755,21 +37072,49 @@
       <x:c r="V125" s="456"/>
     </x:row>
     <x:row r="126">
-      <x:c r="A126" s="454"/>
-      <x:c r="B126" s="455"/>
-      <x:c r="C126" s="455"/>
-      <x:c r="D126" s="461"/>
-      <x:c r="E126" s="455"/>
-      <x:c r="F126" s="455"/>
+      <x:c r="A126" s="454" t="str">
+        <x:v>PRD-FWT-008</x:v>
+      </x:c>
+      <x:c r="B126" s="455" t="str">
+        <x:v>opvouwbare_werktafel</x:v>
+      </x:c>
+      <x:c r="C126" s="455" t="str">
+        <x:v>CNC</x:v>
+      </x:c>
+      <x:c r="D126" s="461" t="str">
+        <x:v>buitencontouren van alle plaatdelen</x:v>
+      </x:c>
+      <x:c r="E126" s="455" t="str">
+        <x:v>Randafschuining</x:v>
+      </x:c>
+      <x:c r="F126" s="455" t="str">
+        <x:v>Gereedschap</x:v>
+      </x:c>
       <x:c r="G126" s="455"/>
-      <x:c r="H126" s="455"/>
-      <x:c r="I126" s="455"/>
-      <x:c r="J126" s="464"/>
-      <x:c r="K126" s="464"/>
-      <x:c r="L126" s="464"/>
-      <x:c r="M126" s="464"/>
-      <x:c r="N126" s="455"/>
-      <x:c r="O126" s="455"/>
+      <x:c r="H126" s="455" t="str">
+        <x:v>vbit_90deg_8mm_shank_6_35</x:v>
+      </x:c>
+      <x:c r="I126" s="455" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J126" s="464" t="str">
+        <x:v>mm breed × mm diep</x:v>
+      </x:c>
+      <x:c r="K126" s="464" t="str">
+        <x:v>Hergebruikt de bestaande generieke buitencontourafschuining; interne slots, gaten en pockets blijven uitgesloten.</x:v>
+      </x:c>
+      <x:c r="L126" s="464" t="n">
+        <x:v>370</x:v>
+      </x:c>
+      <x:c r="M126" s="464" t="str">
+        <x:v>Voorlopig</x:v>
+      </x:c>
+      <x:c r="N126" s="455" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="O126" s="455" t="str">
+        <x:v>CAM-V-002; CsvExporter; Mach3GCodeGenerator</x:v>
+      </x:c>
       <x:c r="P126" s="455"/>
       <x:c r="Q126" s="455"/>
       <x:c r="R126" s="455"/>
@@ -35779,21 +37124,49 @@
       <x:c r="V126" s="456"/>
     </x:row>
     <x:row r="127">
-      <x:c r="A127" s="454"/>
-      <x:c r="B127" s="455"/>
-      <x:c r="C127" s="455"/>
-      <x:c r="D127" s="461"/>
-      <x:c r="E127" s="455"/>
-      <x:c r="F127" s="455"/>
+      <x:c r="A127" s="454" t="str">
+        <x:v>PRD-FWT-009</x:v>
+      </x:c>
+      <x:c r="B127" s="455" t="str">
+        <x:v>opvouwbare_werktafel</x:v>
+      </x:c>
+      <x:c r="C127" s="455" t="str">
+        <x:v>Beweging</x:v>
+      </x:c>
+      <x:c r="D127" s="461" t="str">
+        <x:v>interactieve conceptvisualisatie</x:v>
+      </x:c>
+      <x:c r="E127" s="455" t="str">
+        <x:v>Bewegingscontract</x:v>
+      </x:c>
+      <x:c r="F127" s="455" t="str">
+        <x:v>Component</x:v>
+      </x:c>
       <x:c r="G127" s="455"/>
-      <x:c r="H127" s="455"/>
-      <x:c r="I127" s="455"/>
-      <x:c r="J127" s="464"/>
-      <x:c r="K127" s="464"/>
-      <x:c r="L127" s="464"/>
-      <x:c r="M127" s="464"/>
-      <x:c r="N127" s="455"/>
-      <x:c r="O127" s="455"/>
+      <x:c r="H127" s="455" t="str">
+        <x:v>ggoedkoop_axa_ball_bearing_hinge_rvs_76x76x25</x:v>
+      </x:c>
+      <x:c r="I127" s="455" t="str">
+        <x:v>onderstel=0..1;blad=0..150;vouwrichting=korte-zijde</x:v>
+      </x:c>
+      <x:c r="J127" s="464" t="str">
+        <x:v>fractie; mm</x:v>
+      </x:c>
+      <x:c r="K127" s="464" t="str">
+        <x:v>Slider 1 vouwt de vier korte framepanelen vlak rond zes normale verticale bladscharnierassen en trekt het achterste vaste langspaneel naar een pakket van vier plaatdiktes plus scharnierspeling. Slider 2 laat het losse blad vanuit 150 mm zweefhoogte verticaal in veertien nokslots zakken.</x:v>
+      </x:c>
+      <x:c r="L127" s="464" t="n">
+        <x:v>380</x:v>
+      </x:c>
+      <x:c r="M127" s="464" t="str">
+        <x:v>Voorlopig</x:v>
+      </x:c>
+      <x:c r="N127" s="455" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="O127" s="455" t="str">
+        <x:v>Gebruikersbesluit 2026-09-01; backend keyframecontract</x:v>
+      </x:c>
       <x:c r="P127" s="455"/>
       <x:c r="Q127" s="455"/>
       <x:c r="R127" s="455"/>
@@ -35803,21 +37176,45 @@
       <x:c r="V127" s="456"/>
     </x:row>
     <x:row r="128">
-      <x:c r="A128" s="454"/>
-      <x:c r="B128" s="455"/>
-      <x:c r="C128" s="455"/>
-      <x:c r="D128" s="461"/>
-      <x:c r="E128" s="455"/>
-      <x:c r="F128" s="455"/>
+      <x:c r="A128" s="454" t="str">
+        <x:v>PRD-FWT-010</x:v>
+      </x:c>
+      <x:c r="B128" s="455" t="str">
+        <x:v>opvouwbare_werktafel</x:v>
+      </x:c>
+      <x:c r="C128" s="455" t="str">
+        <x:v>Constructie</x:v>
+      </x:c>
+      <x:c r="D128" s="461" t="str">
+        <x:v>uitgeklapte gebruiksstand</x:v>
+      </x:c>
+      <x:c r="E128" s="455" t="str">
+        <x:v>Bladborging</x:v>
+      </x:c>
+      <x:c r="F128" s="455" t="str">
+        <x:v>Geen</x:v>
+      </x:c>
       <x:c r="G128" s="455"/>
-      <x:c r="H128" s="455"/>
-      <x:c r="I128" s="455"/>
-      <x:c r="J128" s="464"/>
-      <x:c r="K128" s="464"/>
-      <x:c r="L128" s="464"/>
-      <x:c r="M128" s="464"/>
-      <x:c r="N128" s="455"/>
-      <x:c r="O128" s="455"/>
+      <x:c r="H128" s="455" t="str"/>
+      <x:c r="I128" s="455" t="str">
+        <x:v>veertien doorsteeknokken; geen clips, pennen of knevels</x:v>
+      </x:c>
+      <x:c r="J128" s="464" t="str"/>
+      <x:c r="K128" s="464" t="str">
+        <x:v>Zes nokken op de twee vaste langspanelen en acht nokken op de vier korte halve vouwpanelen nemen de open stand geometrisch op. De brede regels en geïntegreerde voeten onder iedere stijl volgen de referentiefoto; werkbelasting en de definitieve 30-mm vloervrijloop worden pas na constructievisualisatie en proefopstelling vastgesteld.</x:v>
+      </x:c>
+      <x:c r="L128" s="464" t="n">
+        <x:v>390</x:v>
+      </x:c>
+      <x:c r="M128" s="464" t="str">
+        <x:v>Proefstuk</x:v>
+      </x:c>
+      <x:c r="N128" s="455" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="O128" s="455" t="str">
+        <x:v>Gebruikersbesluit en geannoteerde fotoreconstructie 2026-09-01</x:v>
+      </x:c>
       <x:c r="P128" s="455"/>
       <x:c r="Q128" s="455"/>
       <x:c r="R128" s="455"/>
@@ -35827,21 +37224,45 @@
       <x:c r="V128" s="456"/>
     </x:row>
     <x:row r="129">
-      <x:c r="A129" s="454"/>
-      <x:c r="B129" s="455"/>
-      <x:c r="C129" s="455"/>
-      <x:c r="D129" s="461"/>
-      <x:c r="E129" s="455"/>
-      <x:c r="F129" s="455"/>
+      <x:c r="A129" s="454" t="str">
+        <x:v>PRD-FWT-011</x:v>
+      </x:c>
+      <x:c r="B129" s="455" t="str">
+        <x:v>opvouwbare_werktafel</x:v>
+      </x:c>
+      <x:c r="C129" s="455" t="str">
+        <x:v>Vrijgave</x:v>
+      </x:c>
+      <x:c r="D129" s="461" t="str">
+        <x:v>productie</x:v>
+      </x:c>
+      <x:c r="E129" s="455" t="str">
+        <x:v>Vrijgaveblokkade</x:v>
+      </x:c>
+      <x:c r="F129" s="455" t="str">
+        <x:v>Geen</x:v>
+      </x:c>
       <x:c r="G129" s="455"/>
-      <x:c r="H129" s="455"/>
-      <x:c r="I129" s="455"/>
-      <x:c r="J129" s="464"/>
-      <x:c r="K129" s="464"/>
-      <x:c r="L129" s="464"/>
-      <x:c r="M129" s="464"/>
-      <x:c r="N129" s="455"/>
-      <x:c r="O129" s="455"/>
+      <x:c r="H129" s="455" t="str"/>
+      <x:c r="I129" s="455" t="str">
+        <x:v>scharnier-gatenpatroon-en-bevestigers;gat-nok-proefpassing;L-eindslot-contour-en-dogbones;belasting-en-stijfheidscontrole;stabiliteit-en-onbedoeld-uitlichten;randafwerking-proefstuk</x:v>
+      </x:c>
+      <x:c r="J129" s="464" t="str"/>
+      <x:c r="K129" s="464" t="str">
+        <x:v>Conceptvisualisatie en offerte zijn toegestaan; CAM, native productie-SolidWorks en productievrijgave blijven geblokkeerd totdat sample, proefpassing en belastingtest zijn vastgelegd.</x:v>
+      </x:c>
+      <x:c r="L129" s="464" t="n">
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="M129" s="464" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="N129" s="455" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="O129" s="455" t="str">
+        <x:v>Gebruikersbesluit 2026-08-31; ProductReleaseContract</x:v>
+      </x:c>
       <x:c r="P129" s="455"/>
       <x:c r="Q129" s="455"/>
       <x:c r="R129" s="455"/>
@@ -35851,21 +37272,45 @@
       <x:c r="V129" s="456"/>
     </x:row>
     <x:row r="130">
-      <x:c r="A130" s="454"/>
-      <x:c r="B130" s="455"/>
-      <x:c r="C130" s="455"/>
-      <x:c r="D130" s="461"/>
-      <x:c r="E130" s="455"/>
-      <x:c r="F130" s="455"/>
+      <x:c r="A130" s="454" t="str">
+        <x:v>PRD-FWT-012</x:v>
+      </x:c>
+      <x:c r="B130" s="455" t="str">
+        <x:v>opvouwbare_werktafel</x:v>
+      </x:c>
+      <x:c r="C130" s="455" t="str">
+        <x:v>Vrijgave</x:v>
+      </x:c>
+      <x:c r="D130" s="461" t="str">
+        <x:v>conceptpakket</x:v>
+      </x:c>
+      <x:c r="E130" s="455" t="str">
+        <x:v>Conceptexport</x:v>
+      </x:c>
+      <x:c r="F130" s="455" t="str">
+        <x:v>Geen</x:v>
+      </x:c>
       <x:c r="G130" s="455"/>
-      <x:c r="H130" s="455"/>
-      <x:c r="I130" s="455"/>
-      <x:c r="J130" s="464"/>
-      <x:c r="K130" s="464"/>
-      <x:c r="L130" s="464"/>
-      <x:c r="M130" s="464"/>
-      <x:c r="N130" s="455"/>
-      <x:c r="O130" s="455"/>
+      <x:c r="H130" s="455" t="str"/>
+      <x:c r="I130" s="455" t="str">
+        <x:v>Klantvoorstel;Interactief 3D;Projectdata</x:v>
+      </x:c>
+      <x:c r="J130" s="464" t="str"/>
+      <x:c r="K130" s="464" t="str">
+        <x:v>Geen productie-CAM of native productiebestanden zolang PRD-FWT-011 open is.</x:v>
+      </x:c>
+      <x:c r="L130" s="464" t="n">
+        <x:v>910</x:v>
+      </x:c>
+      <x:c r="M130" s="464" t="str">
+        <x:v>Voorlopig</x:v>
+      </x:c>
+      <x:c r="N130" s="455" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="O130" s="455" t="str">
+        <x:v>ProductReleaseContract</x:v>
+      </x:c>
       <x:c r="P130" s="455"/>
       <x:c r="Q130" s="455"/>
       <x:c r="R130" s="455"/>
@@ -36064,9 +37509,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb396d107f740434b"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf22fa2ed0f224ee1"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9acf3cfd2c1b48fa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8e2f184d6d84f4c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>